<commit_message>
Prospection : BGE national, boîte non relevée (réponse automatique), pas de relance
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="356">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -446,6 +446,12 @@
   </si>
   <si>
     <t xml:space="preserve">Des outils gratuits pour les entrepreneurs que vous accompagnez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adresse invalide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réponse auto 19/10 : boîte plus relevée. Pas de relance. Viser les BGE régionales.</t>
   </si>
   <si>
     <t xml:space="preserve">CCI Réunion (conseil entreprise)</t>
@@ -1331,7 +1337,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1351,6 +1357,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2781,7 +2795,7 @@
         <v>128</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>22</v>
+        <v>129</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>46314</v>
@@ -2794,7 +2808,7 @@
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
       <c r="O28" s="4" t="s">
-        <v>23</v>
+        <v>130</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2805,16 +2819,16 @@
         <v>57</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>62</v>
@@ -2847,16 +2861,16 @@
         <v>57</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>102</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>62</v>
@@ -2889,16 +2903,16 @@
         <v>57</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>102</v>
       </c>
       <c r="E31" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F31" s="3" t="s">
         <v>137</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>135</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>62</v>
@@ -2931,16 +2945,16 @@
         <v>57</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>102</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G32" s="3" t="s">
         <v>62</v>
@@ -2960,7 +2974,7 @@
       <c r="M32" s="4"/>
       <c r="N32" s="4"/>
       <c r="O32" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2971,16 +2985,16 @@
         <v>57</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>102</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G33" s="3" t="s">
         <v>62</v>
@@ -3000,7 +3014,7 @@
       <c r="M33" s="4"/>
       <c r="N33" s="4"/>
       <c r="O33" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3011,16 +3025,16 @@
         <v>57</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>62</v>
@@ -3040,7 +3054,7 @@
       <c r="M34" s="4"/>
       <c r="N34" s="4"/>
       <c r="O34" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3051,16 +3065,16 @@
         <v>57</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>62</v>
@@ -3080,7 +3094,7 @@
       <c r="M35" s="4"/>
       <c r="N35" s="4"/>
       <c r="O35" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3091,16 +3105,16 @@
         <v>57</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>121</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>62</v>
@@ -3120,7 +3134,7 @@
       <c r="M36" s="4"/>
       <c r="N36" s="4"/>
       <c r="O36" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3131,16 +3145,16 @@
         <v>57</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>62</v>
@@ -3160,7 +3174,7 @@
       <c r="M37" s="4"/>
       <c r="N37" s="4"/>
       <c r="O37" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3171,16 +3185,16 @@
         <v>57</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>93</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>62</v>
@@ -3200,7 +3214,7 @@
       <c r="M38" s="4"/>
       <c r="N38" s="4"/>
       <c r="O38" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3211,16 +3225,16 @@
         <v>57</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>121</v>
       </c>
       <c r="E39" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F39" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>158</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>62</v>
@@ -3240,7 +3254,7 @@
       <c r="M39" s="4"/>
       <c r="N39" s="4"/>
       <c r="O39" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3251,16 +3265,16 @@
         <v>87</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>90</v>
@@ -3280,7 +3294,7 @@
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
       <c r="O40" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3291,13 +3305,13 @@
         <v>87</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>77</v>
@@ -3331,16 +3345,16 @@
         <v>87</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>90</v>
@@ -3360,7 +3374,7 @@
       <c r="M42" s="4"/>
       <c r="N42" s="4"/>
       <c r="O42" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3371,16 +3385,16 @@
         <v>87</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>93</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>90</v>
@@ -3400,7 +3414,7 @@
       <c r="M43" s="4"/>
       <c r="N43" s="4"/>
       <c r="O43" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3411,16 +3425,16 @@
         <v>87</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>90</v>
@@ -3440,7 +3454,7 @@
       <c r="M44" s="4"/>
       <c r="N44" s="4"/>
       <c r="O44" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3451,16 +3465,16 @@
         <v>87</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>121</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>90</v>
@@ -3480,7 +3494,7 @@
       <c r="M45" s="4"/>
       <c r="N45" s="4"/>
       <c r="O45" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3491,16 +3505,16 @@
         <v>87</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>90</v>
@@ -3520,7 +3534,7 @@
       <c r="M46" s="4"/>
       <c r="N46" s="4"/>
       <c r="O46" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3531,16 +3545,16 @@
         <v>87</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>90</v>
@@ -3560,7 +3574,7 @@
       <c r="M47" s="4"/>
       <c r="N47" s="4"/>
       <c r="O47" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3571,16 +3585,16 @@
         <v>87</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>81</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>90</v>
@@ -3600,7 +3614,7 @@
       <c r="M48" s="4"/>
       <c r="N48" s="4"/>
       <c r="O48" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3608,25 +3622,25 @@
         <v>48</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>64</v>
@@ -3648,25 +3662,25 @@
         <v>49</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>75</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I50" s="4" t="s">
         <v>64</v>
@@ -3680,7 +3694,7 @@
       <c r="M50" s="4"/>
       <c r="N50" s="4"/>
       <c r="O50" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3688,25 +3702,25 @@
         <v>50</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>93</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>64</v>
@@ -3728,25 +3742,25 @@
         <v>51</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>75</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>64</v>
@@ -3768,25 +3782,25 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>93</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>64</v>
@@ -3808,25 +3822,25 @@
         <v>53</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>121</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G54" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I54" s="4" t="s">
         <v>64</v>
@@ -3848,25 +3862,25 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>75</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I55" s="4" t="s">
         <v>64</v>
@@ -3888,25 +3902,25 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>121</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I56" s="4" t="s">
         <v>64</v>
@@ -3920,7 +3934,7 @@
       <c r="M56" s="4"/>
       <c r="N56" s="4"/>
       <c r="O56" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3928,25 +3942,25 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>121</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I57" s="4" t="s">
         <v>64</v>
@@ -3960,7 +3974,7 @@
       <c r="M57" s="4"/>
       <c r="N57" s="4"/>
       <c r="O57" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3968,25 +3982,25 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>93</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I58" s="4" t="s">
         <v>64</v>
@@ -4000,7 +4014,7 @@
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
       <c r="O58" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4008,25 +4022,25 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I59" s="4" t="s">
         <v>64</v>
@@ -4040,7 +4054,7 @@
       <c r="M59" s="4"/>
       <c r="N59" s="4"/>
       <c r="O59" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4048,25 +4062,25 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I60" s="4" t="s">
         <v>64</v>
@@ -4080,7 +4094,7 @@
       <c r="M60" s="4"/>
       <c r="N60" s="4"/>
       <c r="O60" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4088,25 +4102,25 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E61" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="F61" s="3" t="s">
         <v>222</v>
-      </c>
-      <c r="F61" s="3" t="s">
-        <v>220</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I61" s="4" t="s">
         <v>64</v>
@@ -4120,7 +4134,7 @@
       <c r="M61" s="4"/>
       <c r="N61" s="4"/>
       <c r="O61" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4128,25 +4142,25 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>81</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I62" s="4" t="s">
         <v>64</v>
@@ -4160,7 +4174,7 @@
       <c r="M62" s="4"/>
       <c r="N62" s="4"/>
       <c r="O62" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4168,25 +4182,25 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I63" s="4" t="s">
         <v>64</v>
@@ -4200,7 +4214,7 @@
       <c r="M63" s="4"/>
       <c r="N63" s="4"/>
       <c r="O63" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4208,25 +4222,25 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>121</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I64" s="4" t="s">
         <v>64</v>
@@ -4240,7 +4254,7 @@
       <c r="M64" s="4"/>
       <c r="N64" s="4"/>
       <c r="O64" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4248,25 +4262,25 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>93</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G65" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I65" s="4" t="s">
         <v>64</v>
@@ -4280,7 +4294,7 @@
       <c r="M65" s="4"/>
       <c r="N65" s="4"/>
       <c r="O65" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4288,25 +4302,25 @@
         <v>65</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="G66" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>64</v>
@@ -4320,7 +4334,7 @@
       <c r="M66" s="4"/>
       <c r="N66" s="4"/>
       <c r="O66" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4328,25 +4342,25 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="I67" s="4" t="s">
         <v>64</v>
@@ -4360,7 +4374,7 @@
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4368,25 +4382,25 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>64</v>
@@ -4400,7 +4414,7 @@
       <c r="M68" s="4"/>
       <c r="N68" s="4"/>
       <c r="O68" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4408,25 +4422,25 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E69" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="H69" s="3" t="s">
         <v>246</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="G69" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>244</v>
       </c>
       <c r="I69" s="4" t="s">
         <v>64</v>
@@ -4440,7 +4454,7 @@
       <c r="M69" s="4"/>
       <c r="N69" s="4"/>
       <c r="O69" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4448,25 +4462,25 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>64</v>
@@ -4480,7 +4494,7 @@
       <c r="M70" s="4"/>
       <c r="N70" s="4"/>
       <c r="O70" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4488,25 +4502,25 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>81</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="I71" s="4" t="s">
         <v>64</v>
@@ -4520,7 +4534,7 @@
       <c r="M71" s="4"/>
       <c r="N71" s="4"/>
       <c r="O71" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4528,25 +4542,25 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>93</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I72" s="4" t="s">
         <v>64</v>
@@ -4560,7 +4574,7 @@
       <c r="M72" s="4"/>
       <c r="N72" s="4"/>
       <c r="O72" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4568,25 +4582,25 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I73" s="4" t="s">
         <v>64</v>
@@ -4600,7 +4614,7 @@
       <c r="M73" s="4"/>
       <c r="N73" s="4"/>
       <c r="O73" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4608,25 +4622,25 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I74" s="4" t="s">
         <v>64</v>
@@ -4640,7 +4654,7 @@
       <c r="M74" s="4"/>
       <c r="N74" s="4"/>
       <c r="O74" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4648,25 +4662,25 @@
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="I75" s="4" t="s">
         <v>64</v>
@@ -4680,7 +4694,7 @@
       <c r="M75" s="4"/>
       <c r="N75" s="4"/>
       <c r="O75" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4688,25 +4702,25 @@
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>64</v>
@@ -4720,7 +4734,7 @@
       <c r="M76" s="4"/>
       <c r="N76" s="4"/>
       <c r="O76" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4728,25 +4742,25 @@
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>106</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>64</v>
@@ -4760,7 +4774,7 @@
       <c r="M77" s="4"/>
       <c r="N77" s="4"/>
       <c r="O77" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4771,19 +4785,19 @@
         <v>15</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>21</v>
@@ -4800,7 +4814,7 @@
       <c r="M78" s="4"/>
       <c r="N78" s="4"/>
       <c r="O78" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4811,22 +4825,22 @@
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>64</v>
@@ -4840,7 +4854,7 @@
       <c r="M79" s="4"/>
       <c r="N79" s="4"/>
       <c r="O79" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4851,22 +4865,22 @@
         <v>15</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>35</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="I80" s="4" t="s">
         <v>64</v>
@@ -4880,7 +4894,7 @@
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
       <c r="O80" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4891,22 +4905,22 @@
         <v>15</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>93</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="I81" s="4" t="s">
         <v>64</v>
@@ -4920,7 +4934,7 @@
       <c r="M81" s="4"/>
       <c r="N81" s="4"/>
       <c r="O81" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4931,22 +4945,22 @@
         <v>49</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G82" s="3" t="s">
         <v>62</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="I82" s="4" t="s">
         <v>64</v>
@@ -4960,7 +4974,7 @@
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
       <c r="O82" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4971,22 +4985,22 @@
         <v>49</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>64</v>
@@ -5000,7 +5014,7 @@
       <c r="M83" s="4"/>
       <c r="N83" s="4"/>
       <c r="O83" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5011,22 +5025,22 @@
         <v>49</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="I84" s="4" t="s">
         <v>64</v>
@@ -5040,7 +5054,7 @@
       <c r="M84" s="4"/>
       <c r="N84" s="4"/>
       <c r="O84" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5048,25 +5062,25 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="G85" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>64</v>
@@ -5080,7 +5094,7 @@
       <c r="M85" s="4"/>
       <c r="N85" s="4"/>
       <c r="O85" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5088,25 +5102,25 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="G86" s="3" t="s">
         <v>127</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>64</v>
@@ -5120,7 +5134,7 @@
       <c r="M86" s="4"/>
       <c r="N86" s="4"/>
       <c r="O86" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5128,25 +5142,25 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="I87" s="4" t="s">
         <v>64</v>
@@ -5171,22 +5185,22 @@
         <v>41</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="I88" s="4" t="s">
         <v>64</v>
@@ -5211,22 +5225,22 @@
         <v>41</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="G89" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="H89" s="3" t="s">
         <v>321</v>
-      </c>
-      <c r="F89" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="G89" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="H89" s="3" t="s">
-        <v>319</v>
       </c>
       <c r="I89" s="4" t="s">
         <v>64</v>
@@ -7466,15 +7480,15 @@
   </sheetData>
   <autoFilter ref="A1:O200"/>
   <conditionalFormatting sqref="I2:I200">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Lien obtenu"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"Adresse invalide"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K200">
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>AND(K2&lt;&gt;"",K2&lt;=TODAY(),L2="",I2="Envoyé")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7515,12 +7529,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -7529,7 +7543,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
@@ -7538,16 +7552,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -7556,7 +7570,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -7565,7 +7579,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -7574,7 +7588,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Refus")</f>
@@ -7583,16 +7597,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
@@ -7601,7 +7615,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -7610,7 +7624,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -7619,12 +7633,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7632,13 +7646,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7745,7 +7759,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A25)</f>
@@ -7762,7 +7776,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
@@ -7779,7 +7793,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A27)</f>
@@ -7796,7 +7810,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A28)</f>
@@ -7813,7 +7827,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -7852,7 +7866,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7860,12 +7874,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7873,27 +7887,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7901,27 +7915,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection : 8 BGE régionales ajoutées (jours 7 et 8)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="379">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -1034,6 +1034,75 @@
   </si>
   <si>
     <t xml:space="preserve">Officiel (page Facebook)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BGE Hauts-de-France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@bge-hautsdefrance.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (site BGE, extrait de recherche), doc 2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BGE Picardie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@bge-picardie.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (site BGE, extrait de recherche)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BGE PaRIF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@bge-parif.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (flyer Versailles Grand Parc, 2021)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BGE Flandre Création</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@bge-flandrecreation.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (dossier Agefice, 2019)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BGE Auvergne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@bgeauvergne.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (proposition Agefice, 2019)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Envoi conseillé : jour 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BGE Côtes-d’Armor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@bge22.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (catalogue BGE Bretagne, 2018)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BGE Ille-et-Vilaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@bge35.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BGE Morbihan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@bge-morbihan.com</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de bord de la prospection</t>
@@ -5258,15 +5327,33 @@
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="3"/>
-      <c r="B90" s="3"/>
-      <c r="C90" s="3"/>
-      <c r="D90" s="3"/>
-      <c r="E90" s="3"/>
-      <c r="F90" s="3"/>
-      <c r="G90" s="3"/>
-      <c r="H90" s="3"/>
-      <c r="I90" s="4"/>
+      <c r="A90" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="F90" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="G90" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H90" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="I90" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="J90" s="5"/>
       <c r="K90" s="6" t="str">
         <f aca="false">IF(J90="","",WORKDAY(J90+4,1))</f>
@@ -5275,18 +5362,38 @@
       <c r="L90" s="5"/>
       <c r="M90" s="4"/>
       <c r="N90" s="4"/>
-      <c r="O90" s="4"/>
+      <c r="O90" s="4" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="3"/>
-      <c r="B91" s="3"/>
-      <c r="C91" s="3"/>
-      <c r="D91" s="3"/>
-      <c r="E91" s="3"/>
-      <c r="F91" s="3"/>
-      <c r="G91" s="3"/>
-      <c r="H91" s="3"/>
-      <c r="I91" s="4"/>
+      <c r="A91" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="F91" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="G91" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H91" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="I91" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="J91" s="5"/>
       <c r="K91" s="6" t="str">
         <f aca="false">IF(J91="","",WORKDAY(J91+4,1))</f>
@@ -5295,18 +5402,38 @@
       <c r="L91" s="5"/>
       <c r="M91" s="4"/>
       <c r="N91" s="4"/>
-      <c r="O91" s="4"/>
+      <c r="O91" s="4" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="3"/>
-      <c r="B92" s="3"/>
-      <c r="C92" s="3"/>
-      <c r="D92" s="3"/>
-      <c r="E92" s="3"/>
-      <c r="F92" s="3"/>
-      <c r="G92" s="3"/>
-      <c r="H92" s="3"/>
-      <c r="I92" s="4"/>
+      <c r="A92" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E92" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="F92" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="G92" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H92" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="I92" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="J92" s="5"/>
       <c r="K92" s="6" t="str">
         <f aca="false">IF(J92="","",WORKDAY(J92+4,1))</f>
@@ -5315,18 +5442,38 @@
       <c r="L92" s="5"/>
       <c r="M92" s="4"/>
       <c r="N92" s="4"/>
-      <c r="O92" s="4"/>
+      <c r="O92" s="4" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="3"/>
-      <c r="B93" s="3"/>
-      <c r="C93" s="3"/>
-      <c r="D93" s="3"/>
-      <c r="E93" s="3"/>
-      <c r="F93" s="3"/>
-      <c r="G93" s="3"/>
-      <c r="H93" s="3"/>
-      <c r="I93" s="4"/>
+      <c r="A93" s="3" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E93" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="F93" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="G93" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H93" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="I93" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="J93" s="5"/>
       <c r="K93" s="6" t="str">
         <f aca="false">IF(J93="","",WORKDAY(J93+4,1))</f>
@@ -5335,18 +5482,38 @@
       <c r="L93" s="5"/>
       <c r="M93" s="4"/>
       <c r="N93" s="4"/>
-      <c r="O93" s="4"/>
+      <c r="O93" s="4" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="3"/>
-      <c r="B94" s="3"/>
-      <c r="C94" s="3"/>
-      <c r="D94" s="3"/>
-      <c r="E94" s="3"/>
-      <c r="F94" s="3"/>
-      <c r="G94" s="3"/>
-      <c r="H94" s="3"/>
-      <c r="I94" s="4"/>
+      <c r="A94" s="3" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E94" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="F94" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="G94" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H94" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="I94" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="J94" s="5"/>
       <c r="K94" s="6" t="str">
         <f aca="false">IF(J94="","",WORKDAY(J94+4,1))</f>
@@ -5355,18 +5522,38 @@
       <c r="L94" s="5"/>
       <c r="M94" s="4"/>
       <c r="N94" s="4"/>
-      <c r="O94" s="4"/>
+      <c r="O94" s="4" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A95" s="3"/>
-      <c r="B95" s="3"/>
-      <c r="C95" s="3"/>
-      <c r="D95" s="3"/>
-      <c r="E95" s="3"/>
-      <c r="F95" s="3"/>
-      <c r="G95" s="3"/>
-      <c r="H95" s="3"/>
-      <c r="I95" s="4"/>
+      <c r="A95" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E95" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="F95" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="G95" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H95" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="I95" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="J95" s="5"/>
       <c r="K95" s="6" t="str">
         <f aca="false">IF(J95="","",WORKDAY(J95+4,1))</f>
@@ -5375,18 +5562,38 @@
       <c r="L95" s="5"/>
       <c r="M95" s="4"/>
       <c r="N95" s="4"/>
-      <c r="O95" s="4"/>
+      <c r="O95" s="4" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A96" s="3"/>
-      <c r="B96" s="3"/>
-      <c r="C96" s="3"/>
-      <c r="D96" s="3"/>
-      <c r="E96" s="3"/>
-      <c r="F96" s="3"/>
-      <c r="G96" s="3"/>
-      <c r="H96" s="3"/>
-      <c r="I96" s="4"/>
+      <c r="A96" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E96" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="F96" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="G96" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H96" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="I96" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="J96" s="5"/>
       <c r="K96" s="6" t="str">
         <f aca="false">IF(J96="","",WORKDAY(J96+4,1))</f>
@@ -5395,18 +5602,38 @@
       <c r="L96" s="5"/>
       <c r="M96" s="4"/>
       <c r="N96" s="4"/>
-      <c r="O96" s="4"/>
+      <c r="O96" s="4" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A97" s="3"/>
-      <c r="B97" s="3"/>
-      <c r="C97" s="3"/>
-      <c r="D97" s="3"/>
-      <c r="E97" s="3"/>
-      <c r="F97" s="3"/>
-      <c r="G97" s="3"/>
-      <c r="H97" s="3"/>
-      <c r="I97" s="4"/>
+      <c r="A97" s="3" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E97" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="F97" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="G97" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H97" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="I97" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="J97" s="5"/>
       <c r="K97" s="6" t="str">
         <f aca="false">IF(J97="","",WORKDAY(J97+4,1))</f>
@@ -5415,7 +5642,9 @@
       <c r="L97" s="5"/>
       <c r="M97" s="4"/>
       <c r="N97" s="4"/>
-      <c r="O97" s="4"/>
+      <c r="O97" s="4" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3"/>
@@ -7529,30 +7758,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>325</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>326</v>
+        <v>349</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
-        <v>87</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>327</v>
+        <v>350</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>328</v>
+        <v>351</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
@@ -7561,7 +7790,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>329</v>
+        <v>352</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -7570,7 +7799,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>330</v>
+        <v>353</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -7579,7 +7808,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>331</v>
+        <v>354</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -7588,7 +7817,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>332</v>
+        <v>355</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Refus")</f>
@@ -7597,7 +7826,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>333</v>
+        <v>356</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
@@ -7606,7 +7835,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>334</v>
+        <v>357</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
@@ -7615,7 +7844,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>335</v>
+        <v>358</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -7624,7 +7853,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>336</v>
+        <v>359</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -7633,12 +7862,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>337</v>
+        <v>360</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>338</v>
+        <v>361</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7646,13 +7875,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>339</v>
+        <v>362</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>340</v>
+        <v>363</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>341</v>
+        <v>364</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7746,7 +7975,7 @@
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A24)</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C24" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A24,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
@@ -7827,11 +8056,11 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>342</v>
+        <v>365</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
@@ -7866,7 +8095,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>343</v>
+        <v>366</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7874,12 +8103,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>344</v>
+        <v>367</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>345</v>
+        <v>368</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7887,27 +8116,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>346</v>
+        <v>369</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>347</v>
+        <v>370</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>348</v>
+        <v>371</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>349</v>
+        <v>372</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>350</v>
+        <v>373</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7915,27 +8144,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>351</v>
+        <v>374</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>352</v>
+        <v>375</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>353</v>
+        <v>376</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>354</v>
+        <v>377</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>355</v>
+        <v>378</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection : brouillons sans destinataire supprimés
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -202,10 +202,10 @@
     <t xml:space="preserve">Un simulateur de seuil de TVA gratuit pour compléter votre guide auto-entrepreneur</t>
   </si>
   <si>
-    <t xml:space="preserve">À compléter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brouillon sans destinataire : passer par le formulaire du site, ou supprimer</t>
+    <t xml:space="preserve">Pas de réponse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brouillon supprimé le 19/10 (pas d’adresse publique) : passer par le formulaire du site si besoin</t>
   </si>
   <si>
     <t xml:space="preserve">Fédération</t>
@@ -7785,7 +7785,7 @@
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Prospection : réponse du Blog du Dirigeant (offre d'article sponsorisé)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="382">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -143,6 +143,15 @@
   </si>
   <si>
     <t xml:space="preserve">Une donnée inédite pour vos lecteurs dirigeants de TPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Répondu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19/10 : propose un article sponsorisé (500 € HT fourni, 650 € HT rédigé), lien dofollow. Réponse en attente de décision.</t>
   </si>
   <si>
     <t xml:space="preserve">Compta-Online</t>
@@ -1848,7 +1857,7 @@
         <v>27</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>46314</v>
@@ -1858,10 +1867,12 @@
         <v>46321</v>
       </c>
       <c r="L3" s="5"/>
-      <c r="M3" s="4"/>
+      <c r="M3" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="N3" s="4"/>
       <c r="O3" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1872,22 +1883,22 @@
         <v>15</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>22</v>
@@ -1914,22 +1925,22 @@
         <v>15</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>22</v>
@@ -1956,22 +1967,22 @@
         <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>22</v>
@@ -1995,28 +2006,28 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J7" s="5"/>
       <c r="K7" s="6" t="str">
@@ -2027,7 +2038,7 @@
       <c r="M7" s="4"/>
       <c r="N7" s="4"/>
       <c r="O7" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2035,25 +2046,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>22</v>
@@ -2077,25 +2088,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>52</v>
-      </c>
       <c r="H9" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>22</v>
@@ -2119,28 +2130,28 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J10" s="5"/>
       <c r="K10" s="6" t="str">
@@ -2151,7 +2162,7 @@
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
       <c r="O10" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2159,25 +2170,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>63</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>22</v>
@@ -2201,28 +2212,28 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J12" s="5"/>
       <c r="K12" s="6" t="str">
@@ -2233,7 +2244,7 @@
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
       <c r="O12" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2241,28 +2252,28 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J13" s="5"/>
       <c r="K13" s="6" t="str">
@@ -2273,7 +2284,7 @@
       <c r="M13" s="4"/>
       <c r="N13" s="4"/>
       <c r="O13" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2281,28 +2292,28 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>75</v>
-      </c>
       <c r="E14" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J14" s="5"/>
       <c r="K14" s="6" t="str">
@@ -2313,7 +2324,7 @@
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
       <c r="O14" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2321,28 +2332,28 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C15" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="G15" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J15" s="5"/>
       <c r="K15" s="6" t="str">
@@ -2353,7 +2364,7 @@
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
       <c r="O15" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2361,28 +2372,28 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J16" s="5"/>
       <c r="K16" s="6" t="str">
@@ -2393,7 +2404,7 @@
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
       <c r="O16" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2401,28 +2412,28 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J17" s="5"/>
       <c r="K17" s="6" t="str">
@@ -2433,7 +2444,7 @@
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
       <c r="O17" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2441,28 +2452,28 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D18" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G18" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="H18" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="I18" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J18" s="5"/>
       <c r="K18" s="6" t="str">
@@ -2473,7 +2484,7 @@
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
       <c r="O18" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2481,28 +2492,28 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J19" s="5"/>
       <c r="K19" s="6" t="str">
@@ -2513,7 +2524,7 @@
       <c r="M19" s="4"/>
       <c r="N19" s="4"/>
       <c r="O19" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2521,28 +2532,28 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J20" s="5"/>
       <c r="K20" s="6" t="str">
@@ -2553,7 +2564,7 @@
       <c r="M20" s="4"/>
       <c r="N20" s="4"/>
       <c r="O20" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2561,28 +2572,28 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J21" s="5"/>
       <c r="K21" s="6" t="str">
@@ -2593,7 +2604,7 @@
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
       <c r="O21" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2601,28 +2612,28 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J22" s="5"/>
       <c r="K22" s="6" t="str">
@@ -2633,7 +2644,7 @@
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
       <c r="O22" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2641,28 +2652,28 @@
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J23" s="5"/>
       <c r="K23" s="6" t="str">
@@ -2673,7 +2684,7 @@
       <c r="M23" s="4"/>
       <c r="N23" s="4"/>
       <c r="O23" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2681,28 +2692,28 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J24" s="5"/>
       <c r="K24" s="6" t="str">
@@ -2713,7 +2724,7 @@
       <c r="M24" s="4"/>
       <c r="N24" s="4"/>
       <c r="O24" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2721,28 +2732,28 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J25" s="5"/>
       <c r="K25" s="6" t="str">
@@ -2753,7 +2764,7 @@
       <c r="M25" s="4"/>
       <c r="N25" s="4"/>
       <c r="O25" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2761,25 +2772,25 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>84</v>
-      </c>
       <c r="E26" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I26" s="4" t="s">
         <v>22</v>
@@ -2803,28 +2814,28 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J27" s="5"/>
       <c r="K27" s="6" t="str">
@@ -2835,7 +2846,7 @@
       <c r="M27" s="4"/>
       <c r="N27" s="4"/>
       <c r="O27" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2843,28 +2854,28 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="J28" s="5" t="n">
         <v>46314</v>
@@ -2877,7 +2888,7 @@
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
       <c r="O28" s="4" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2885,25 +2896,25 @@
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I29" s="4" t="s">
         <v>22</v>
@@ -2927,25 +2938,25 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I30" s="4" t="s">
         <v>22</v>
@@ -2969,25 +2980,25 @@
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I31" s="4" t="s">
         <v>22</v>
@@ -3011,28 +3022,28 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C32" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="F32" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="D32" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>137</v>
-      </c>
       <c r="G32" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J32" s="5"/>
       <c r="K32" s="6" t="str">
@@ -3043,7 +3054,7 @@
       <c r="M32" s="4"/>
       <c r="N32" s="4"/>
       <c r="O32" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3051,28 +3062,28 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J33" s="5"/>
       <c r="K33" s="6" t="str">
@@ -3083,7 +3094,7 @@
       <c r="M33" s="4"/>
       <c r="N33" s="4"/>
       <c r="O33" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3091,28 +3102,28 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J34" s="5"/>
       <c r="K34" s="6" t="str">
@@ -3123,7 +3134,7 @@
       <c r="M34" s="4"/>
       <c r="N34" s="4"/>
       <c r="O34" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3131,28 +3142,28 @@
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J35" s="5"/>
       <c r="K35" s="6" t="str">
@@ -3163,7 +3174,7 @@
       <c r="M35" s="4"/>
       <c r="N35" s="4"/>
       <c r="O35" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3171,28 +3182,28 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J36" s="5"/>
       <c r="K36" s="6" t="str">
@@ -3203,7 +3214,7 @@
       <c r="M36" s="4"/>
       <c r="N36" s="4"/>
       <c r="O36" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3211,28 +3222,28 @@
         <v>36</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J37" s="5"/>
       <c r="K37" s="6" t="str">
@@ -3243,7 +3254,7 @@
       <c r="M37" s="4"/>
       <c r="N37" s="4"/>
       <c r="O37" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3251,28 +3262,28 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J38" s="5"/>
       <c r="K38" s="6" t="str">
@@ -3283,7 +3294,7 @@
       <c r="M38" s="4"/>
       <c r="N38" s="4"/>
       <c r="O38" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3291,28 +3302,28 @@
         <v>38</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J39" s="5"/>
       <c r="K39" s="6" t="str">
@@ -3323,7 +3334,7 @@
       <c r="M39" s="4"/>
       <c r="N39" s="4"/>
       <c r="O39" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3331,28 +3342,28 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J40" s="5"/>
       <c r="K40" s="6" t="str">
@@ -3363,7 +3374,7 @@
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
       <c r="O40" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3371,28 +3382,28 @@
         <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J41" s="5"/>
       <c r="K41" s="6" t="str">
@@ -3403,7 +3414,7 @@
       <c r="M41" s="4"/>
       <c r="N41" s="4"/>
       <c r="O41" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3411,28 +3422,28 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J42" s="5"/>
       <c r="K42" s="6" t="str">
@@ -3443,7 +3454,7 @@
       <c r="M42" s="4"/>
       <c r="N42" s="4"/>
       <c r="O42" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3451,28 +3462,28 @@
         <v>42</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D43" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G43" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="G43" s="3" t="s">
-        <v>90</v>
-      </c>
       <c r="H43" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J43" s="5"/>
       <c r="K43" s="6" t="str">
@@ -3483,7 +3494,7 @@
       <c r="M43" s="4"/>
       <c r="N43" s="4"/>
       <c r="O43" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3491,28 +3502,28 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J44" s="5"/>
       <c r="K44" s="6" t="str">
@@ -3523,7 +3534,7 @@
       <c r="M44" s="4"/>
       <c r="N44" s="4"/>
       <c r="O44" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3531,28 +3542,28 @@
         <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J45" s="5"/>
       <c r="K45" s="6" t="str">
@@ -3563,7 +3574,7 @@
       <c r="M45" s="4"/>
       <c r="N45" s="4"/>
       <c r="O45" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3571,28 +3582,28 @@
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D46" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C46" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>84</v>
-      </c>
       <c r="E46" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J46" s="5"/>
       <c r="K46" s="6" t="str">
@@ -3603,7 +3614,7 @@
       <c r="M46" s="4"/>
       <c r="N46" s="4"/>
       <c r="O46" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3611,28 +3622,28 @@
         <v>46</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J47" s="5"/>
       <c r="K47" s="6" t="str">
@@ -3643,7 +3654,7 @@
       <c r="M47" s="4"/>
       <c r="N47" s="4"/>
       <c r="O47" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3651,28 +3662,28 @@
         <v>47</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J48" s="5"/>
       <c r="K48" s="6" t="str">
@@ -3683,7 +3694,7 @@
       <c r="M48" s="4"/>
       <c r="N48" s="4"/>
       <c r="O48" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3691,28 +3702,28 @@
         <v>48</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J49" s="5"/>
       <c r="K49" s="6" t="str">
@@ -3723,7 +3734,7 @@
       <c r="M49" s="4"/>
       <c r="N49" s="4"/>
       <c r="O49" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3731,28 +3742,28 @@
         <v>49</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F50" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H50" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="G50" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="H50" s="3" t="s">
-        <v>190</v>
-      </c>
       <c r="I50" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J50" s="5"/>
       <c r="K50" s="6" t="str">
@@ -3763,7 +3774,7 @@
       <c r="M50" s="4"/>
       <c r="N50" s="4"/>
       <c r="O50" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3771,28 +3782,28 @@
         <v>50</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J51" s="5"/>
       <c r="K51" s="6" t="str">
@@ -3803,7 +3814,7 @@
       <c r="M51" s="4"/>
       <c r="N51" s="4"/>
       <c r="O51" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3811,28 +3822,28 @@
         <v>51</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J52" s="5"/>
       <c r="K52" s="6" t="str">
@@ -3843,7 +3854,7 @@
       <c r="M52" s="4"/>
       <c r="N52" s="4"/>
       <c r="O52" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3851,28 +3862,28 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J53" s="5"/>
       <c r="K53" s="6" t="str">
@@ -3883,7 +3894,7 @@
       <c r="M53" s="4"/>
       <c r="N53" s="4"/>
       <c r="O53" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3891,28 +3902,28 @@
         <v>53</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J54" s="5"/>
       <c r="K54" s="6" t="str">
@@ -3923,7 +3934,7 @@
       <c r="M54" s="4"/>
       <c r="N54" s="4"/>
       <c r="O54" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3931,28 +3942,28 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J55" s="5"/>
       <c r="K55" s="6" t="str">
@@ -3963,7 +3974,7 @@
       <c r="M55" s="4"/>
       <c r="N55" s="4"/>
       <c r="O55" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3971,28 +3982,28 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J56" s="5"/>
       <c r="K56" s="6" t="str">
@@ -4003,7 +4014,7 @@
       <c r="M56" s="4"/>
       <c r="N56" s="4"/>
       <c r="O56" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4011,28 +4022,28 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J57" s="5"/>
       <c r="K57" s="6" t="str">
@@ -4043,7 +4054,7 @@
       <c r="M57" s="4"/>
       <c r="N57" s="4"/>
       <c r="O57" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4051,28 +4062,28 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J58" s="5"/>
       <c r="K58" s="6" t="str">
@@ -4083,7 +4094,7 @@
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
       <c r="O58" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4091,28 +4102,28 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J59" s="5"/>
       <c r="K59" s="6" t="str">
@@ -4123,7 +4134,7 @@
       <c r="M59" s="4"/>
       <c r="N59" s="4"/>
       <c r="O59" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4131,28 +4142,28 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F60" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H60" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="G60" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="H60" s="3" t="s">
-        <v>219</v>
-      </c>
       <c r="I60" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J60" s="5"/>
       <c r="K60" s="6" t="str">
@@ -4163,7 +4174,7 @@
       <c r="M60" s="4"/>
       <c r="N60" s="4"/>
       <c r="O60" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4171,28 +4182,28 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F61" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H61" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="G61" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="H61" s="3" t="s">
-        <v>219</v>
-      </c>
       <c r="I61" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J61" s="5"/>
       <c r="K61" s="6" t="str">
@@ -4203,7 +4214,7 @@
       <c r="M61" s="4"/>
       <c r="N61" s="4"/>
       <c r="O61" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4211,28 +4222,28 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C62" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="F62" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="D62" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="F62" s="3" t="s">
+      <c r="G62" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H62" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="G62" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="H62" s="3" t="s">
-        <v>219</v>
-      </c>
       <c r="I62" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J62" s="5"/>
       <c r="K62" s="6" t="str">
@@ -4243,7 +4254,7 @@
       <c r="M62" s="4"/>
       <c r="N62" s="4"/>
       <c r="O62" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4251,28 +4262,28 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="F63" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H63" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="G63" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="H63" s="3" t="s">
-        <v>219</v>
-      </c>
       <c r="I63" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J63" s="5"/>
       <c r="K63" s="6" t="str">
@@ -4283,7 +4294,7 @@
       <c r="M63" s="4"/>
       <c r="N63" s="4"/>
       <c r="O63" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4291,28 +4302,28 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="F64" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H64" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="G64" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="H64" s="3" t="s">
-        <v>219</v>
-      </c>
       <c r="I64" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J64" s="5"/>
       <c r="K64" s="6" t="str">
@@ -4323,7 +4334,7 @@
       <c r="M64" s="4"/>
       <c r="N64" s="4"/>
       <c r="O64" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4331,28 +4342,28 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F65" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H65" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="G65" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="H65" s="3" t="s">
-        <v>219</v>
-      </c>
       <c r="I65" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J65" s="5"/>
       <c r="K65" s="6" t="str">
@@ -4363,7 +4374,7 @@
       <c r="M65" s="4"/>
       <c r="N65" s="4"/>
       <c r="O65" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4371,28 +4382,28 @@
         <v>65</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J66" s="5"/>
       <c r="K66" s="6" t="str">
@@ -4403,7 +4414,7 @@
       <c r="M66" s="4"/>
       <c r="N66" s="4"/>
       <c r="O66" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4411,28 +4422,28 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J67" s="5"/>
       <c r="K67" s="6" t="str">
@@ -4443,7 +4454,7 @@
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4451,28 +4462,28 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J68" s="5"/>
       <c r="K68" s="6" t="str">
@@ -4483,7 +4494,7 @@
       <c r="M68" s="4"/>
       <c r="N68" s="4"/>
       <c r="O68" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4491,28 +4502,28 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="F69" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="H69" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="G69" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>246</v>
-      </c>
       <c r="I69" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J69" s="5"/>
       <c r="K69" s="6" t="str">
@@ -4523,7 +4534,7 @@
       <c r="M69" s="4"/>
       <c r="N69" s="4"/>
       <c r="O69" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4531,28 +4542,28 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J70" s="5"/>
       <c r="K70" s="6" t="str">
@@ -4563,7 +4574,7 @@
       <c r="M70" s="4"/>
       <c r="N70" s="4"/>
       <c r="O70" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4571,28 +4582,28 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J71" s="5"/>
       <c r="K71" s="6" t="str">
@@ -4603,7 +4614,7 @@
       <c r="M71" s="4"/>
       <c r="N71" s="4"/>
       <c r="O71" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4611,28 +4622,28 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J72" s="5"/>
       <c r="K72" s="6" t="str">
@@ -4643,7 +4654,7 @@
       <c r="M72" s="4"/>
       <c r="N72" s="4"/>
       <c r="O72" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4651,28 +4662,28 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J73" s="5"/>
       <c r="K73" s="6" t="str">
@@ -4683,7 +4694,7 @@
       <c r="M73" s="4"/>
       <c r="N73" s="4"/>
       <c r="O73" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4691,28 +4702,28 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J74" s="5"/>
       <c r="K74" s="6" t="str">
@@ -4723,7 +4734,7 @@
       <c r="M74" s="4"/>
       <c r="N74" s="4"/>
       <c r="O74" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4731,28 +4742,28 @@
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="I75" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J75" s="5"/>
       <c r="K75" s="6" t="str">
@@ -4763,7 +4774,7 @@
       <c r="M75" s="4"/>
       <c r="N75" s="4"/>
       <c r="O75" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4771,28 +4782,28 @@
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J76" s="5"/>
       <c r="K76" s="6" t="str">
@@ -4803,7 +4814,7 @@
       <c r="M76" s="4"/>
       <c r="N76" s="4"/>
       <c r="O76" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4811,28 +4822,28 @@
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J77" s="5"/>
       <c r="K77" s="6" t="str">
@@ -4843,7 +4854,7 @@
       <c r="M77" s="4"/>
       <c r="N77" s="4"/>
       <c r="O77" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4854,25 +4865,25 @@
         <v>15</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>21</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J78" s="5"/>
       <c r="K78" s="6" t="str">
@@ -4883,7 +4894,7 @@
       <c r="M78" s="4"/>
       <c r="N78" s="4"/>
       <c r="O78" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4894,25 +4905,25 @@
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J79" s="5"/>
       <c r="K79" s="6" t="str">
@@ -4923,7 +4934,7 @@
       <c r="M79" s="4"/>
       <c r="N79" s="4"/>
       <c r="O79" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4934,25 +4945,25 @@
         <v>15</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J80" s="5"/>
       <c r="K80" s="6" t="str">
@@ -4963,7 +4974,7 @@
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
       <c r="O80" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4974,25 +4985,25 @@
         <v>15</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J81" s="5"/>
       <c r="K81" s="6" t="str">
@@ -5003,7 +5014,7 @@
       <c r="M81" s="4"/>
       <c r="N81" s="4"/>
       <c r="O81" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5011,28 +5022,28 @@
         <v>81</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G82" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J82" s="5"/>
       <c r="K82" s="6" t="str">
@@ -5043,7 +5054,7 @@
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
       <c r="O82" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5051,28 +5062,28 @@
         <v>82</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J83" s="5"/>
       <c r="K83" s="6" t="str">
@@ -5083,7 +5094,7 @@
       <c r="M83" s="4"/>
       <c r="N83" s="4"/>
       <c r="O83" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5091,28 +5102,28 @@
         <v>83</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J84" s="5"/>
       <c r="K84" s="6" t="str">
@@ -5123,7 +5134,7 @@
       <c r="M84" s="4"/>
       <c r="N84" s="4"/>
       <c r="O84" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5131,28 +5142,28 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="I85" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J85" s="5"/>
       <c r="K85" s="6" t="str">
@@ -5163,7 +5174,7 @@
       <c r="M85" s="4"/>
       <c r="N85" s="4"/>
       <c r="O85" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5171,28 +5182,28 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="F86" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="G86" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H86" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="G86" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="H86" s="3" t="s">
-        <v>309</v>
-      </c>
       <c r="I86" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J86" s="5"/>
       <c r="K86" s="6" t="str">
@@ -5203,7 +5214,7 @@
       <c r="M86" s="4"/>
       <c r="N86" s="4"/>
       <c r="O86" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5211,28 +5222,28 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J87" s="5"/>
       <c r="K87" s="6" t="str">
@@ -5243,7 +5254,7 @@
       <c r="M87" s="4"/>
       <c r="N87" s="4"/>
       <c r="O87" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5251,28 +5262,28 @@
         <v>87</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J88" s="5"/>
       <c r="K88" s="6" t="str">
@@ -5283,7 +5294,7 @@
       <c r="M88" s="4"/>
       <c r="N88" s="4"/>
       <c r="O88" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5291,28 +5302,28 @@
         <v>88</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="G89" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="F89" s="3" t="s">
+      <c r="H89" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="G89" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="H89" s="3" t="s">
-        <v>321</v>
-      </c>
       <c r="I89" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J89" s="5"/>
       <c r="K89" s="6" t="str">
@@ -5323,7 +5334,7 @@
       <c r="M89" s="4"/>
       <c r="N89" s="4"/>
       <c r="O89" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5331,28 +5342,28 @@
         <v>89</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J90" s="5"/>
       <c r="K90" s="6" t="str">
@@ -5363,7 +5374,7 @@
       <c r="M90" s="4"/>
       <c r="N90" s="4"/>
       <c r="O90" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5371,28 +5382,28 @@
         <v>90</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J91" s="5"/>
       <c r="K91" s="6" t="str">
@@ -5403,7 +5414,7 @@
       <c r="M91" s="4"/>
       <c r="N91" s="4"/>
       <c r="O91" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5411,28 +5422,28 @@
         <v>91</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J92" s="5"/>
       <c r="K92" s="6" t="str">
@@ -5443,7 +5454,7 @@
       <c r="M92" s="4"/>
       <c r="N92" s="4"/>
       <c r="O92" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5451,28 +5462,28 @@
         <v>92</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J93" s="5"/>
       <c r="K93" s="6" t="str">
@@ -5483,7 +5494,7 @@
       <c r="M93" s="4"/>
       <c r="N93" s="4"/>
       <c r="O93" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5491,28 +5502,28 @@
         <v>93</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="G94" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J94" s="5"/>
       <c r="K94" s="6" t="str">
@@ -5523,7 +5534,7 @@
       <c r="M94" s="4"/>
       <c r="N94" s="4"/>
       <c r="O94" s="4" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5531,28 +5542,28 @@
         <v>94</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="G95" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H95" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I95" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J95" s="5"/>
       <c r="K95" s="6" t="str">
@@ -5563,7 +5574,7 @@
       <c r="M95" s="4"/>
       <c r="N95" s="4"/>
       <c r="O95" s="4" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5571,28 +5582,28 @@
         <v>95</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I96" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J96" s="5"/>
       <c r="K96" s="6" t="str">
@@ -5603,7 +5614,7 @@
       <c r="M96" s="4"/>
       <c r="N96" s="4"/>
       <c r="O96" s="4" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5611,28 +5622,28 @@
         <v>96</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C97" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E97" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="F97" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="D97" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E97" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="F97" s="3" t="s">
-        <v>343</v>
-      </c>
       <c r="G97" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="J97" s="5"/>
       <c r="K97" s="6" t="str">
@@ -5643,7 +5654,7 @@
       <c r="M97" s="4"/>
       <c r="N97" s="4"/>
       <c r="O97" s="4" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7758,12 +7769,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -7772,7 +7783,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
@@ -7781,7 +7792,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
@@ -7790,7 +7801,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -7799,16 +7810,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -7817,7 +7828,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Refus")</f>
@@ -7826,7 +7837,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
@@ -7835,16 +7846,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0</v>
+        <v>0.0769230769230769</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -7853,7 +7864,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -7862,12 +7873,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7875,13 +7886,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7903,7 +7914,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A20)</f>
@@ -7920,7 +7931,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B21" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A21)</f>
@@ -7937,7 +7948,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A22)</f>
@@ -7954,7 +7965,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A23)</f>
@@ -7971,7 +7982,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A24)</f>
@@ -7988,7 +7999,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A25)</f>
@@ -8005,7 +8016,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
@@ -8022,7 +8033,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A27)</f>
@@ -8039,7 +8050,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A28)</f>
@@ -8056,7 +8067,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -8095,7 +8106,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8103,12 +8114,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8116,27 +8127,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8144,27 +8155,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection : 13 envois du 20/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="381">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -494,9 +494,6 @@
   </si>
   <si>
     <t xml:space="preserve">entreprendre@indre.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Envoi conseillé : jour 2</t>
   </si>
   <si>
     <t xml:space="preserve">CCI Loir-et-Cher</t>
@@ -3043,18 +3040,20 @@
         <v>66</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J32" s="5"/>
-      <c r="K32" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K32" s="6" t="n">
         <f aca="false">IF(J32="","",WORKDAY(J32+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L32" s="5"/>
       <c r="M32" s="4"/>
       <c r="N32" s="4"/>
       <c r="O32" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3065,13 +3064,13 @@
         <v>60</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>105</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>140</v>
@@ -3083,18 +3082,20 @@
         <v>66</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J33" s="5"/>
-      <c r="K33" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K33" s="6" t="n">
         <f aca="false">IF(J33="","",WORKDAY(J33+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L33" s="5"/>
       <c r="M33" s="4"/>
       <c r="N33" s="4"/>
       <c r="O33" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3105,16 +3106,16 @@
         <v>60</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E34" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="F34" s="3" t="s">
         <v>149</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>150</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>65</v>
@@ -3123,18 +3124,20 @@
         <v>66</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J34" s="5"/>
-      <c r="K34" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J34" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K34" s="6" t="n">
         <f aca="false">IF(J34="","",WORKDAY(J34+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L34" s="5"/>
       <c r="M34" s="4"/>
       <c r="N34" s="4"/>
       <c r="O34" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3145,16 +3148,16 @@
         <v>60</v>
       </c>
       <c r="C35" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="E35" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="F35" s="3" t="s">
         <v>153</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>154</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>65</v>
@@ -3163,18 +3166,20 @@
         <v>66</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J35" s="5"/>
-      <c r="K35" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K35" s="6" t="n">
         <f aca="false">IF(J35="","",WORKDAY(J35+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L35" s="5"/>
       <c r="M35" s="4"/>
       <c r="N35" s="4"/>
       <c r="O35" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3185,16 +3190,16 @@
         <v>60</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E36" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>157</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>65</v>
@@ -3203,18 +3208,20 @@
         <v>66</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J36" s="5"/>
-      <c r="K36" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J36" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K36" s="6" t="n">
         <f aca="false">IF(J36="","",WORKDAY(J36+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L36" s="5"/>
       <c r="M36" s="4"/>
       <c r="N36" s="4"/>
       <c r="O36" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3225,16 +3232,16 @@
         <v>60</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>100</v>
       </c>
       <c r="E37" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>159</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>160</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>65</v>
@@ -3243,18 +3250,20 @@
         <v>66</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J37" s="5"/>
-      <c r="K37" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J37" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K37" s="6" t="n">
         <f aca="false">IF(J37="","",WORKDAY(J37+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L37" s="5"/>
       <c r="M37" s="4"/>
       <c r="N37" s="4"/>
       <c r="O37" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3265,16 +3274,16 @@
         <v>60</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E38" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F38" s="3" t="s">
         <v>162</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>163</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>65</v>
@@ -3283,18 +3292,20 @@
         <v>66</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J38" s="5"/>
-      <c r="K38" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J38" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K38" s="6" t="n">
         <f aca="false">IF(J38="","",WORKDAY(J38+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L38" s="5"/>
       <c r="M38" s="4"/>
       <c r="N38" s="4"/>
       <c r="O38" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3305,16 +3316,16 @@
         <v>60</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>65</v>
@@ -3323,18 +3334,20 @@
         <v>66</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J39" s="5"/>
-      <c r="K39" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J39" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K39" s="6" t="n">
         <f aca="false">IF(J39="","",WORKDAY(J39+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L39" s="5"/>
       <c r="M39" s="4"/>
       <c r="N39" s="4"/>
       <c r="O39" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3345,16 +3358,16 @@
         <v>90</v>
       </c>
       <c r="C40" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E40" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="D40" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E40" s="3" t="s">
+      <c r="F40" s="3" t="s">
         <v>167</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>168</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>93</v>
@@ -3363,18 +3376,20 @@
         <v>94</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J40" s="5"/>
-      <c r="K40" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J40" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K40" s="6" t="n">
         <f aca="false">IF(J40="","",WORKDAY(J40+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L40" s="5"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4"/>
       <c r="O40" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3385,13 +3400,13 @@
         <v>90</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>80</v>
@@ -3425,16 +3440,16 @@
         <v>90</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E42" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="F42" s="3" t="s">
         <v>172</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>173</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>93</v>
@@ -3443,18 +3458,20 @@
         <v>94</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J42" s="5"/>
-      <c r="K42" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J42" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K42" s="6" t="n">
         <f aca="false">IF(J42="","",WORKDAY(J42+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L42" s="5"/>
       <c r="M42" s="4"/>
       <c r="N42" s="4"/>
       <c r="O42" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3465,16 +3482,16 @@
         <v>90</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>93</v>
@@ -3483,18 +3500,20 @@
         <v>94</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J43" s="5"/>
-      <c r="K43" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J43" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K43" s="6" t="n">
         <f aca="false">IF(J43="","",WORKDAY(J43+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L43" s="5"/>
       <c r="M43" s="4"/>
       <c r="N43" s="4"/>
       <c r="O43" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3505,16 +3524,16 @@
         <v>90</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E44" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="F44" s="3" t="s">
         <v>177</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>178</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>93</v>
@@ -3523,18 +3542,20 @@
         <v>94</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J44" s="5"/>
-      <c r="K44" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J44" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K44" s="6" t="n">
         <f aca="false">IF(J44="","",WORKDAY(J44+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L44" s="5"/>
       <c r="M44" s="4"/>
       <c r="N44" s="4"/>
       <c r="O44" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3545,16 +3566,16 @@
         <v>90</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>93</v>
@@ -3563,18 +3584,20 @@
         <v>94</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J45" s="5"/>
-      <c r="K45" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J45" s="5" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K45" s="6" t="n">
         <f aca="false">IF(J45="","",WORKDAY(J45+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L45" s="5"/>
       <c r="M45" s="4"/>
       <c r="N45" s="4"/>
       <c r="O45" s="4" t="s">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3585,16 +3608,16 @@
         <v>90</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>93</v>
@@ -3614,7 +3637,7 @@
       <c r="M46" s="4"/>
       <c r="N46" s="4"/>
       <c r="O46" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3625,16 +3648,16 @@
         <v>90</v>
       </c>
       <c r="C47" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E47" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="D47" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>185</v>
-      </c>
       <c r="F47" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>93</v>
@@ -3654,7 +3677,7 @@
       <c r="M47" s="4"/>
       <c r="N47" s="4"/>
       <c r="O47" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3665,16 +3688,16 @@
         <v>90</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E48" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F48" s="3" t="s">
         <v>187</v>
-      </c>
-      <c r="F48" s="3" t="s">
-        <v>188</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>93</v>
@@ -3694,7 +3717,7 @@
       <c r="M48" s="4"/>
       <c r="N48" s="4"/>
       <c r="O48" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3702,25 +3725,25 @@
         <v>48</v>
       </c>
       <c r="B49" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>189</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>190</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E49" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="F49" s="3" t="s">
         <v>191</v>
-      </c>
-      <c r="F49" s="3" t="s">
-        <v>192</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>67</v>
@@ -3742,25 +3765,25 @@
         <v>49</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E50" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F50" s="3" t="s">
         <v>195</v>
-      </c>
-      <c r="F50" s="3" t="s">
-        <v>196</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I50" s="4" t="s">
         <v>67</v>
@@ -3774,7 +3797,7 @@
       <c r="M50" s="4"/>
       <c r="N50" s="4"/>
       <c r="O50" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3782,25 +3805,25 @@
         <v>50</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>67</v>
@@ -3822,25 +3845,25 @@
         <v>51</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>67</v>
@@ -3862,25 +3885,25 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>67</v>
@@ -3902,25 +3925,25 @@
         <v>53</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G54" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I54" s="4" t="s">
         <v>67</v>
@@ -3942,25 +3965,25 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E55" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F55" s="3" t="s">
         <v>206</v>
-      </c>
-      <c r="F55" s="3" t="s">
-        <v>207</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I55" s="4" t="s">
         <v>67</v>
@@ -3982,25 +4005,25 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E56" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="F56" s="3" t="s">
         <v>209</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>210</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I56" s="4" t="s">
         <v>67</v>
@@ -4014,7 +4037,7 @@
       <c r="M56" s="4"/>
       <c r="N56" s="4"/>
       <c r="O56" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4022,25 +4045,25 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E57" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F57" s="3" t="s">
         <v>212</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>213</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I57" s="4" t="s">
         <v>67</v>
@@ -4054,7 +4077,7 @@
       <c r="M57" s="4"/>
       <c r="N57" s="4"/>
       <c r="O57" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4062,25 +4085,25 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E58" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="F58" s="3" t="s">
         <v>215</v>
-      </c>
-      <c r="F58" s="3" t="s">
-        <v>216</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I58" s="4" t="s">
         <v>67</v>
@@ -4094,7 +4117,7 @@
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
       <c r="O58" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4102,25 +4125,25 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C59" s="3" t="s">
         <v>218</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>219</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E59" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="F59" s="3" t="s">
         <v>220</v>
-      </c>
-      <c r="F59" s="3" t="s">
-        <v>221</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I59" s="4" t="s">
         <v>67</v>
@@ -4134,7 +4157,7 @@
       <c r="M59" s="4"/>
       <c r="N59" s="4"/>
       <c r="O59" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4142,25 +4165,25 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E60" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="F60" s="3" t="s">
         <v>224</v>
-      </c>
-      <c r="F60" s="3" t="s">
-        <v>225</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I60" s="4" t="s">
         <v>67</v>
@@ -4174,7 +4197,7 @@
       <c r="M60" s="4"/>
       <c r="N60" s="4"/>
       <c r="O60" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4182,25 +4205,25 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I61" s="4" t="s">
         <v>67</v>
@@ -4214,7 +4237,7 @@
       <c r="M61" s="4"/>
       <c r="N61" s="4"/>
       <c r="O61" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4222,25 +4245,25 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I62" s="4" t="s">
         <v>67</v>
@@ -4254,7 +4277,7 @@
       <c r="M62" s="4"/>
       <c r="N62" s="4"/>
       <c r="O62" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4262,25 +4285,25 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I63" s="4" t="s">
         <v>67</v>
@@ -4294,7 +4317,7 @@
       <c r="M63" s="4"/>
       <c r="N63" s="4"/>
       <c r="O63" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4302,25 +4325,25 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I64" s="4" t="s">
         <v>67</v>
@@ -4334,7 +4357,7 @@
       <c r="M64" s="4"/>
       <c r="N64" s="4"/>
       <c r="O64" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4342,25 +4365,25 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G65" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I65" s="4" t="s">
         <v>67</v>
@@ -4374,7 +4397,7 @@
       <c r="M65" s="4"/>
       <c r="N65" s="4"/>
       <c r="O65" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4382,25 +4405,25 @@
         <v>65</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E66" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="F66" s="3" t="s">
         <v>237</v>
-      </c>
-      <c r="F66" s="3" t="s">
-        <v>238</v>
       </c>
       <c r="G66" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>67</v>
@@ -4414,7 +4437,7 @@
       <c r="M66" s="4"/>
       <c r="N66" s="4"/>
       <c r="O66" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4422,25 +4445,25 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="C67" s="3" t="s">
         <v>239</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>240</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="F67" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="F67" s="3" t="s">
+      <c r="G67" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="G67" s="3" t="s">
+      <c r="H67" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>244</v>
       </c>
       <c r="I67" s="4" t="s">
         <v>67</v>
@@ -4454,7 +4477,7 @@
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4462,25 +4485,25 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="F68" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="F68" s="3" t="s">
+      <c r="G68" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="H68" s="3" t="s">
         <v>248</v>
-      </c>
-      <c r="G68" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="H68" s="3" t="s">
-        <v>249</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>67</v>
@@ -4494,7 +4517,7 @@
       <c r="M68" s="4"/>
       <c r="N68" s="4"/>
       <c r="O68" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4502,25 +4525,25 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E69" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="F69" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="F69" s="3" t="s">
-        <v>252</v>
-      </c>
       <c r="G69" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I69" s="4" t="s">
         <v>67</v>
@@ -4534,7 +4557,7 @@
       <c r="M69" s="4"/>
       <c r="N69" s="4"/>
       <c r="O69" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4542,25 +4565,25 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E70" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F70" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="F70" s="3" t="s">
-        <v>255</v>
-      </c>
       <c r="G70" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>67</v>
@@ -4574,7 +4597,7 @@
       <c r="M70" s="4"/>
       <c r="N70" s="4"/>
       <c r="O70" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4582,25 +4605,25 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E71" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="F71" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="F71" s="3" t="s">
+      <c r="G71" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="G71" s="3" t="s">
+      <c r="H71" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="H71" s="3" t="s">
-        <v>260</v>
       </c>
       <c r="I71" s="4" t="s">
         <v>67</v>
@@ -4614,7 +4637,7 @@
       <c r="M71" s="4"/>
       <c r="N71" s="4"/>
       <c r="O71" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4622,25 +4645,25 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E72" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="F72" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="F72" s="3" t="s">
-        <v>263</v>
-      </c>
       <c r="G72" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I72" s="4" t="s">
         <v>67</v>
@@ -4654,7 +4677,7 @@
       <c r="M72" s="4"/>
       <c r="N72" s="4"/>
       <c r="O72" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4662,25 +4685,25 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E73" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="F73" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="F73" s="3" t="s">
-        <v>266</v>
-      </c>
       <c r="G73" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I73" s="4" t="s">
         <v>67</v>
@@ -4694,7 +4717,7 @@
       <c r="M73" s="4"/>
       <c r="N73" s="4"/>
       <c r="O73" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4702,25 +4725,25 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E74" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="F74" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="F74" s="3" t="s">
-        <v>269</v>
-      </c>
       <c r="G74" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I74" s="4" t="s">
         <v>67</v>
@@ -4734,7 +4757,7 @@
       <c r="M74" s="4"/>
       <c r="N74" s="4"/>
       <c r="O74" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4742,25 +4765,25 @@
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>100</v>
       </c>
       <c r="E75" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="F75" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="F75" s="3" t="s">
+      <c r="G75" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="H75" s="3" t="s">
         <v>272</v>
-      </c>
-      <c r="G75" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="H75" s="3" t="s">
-        <v>273</v>
       </c>
       <c r="I75" s="4" t="s">
         <v>67</v>
@@ -4774,7 +4797,7 @@
       <c r="M75" s="4"/>
       <c r="N75" s="4"/>
       <c r="O75" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4782,25 +4805,25 @@
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C76" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E76" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="D76" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E76" s="3" t="s">
+      <c r="F76" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="F76" s="3" t="s">
-        <v>276</v>
-      </c>
       <c r="G76" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>67</v>
@@ -4814,7 +4837,7 @@
       <c r="M76" s="4"/>
       <c r="N76" s="4"/>
       <c r="O76" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4822,25 +4845,25 @@
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E77" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="F77" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="F77" s="3" t="s">
-        <v>279</v>
-      </c>
       <c r="G77" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>67</v>
@@ -4854,7 +4877,7 @@
       <c r="M77" s="4"/>
       <c r="N77" s="4"/>
       <c r="O77" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4865,19 +4888,19 @@
         <v>15</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="F78" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="F78" s="3" t="s">
+      <c r="G78" s="3" t="s">
         <v>282</v>
-      </c>
-      <c r="G78" s="3" t="s">
-        <v>283</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>21</v>
@@ -4894,7 +4917,7 @@
       <c r="M78" s="4"/>
       <c r="N78" s="4"/>
       <c r="O78" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4905,22 +4928,22 @@
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="F79" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="F79" s="3" t="s">
+      <c r="G79" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="G79" s="3" t="s">
+      <c r="H79" s="3" t="s">
         <v>287</v>
-      </c>
-      <c r="H79" s="3" t="s">
-        <v>288</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>67</v>
@@ -4934,7 +4957,7 @@
       <c r="M79" s="4"/>
       <c r="N79" s="4"/>
       <c r="O79" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4945,22 +4968,22 @@
         <v>15</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F80" s="3" t="s">
         <v>290</v>
-      </c>
-      <c r="F80" s="3" t="s">
-        <v>291</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>38</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I80" s="4" t="s">
         <v>67</v>
@@ -4974,7 +4997,7 @@
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
       <c r="O80" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4985,22 +5008,22 @@
         <v>15</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E81" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="F81" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="F81" s="3" t="s">
-        <v>295</v>
-      </c>
       <c r="G81" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="H81" s="3" t="s">
         <v>287</v>
-      </c>
-      <c r="H81" s="3" t="s">
-        <v>288</v>
       </c>
       <c r="I81" s="4" t="s">
         <v>67</v>
@@ -5014,7 +5037,7 @@
       <c r="M81" s="4"/>
       <c r="N81" s="4"/>
       <c r="O81" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5025,22 +5048,22 @@
         <v>52</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G82" s="3" t="s">
         <v>65</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I82" s="4" t="s">
         <v>67</v>
@@ -5054,7 +5077,7 @@
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
       <c r="O82" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5065,22 +5088,22 @@
         <v>52</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="F83" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="F83" s="3" t="s">
+      <c r="G83" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="H83" s="3" t="s">
         <v>301</v>
-      </c>
-      <c r="G83" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="H83" s="3" t="s">
-        <v>302</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>67</v>
@@ -5094,7 +5117,7 @@
       <c r="M83" s="4"/>
       <c r="N83" s="4"/>
       <c r="O83" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5105,22 +5128,22 @@
         <v>52</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E84" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="F84" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="F84" s="3" t="s">
+      <c r="G84" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="G84" s="3" t="s">
+      <c r="H84" s="3" t="s">
         <v>306</v>
-      </c>
-      <c r="H84" s="3" t="s">
-        <v>307</v>
       </c>
       <c r="I84" s="4" t="s">
         <v>67</v>
@@ -5134,7 +5157,7 @@
       <c r="M84" s="4"/>
       <c r="N84" s="4"/>
       <c r="O84" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5142,25 +5165,25 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="C85" s="3" t="s">
         <v>308</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>309</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="F85" s="3" t="s">
         <v>310</v>
-      </c>
-      <c r="F85" s="3" t="s">
-        <v>311</v>
       </c>
       <c r="G85" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>67</v>
@@ -5174,7 +5197,7 @@
       <c r="M85" s="4"/>
       <c r="N85" s="4"/>
       <c r="O85" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5182,25 +5205,25 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>100</v>
       </c>
       <c r="E86" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="F86" s="3" t="s">
         <v>314</v>
-      </c>
-      <c r="F86" s="3" t="s">
-        <v>315</v>
       </c>
       <c r="G86" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>67</v>
@@ -5214,7 +5237,7 @@
       <c r="M86" s="4"/>
       <c r="N86" s="4"/>
       <c r="O86" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5222,25 +5245,25 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="F87" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="F87" s="3" t="s">
+      <c r="G87" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="G87" s="3" t="s">
+      <c r="H87" s="3" t="s">
         <v>319</v>
-      </c>
-      <c r="H87" s="3" t="s">
-        <v>320</v>
       </c>
       <c r="I87" s="4" t="s">
         <v>67</v>
@@ -5265,22 +5288,22 @@
         <v>44</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E88" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="G88" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="F88" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="G88" s="3" t="s">
+      <c r="H88" s="3" t="s">
         <v>323</v>
-      </c>
-      <c r="H88" s="3" t="s">
-        <v>324</v>
       </c>
       <c r="I88" s="4" t="s">
         <v>67</v>
@@ -5305,22 +5328,22 @@
         <v>44</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="F89" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="F89" s="3" t="s">
-        <v>327</v>
-      </c>
       <c r="G89" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="H89" s="3" t="s">
         <v>323</v>
-      </c>
-      <c r="H89" s="3" t="s">
-        <v>324</v>
       </c>
       <c r="I89" s="4" t="s">
         <v>67</v>
@@ -5345,22 +5368,22 @@
         <v>126</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E90" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="F90" s="3" t="s">
         <v>329</v>
-      </c>
-      <c r="F90" s="3" t="s">
-        <v>330</v>
       </c>
       <c r="G90" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I90" s="4" t="s">
         <v>67</v>
@@ -5374,7 +5397,7 @@
       <c r="M90" s="4"/>
       <c r="N90" s="4"/>
       <c r="O90" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5385,22 +5408,22 @@
         <v>126</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E91" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="F91" s="3" t="s">
         <v>332</v>
-      </c>
-      <c r="F91" s="3" t="s">
-        <v>333</v>
       </c>
       <c r="G91" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I91" s="4" t="s">
         <v>67</v>
@@ -5414,7 +5437,7 @@
       <c r="M91" s="4"/>
       <c r="N91" s="4"/>
       <c r="O91" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5425,22 +5448,22 @@
         <v>126</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E92" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="F92" s="3" t="s">
         <v>335</v>
-      </c>
-      <c r="F92" s="3" t="s">
-        <v>336</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I92" s="4" t="s">
         <v>67</v>
@@ -5454,7 +5477,7 @@
       <c r="M92" s="4"/>
       <c r="N92" s="4"/>
       <c r="O92" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5465,22 +5488,22 @@
         <v>126</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E93" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="F93" s="3" t="s">
         <v>338</v>
-      </c>
-      <c r="F93" s="3" t="s">
-        <v>339</v>
       </c>
       <c r="G93" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I93" s="4" t="s">
         <v>67</v>
@@ -5494,7 +5517,7 @@
       <c r="M93" s="4"/>
       <c r="N93" s="4"/>
       <c r="O93" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5505,22 +5528,22 @@
         <v>126</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E94" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="F94" s="3" t="s">
         <v>341</v>
-      </c>
-      <c r="F94" s="3" t="s">
-        <v>342</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I94" s="4" t="s">
         <v>67</v>
@@ -5534,7 +5557,7 @@
       <c r="M94" s="4"/>
       <c r="N94" s="4"/>
       <c r="O94" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5545,22 +5568,22 @@
         <v>126</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E95" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="F95" s="3" t="s">
         <v>345</v>
-      </c>
-      <c r="F95" s="3" t="s">
-        <v>346</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H95" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I95" s="4" t="s">
         <v>67</v>
@@ -5574,7 +5597,7 @@
       <c r="M95" s="4"/>
       <c r="N95" s="4"/>
       <c r="O95" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5585,22 +5608,22 @@
         <v>126</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="G96" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I96" s="4" t="s">
         <v>67</v>
@@ -5614,7 +5637,7 @@
       <c r="M96" s="4"/>
       <c r="N96" s="4"/>
       <c r="O96" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5625,22 +5648,22 @@
         <v>126</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="G97" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I97" s="4" t="s">
         <v>67</v>
@@ -5654,7 +5677,7 @@
       <c r="M97" s="4"/>
       <c r="N97" s="4"/>
       <c r="O97" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7769,12 +7792,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -7783,25 +7806,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>82</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>13</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -7810,7 +7833,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -7819,7 +7842,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -7828,7 +7851,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Refus")</f>
@@ -7837,7 +7860,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
@@ -7846,16 +7869,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.0769230769230769</v>
+        <v>0.0384615384615385</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -7864,7 +7887,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -7873,12 +7896,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7886,13 +7909,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>365</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="D18" s="9" t="s">
         <v>366</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7956,7 +7979,7 @@
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A22,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D22" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A22,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -7973,7 +7996,7 @@
       </c>
       <c r="C23" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A23,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D23" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A23,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -7999,7 +8022,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A25)</f>
@@ -8016,7 +8039,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
@@ -8033,7 +8056,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A27)</f>
@@ -8050,7 +8073,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A28)</f>
@@ -8067,7 +8090,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -8075,7 +8098,7 @@
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">SUM(D19:D28)</f>
@@ -8106,7 +8129,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8114,12 +8137,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8127,27 +8150,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8155,27 +8178,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection 21/10 : 12 envois, 1 refus STOP, 1 rebond
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="384">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -580,12 +580,21 @@
     <t xml:space="preserve">Officiel (cma-idf.fr)</t>
   </si>
   <si>
+    <t xml:space="preserve">Refus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20/10 : réponse STOP de contact.75@cma-idf.fr. Plus aucun mail.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CMA Rhône</t>
   </si>
   <si>
     <t xml:space="preserve">contact@cma-auvergnerhonealpes.fr</t>
   </si>
   <si>
+    <t xml:space="preserve">20/10 : accusé de réception automatique (ticket #880132), transmis au service concerné. Relance prévue le 26/10/2026.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CMA Grand Est (Metz)</t>
   </si>
   <si>
@@ -595,6 +604,9 @@
     <t xml:space="preserve">Officiel (cma-alsace-moselle-grandest.fr)</t>
   </si>
   <si>
+    <t xml:space="preserve">20/10 : rebond, domaine cma-grand-est.com introuvable. Pas de relance.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CMA Bouches-du-Rhône</t>
   </si>
   <si>
@@ -1130,9 +1142,6 @@
   </si>
   <si>
     <t xml:space="preserve">Liens obtenus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Refus</t>
   </si>
   <si>
     <t xml:space="preserve">Adresses invalides (rebonds)</t>
@@ -3458,7 +3467,7 @@
         <v>94</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>22</v>
+        <v>173</v>
       </c>
       <c r="J42" s="5" t="n">
         <v>46315</v>
@@ -3468,10 +3477,12 @@
         <v>46321</v>
       </c>
       <c r="L42" s="5"/>
-      <c r="M42" s="4"/>
+      <c r="M42" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="N42" s="4"/>
       <c r="O42" s="4" t="s">
-        <v>23</v>
+        <v>174</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3482,13 +3493,13 @@
         <v>90</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>167</v>
@@ -3513,7 +3524,7 @@
       <c r="M43" s="4"/>
       <c r="N43" s="4"/>
       <c r="O43" s="4" t="s">
-        <v>23</v>
+        <v>177</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3524,16 +3535,16 @@
         <v>90</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>93</v>
@@ -3542,7 +3553,7 @@
         <v>94</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>22</v>
+        <v>132</v>
       </c>
       <c r="J44" s="5" t="n">
         <v>46315</v>
@@ -3555,7 +3566,7 @@
       <c r="M44" s="4"/>
       <c r="N44" s="4"/>
       <c r="O44" s="4" t="s">
-        <v>23</v>
+        <v>181</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3566,13 +3577,13 @@
         <v>90</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>167</v>
@@ -3608,13 +3619,13 @@
         <v>90</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>167</v>
@@ -3637,7 +3648,7 @@
       <c r="M46" s="4"/>
       <c r="N46" s="4"/>
       <c r="O46" s="4" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3648,13 +3659,13 @@
         <v>90</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>151</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>167</v>
@@ -3666,18 +3677,20 @@
         <v>94</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J47" s="5"/>
-      <c r="K47" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J47" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K47" s="6" t="n">
         <f aca="false">IF(J47="","",WORKDAY(J47+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L47" s="5"/>
       <c r="M47" s="4"/>
       <c r="N47" s="4"/>
       <c r="O47" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3688,16 +3701,16 @@
         <v>90</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>93</v>
@@ -3706,18 +3719,20 @@
         <v>94</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J48" s="5"/>
-      <c r="K48" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J48" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K48" s="6" t="n">
         <f aca="false">IF(J48="","",WORKDAY(J48+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L48" s="5"/>
       <c r="M48" s="4"/>
       <c r="N48" s="4"/>
       <c r="O48" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3725,25 +3740,25 @@
         <v>48</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>67</v>
@@ -3765,39 +3780,41 @@
         <v>49</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J50" s="5"/>
-      <c r="K50" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J50" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K50" s="6" t="n">
         <f aca="false">IF(J50="","",WORKDAY(J50+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L50" s="5"/>
       <c r="M50" s="4"/>
       <c r="N50" s="4"/>
       <c r="O50" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3805,25 +3822,25 @@
         <v>50</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>67</v>
@@ -3845,25 +3862,25 @@
         <v>51</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>67</v>
@@ -3885,25 +3902,25 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>67</v>
@@ -3925,25 +3942,25 @@
         <v>53</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="G54" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I54" s="4" t="s">
         <v>67</v>
@@ -3965,25 +3982,25 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I55" s="4" t="s">
         <v>67</v>
@@ -4005,39 +4022,41 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J56" s="5"/>
-      <c r="K56" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J56" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K56" s="6" t="n">
         <f aca="false">IF(J56="","",WORKDAY(J56+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L56" s="5"/>
       <c r="M56" s="4"/>
       <c r="N56" s="4"/>
       <c r="O56" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4045,39 +4064,41 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J57" s="5"/>
-      <c r="K57" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J57" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K57" s="6" t="n">
         <f aca="false">IF(J57="","",WORKDAY(J57+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L57" s="5"/>
       <c r="M57" s="4"/>
       <c r="N57" s="4"/>
       <c r="O57" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4085,25 +4106,25 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I58" s="4" t="s">
         <v>67</v>
@@ -4117,7 +4138,7 @@
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
       <c r="O58" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4125,39 +4146,41 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J59" s="5"/>
-      <c r="K59" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J59" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K59" s="6" t="n">
         <f aca="false">IF(J59="","",WORKDAY(J59+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L59" s="5"/>
       <c r="M59" s="4"/>
       <c r="N59" s="4"/>
       <c r="O59" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4165,39 +4188,41 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J60" s="5"/>
-      <c r="K60" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J60" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K60" s="6" t="n">
         <f aca="false">IF(J60="","",WORKDAY(J60+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L60" s="5"/>
       <c r="M60" s="4"/>
       <c r="N60" s="4"/>
       <c r="O60" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4205,39 +4230,41 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J61" s="5"/>
-      <c r="K61" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J61" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K61" s="6" t="n">
         <f aca="false">IF(J61="","",WORKDAY(J61+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L61" s="5"/>
       <c r="M61" s="4"/>
       <c r="N61" s="4"/>
       <c r="O61" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4245,39 +4272,41 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E62" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F62" s="3" t="s">
         <v>228</v>
-      </c>
-      <c r="F62" s="3" t="s">
-        <v>224</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J62" s="5"/>
-      <c r="K62" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J62" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K62" s="6" t="n">
         <f aca="false">IF(J62="","",WORKDAY(J62+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L62" s="5"/>
       <c r="M62" s="4"/>
       <c r="N62" s="4"/>
       <c r="O62" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4285,39 +4314,41 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J63" s="5"/>
-      <c r="K63" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J63" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K63" s="6" t="n">
         <f aca="false">IF(J63="","",WORKDAY(J63+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L63" s="5"/>
       <c r="M63" s="4"/>
       <c r="N63" s="4"/>
       <c r="O63" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4325,39 +4356,41 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J64" s="5"/>
-      <c r="K64" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J64" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K64" s="6" t="n">
         <f aca="false">IF(J64="","",WORKDAY(J64+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L64" s="5"/>
       <c r="M64" s="4"/>
       <c r="N64" s="4"/>
       <c r="O64" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4365,39 +4398,41 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="G65" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J65" s="5"/>
-      <c r="K65" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J65" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K65" s="6" t="n">
         <f aca="false">IF(J65="","",WORKDAY(J65+4,1))</f>
-        <v/>
+        <v>46321</v>
       </c>
       <c r="L65" s="5"/>
       <c r="M65" s="4"/>
       <c r="N65" s="4"/>
       <c r="O65" s="4" t="s">
-        <v>182</v>
+        <v>23</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4405,25 +4440,25 @@
         <v>65</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="G66" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>67</v>
@@ -4437,7 +4472,7 @@
       <c r="M66" s="4"/>
       <c r="N66" s="4"/>
       <c r="O66" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4445,25 +4480,25 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="I67" s="4" t="s">
         <v>67</v>
@@ -4477,7 +4512,7 @@
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4485,25 +4520,25 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="F68" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="G68" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="F68" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="G68" s="3" t="s">
-        <v>242</v>
-      </c>
       <c r="H68" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>67</v>
@@ -4517,7 +4552,7 @@
       <c r="M68" s="4"/>
       <c r="N68" s="4"/>
       <c r="O68" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4525,25 +4560,25 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="I69" s="4" t="s">
         <v>67</v>
@@ -4557,7 +4592,7 @@
       <c r="M69" s="4"/>
       <c r="N69" s="4"/>
       <c r="O69" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4565,25 +4600,25 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>67</v>
@@ -4597,7 +4632,7 @@
       <c r="M70" s="4"/>
       <c r="N70" s="4"/>
       <c r="O70" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4605,25 +4640,25 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="I71" s="4" t="s">
         <v>67</v>
@@ -4637,7 +4672,7 @@
       <c r="M71" s="4"/>
       <c r="N71" s="4"/>
       <c r="O71" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4645,25 +4680,25 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="I72" s="4" t="s">
         <v>67</v>
@@ -4677,7 +4712,7 @@
       <c r="M72" s="4"/>
       <c r="N72" s="4"/>
       <c r="O72" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4685,25 +4720,25 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="I73" s="4" t="s">
         <v>67</v>
@@ -4717,7 +4752,7 @@
       <c r="M73" s="4"/>
       <c r="N73" s="4"/>
       <c r="O73" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4725,25 +4760,25 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="I74" s="4" t="s">
         <v>67</v>
@@ -4757,7 +4792,7 @@
       <c r="M74" s="4"/>
       <c r="N74" s="4"/>
       <c r="O74" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4765,25 +4800,25 @@
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>100</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="I75" s="4" t="s">
         <v>67</v>
@@ -4797,7 +4832,7 @@
       <c r="M75" s="4"/>
       <c r="N75" s="4"/>
       <c r="O75" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4805,25 +4840,25 @@
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>151</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>67</v>
@@ -4837,7 +4872,7 @@
       <c r="M76" s="4"/>
       <c r="N76" s="4"/>
       <c r="O76" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4845,25 +4880,25 @@
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>67</v>
@@ -4877,7 +4912,7 @@
       <c r="M77" s="4"/>
       <c r="N77" s="4"/>
       <c r="O77" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4888,19 +4923,19 @@
         <v>15</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>21</v>
@@ -4917,7 +4952,7 @@
       <c r="M78" s="4"/>
       <c r="N78" s="4"/>
       <c r="O78" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4928,22 +4963,22 @@
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>67</v>
@@ -4957,7 +4992,7 @@
       <c r="M79" s="4"/>
       <c r="N79" s="4"/>
       <c r="O79" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4968,22 +5003,22 @@
         <v>15</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>38</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="I80" s="4" t="s">
         <v>67</v>
@@ -4997,7 +5032,7 @@
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
       <c r="O80" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5008,22 +5043,22 @@
         <v>15</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="I81" s="4" t="s">
         <v>67</v>
@@ -5037,7 +5072,7 @@
       <c r="M81" s="4"/>
       <c r="N81" s="4"/>
       <c r="O81" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5048,22 +5083,22 @@
         <v>52</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="G82" s="3" t="s">
         <v>65</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="I82" s="4" t="s">
         <v>67</v>
@@ -5077,7 +5112,7 @@
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
       <c r="O82" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5088,22 +5123,22 @@
         <v>52</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>67</v>
@@ -5117,7 +5152,7 @@
       <c r="M83" s="4"/>
       <c r="N83" s="4"/>
       <c r="O83" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5128,22 +5163,22 @@
         <v>52</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="I84" s="4" t="s">
         <v>67</v>
@@ -5157,7 +5192,7 @@
       <c r="M84" s="4"/>
       <c r="N84" s="4"/>
       <c r="O84" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5165,25 +5200,25 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="G85" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>67</v>
@@ -5197,7 +5232,7 @@
       <c r="M85" s="4"/>
       <c r="N85" s="4"/>
       <c r="O85" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5205,25 +5240,25 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>100</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="G86" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>67</v>
@@ -5237,7 +5272,7 @@
       <c r="M86" s="4"/>
       <c r="N86" s="4"/>
       <c r="O86" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5245,25 +5280,25 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="I87" s="4" t="s">
         <v>67</v>
@@ -5288,22 +5323,22 @@
         <v>44</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>167</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="I88" s="4" t="s">
         <v>67</v>
@@ -5328,22 +5363,22 @@
         <v>44</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="F89" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="G89" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="G89" s="3" t="s">
-        <v>322</v>
-      </c>
       <c r="H89" s="3" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="I89" s="4" t="s">
         <v>67</v>
@@ -5368,22 +5403,22 @@
         <v>126</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="G90" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I90" s="4" t="s">
         <v>67</v>
@@ -5397,7 +5432,7 @@
       <c r="M90" s="4"/>
       <c r="N90" s="4"/>
       <c r="O90" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5408,22 +5443,22 @@
         <v>126</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="G91" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I91" s="4" t="s">
         <v>67</v>
@@ -5437,7 +5472,7 @@
       <c r="M91" s="4"/>
       <c r="N91" s="4"/>
       <c r="O91" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5448,22 +5483,22 @@
         <v>126</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I92" s="4" t="s">
         <v>67</v>
@@ -5477,7 +5512,7 @@
       <c r="M92" s="4"/>
       <c r="N92" s="4"/>
       <c r="O92" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5488,22 +5523,22 @@
         <v>126</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="G93" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I93" s="4" t="s">
         <v>67</v>
@@ -5517,7 +5552,7 @@
       <c r="M93" s="4"/>
       <c r="N93" s="4"/>
       <c r="O93" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5528,22 +5563,22 @@
         <v>126</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I94" s="4" t="s">
         <v>67</v>
@@ -5557,7 +5592,7 @@
       <c r="M94" s="4"/>
       <c r="N94" s="4"/>
       <c r="O94" s="4" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5568,22 +5603,22 @@
         <v>126</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H95" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I95" s="4" t="s">
         <v>67</v>
@@ -5597,7 +5632,7 @@
       <c r="M95" s="4"/>
       <c r="N95" s="4"/>
       <c r="O95" s="4" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5608,22 +5643,22 @@
         <v>126</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="G96" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I96" s="4" t="s">
         <v>67</v>
@@ -5637,7 +5672,7 @@
       <c r="M96" s="4"/>
       <c r="N96" s="4"/>
       <c r="O96" s="4" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5648,22 +5683,22 @@
         <v>126</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E97" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="F97" s="3" t="s">
         <v>349</v>
-      </c>
-      <c r="F97" s="3" t="s">
-        <v>345</v>
       </c>
       <c r="G97" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="I97" s="4" t="s">
         <v>67</v>
@@ -5677,7 +5712,7 @@
       <c r="M97" s="4"/>
       <c r="N97" s="4"/>
       <c r="O97" s="4" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7792,12 +7827,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -7806,25 +7841,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>69</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>26</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -7833,16 +7868,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -7851,34 +7886,34 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>357</v>
+        <v>173</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Refus")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.0384615384615385</v>
+        <v>0.0540540540540541</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -7887,7 +7922,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -7896,12 +7931,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7909,13 +7944,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7996,7 +8031,7 @@
       </c>
       <c r="C23" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A23,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D23" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A23,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8022,7 +8057,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A25)</f>
@@ -8030,7 +8065,7 @@
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8039,7 +8074,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
@@ -8047,7 +8082,7 @@
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A26,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D26" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A26,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8056,7 +8091,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A27)</f>
@@ -8073,7 +8108,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A28)</f>
@@ -8090,7 +8125,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -8098,7 +8133,7 @@
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">SUM(D19:D28)</f>
@@ -8129,7 +8164,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8137,12 +8172,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8150,27 +8185,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8178,27 +8213,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection 22/10 : 13 envois, 2 rebonds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="386">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -619,7 +619,7 @@
     <t xml:space="preserve">contact72@cma-paysdelaloire.fr</t>
   </si>
   <si>
-    <t xml:space="preserve">Envoi conseillé : jour 3</t>
+    <t xml:space="preserve">Relance prévue le 27/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">CMA Hérault</t>
@@ -661,6 +661,9 @@
     <t xml:space="preserve">Officiel (plaquette)</t>
   </si>
   <si>
+    <t xml:space="preserve">21/10 : rebond, domaine initiative-orne.com introuvable. Pas de relance.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Initiative Genevois</t>
   </si>
   <si>
@@ -739,6 +742,9 @@
     <t xml:space="preserve">Des ressources gratuites pour les dirigeants que vous accompagnez</t>
   </si>
   <si>
+    <t xml:space="preserve">21/10 : rebond, message bloqué par le serveur de Réseau Entreprendre. Pas de relance.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réseau Entreprendre Lorraine</t>
   </si>
   <si>
@@ -805,217 +811,217 @@
     <t xml:space="preserve">Un calculateur de TJM gratuit pour les entrepreneurs à l’essai</t>
   </si>
   <si>
+    <t xml:space="preserve">Coopérer pour entreprendre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">info@cooperer.coop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (annuaire Avise)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un calculateur de TJM gratuit pour les entrepreneurs-salariés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coopérer pour entreprendre Bretagne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bretagne@cooperer.coop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (ess-bretagne.org)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fédération des CAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">les-cae@scop.coop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (ambition-ess.org)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URSCOP Nouvelle-Aquitaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">urnouvelleaquitaine@scop.coop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (les-scop-nouvelle-aquitaine.coop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-list + TJM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les CAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cabestan (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@cabestan.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (plaquette)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CoopConnexion (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@coopconnexion.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (coopconnexion.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coopetic (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@coopetic.coop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (coopetic.coop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coopilote (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">administratif@coopilote.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (coopilote.com), adresse administrative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour vos entrepreneurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Comptoir des Entrepreneurs (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@lecomptoirdesentrepreneurs.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (fiche les-scop.coop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coopenates (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@coopenates.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (fiche les-cae.coop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Widoobiz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">redaction@widoobiz.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (page d’environ 6 ans)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baromètre des prix + TJM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Journal des Entreprises</t>
+  </si>
+  <si>
+    <t xml:space="preserve">redacweb@lejournaldesentreprises.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (leadiq.com), non confirmée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-list + baromètre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les TPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espace Auto-Entrepreneur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@espace-autoentrepreneur.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (page presse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Des simulateurs gratuits pour vos lecteurs auto-entrepreneurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Courrier des Entreprises</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@lecourrierdesentreprises.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (site)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SDI (Syndicat des indépendants et TPE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@sdi-pme.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour vos adhérents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNION-Indépendants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@union-independants.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (arpe.gouv.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un calculateur de TJM gratuit pour les indépendants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEPS (portage salarial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">presse@peps-syndicat.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (peps-syndicat.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculateur TJM + baromètre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un calculateur de TJM gratuit pour les consultants indépendants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Association</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60 000 rebonds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@60000rebonds.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (variante en .fr ailleurs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Des simulateurs gratuits pour les entrepreneurs qui rebondissent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60 000 rebonds Bourgogne-Franche-Comté</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bfc@60000rebonds.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (page régionale)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Envoi conseillé : jour 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coopérer pour entreprendre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">info@cooperer.coop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (annuaire Avise)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un calculateur de TJM gratuit pour les entrepreneurs-salariés</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coopérer pour entreprendre Bretagne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bretagne@cooperer.coop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (ess-bretagne.org)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fédération des CAE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">les-cae@scop.coop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (ambition-ess.org)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">URSCOP Nouvelle-Aquitaine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">urnouvelleaquitaine@scop.coop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (les-scop-nouvelle-aquitaine.coop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-list + TJM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les CAE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cabestan (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@cabestan.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (plaquette)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CoopConnexion (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@coopconnexion.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (coopconnexion.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coopetic (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@coopetic.coop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (coopetic.coop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coopilote (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">administratif@coopilote.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (coopilote.com), adresse administrative</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour vos entrepreneurs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Comptoir des Entrepreneurs (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@lecomptoirdesentrepreneurs.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (fiche les-scop.coop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coopenates (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@coopenates.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (fiche les-cae.coop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Widoobiz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">redaction@widoobiz.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (page d’environ 6 ans)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baromètre des prix + TJM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Journal des Entreprises</t>
-  </si>
-  <si>
-    <t xml:space="preserve">redacweb@lejournaldesentreprises.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (leadiq.com), non confirmée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-list + baromètre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les TPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Espace Auto-Entrepreneur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@espace-autoentrepreneur.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (page presse)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Des simulateurs gratuits pour vos lecteurs auto-entrepreneurs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Courrier des Entreprises</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@lecourrierdesentreprises.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (site)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SDI (Syndicat des indépendants et TPE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@sdi-pme.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour vos adhérents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNION-Indépendants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@union-independants.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (arpe.gouv.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un calculateur de TJM gratuit pour les indépendants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PEPS (portage salarial)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">presse@peps-syndicat.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (peps-syndicat.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculateur TJM + baromètre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un calculateur de TJM gratuit pour les consultants indépendants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Association</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60 000 rebonds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@60000rebonds.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (variante en .fr ailleurs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Des simulateurs gratuits pour les entrepreneurs qui rebondissent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60 000 rebonds Bourgogne-Franche-Comté</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bfc@60000rebonds.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (page régionale)</t>
   </si>
   <si>
     <t xml:space="preserve">Moovjee (mentorat)</t>
@@ -3637,12 +3643,14 @@
         <v>94</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J46" s="5"/>
-      <c r="K46" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J46" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K46" s="6" t="n">
         <f aca="false">IF(J46="","",WORKDAY(J46+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L46" s="5"/>
       <c r="M46" s="4"/>
@@ -3801,7 +3809,7 @@
         <v>196</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>22</v>
+        <v>132</v>
       </c>
       <c r="J50" s="5" t="n">
         <v>46316</v>
@@ -3814,7 +3822,7 @@
       <c r="M50" s="4"/>
       <c r="N50" s="4"/>
       <c r="O50" s="4" t="s">
-        <v>23</v>
+        <v>200</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3825,13 +3833,13 @@
         <v>192</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>195</v>
@@ -3865,13 +3873,13 @@
         <v>192</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>195</v>
@@ -3905,13 +3913,13 @@
         <v>192</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>195</v>
@@ -3945,13 +3953,13 @@
         <v>192</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>195</v>
@@ -3985,16 +3993,16 @@
         <v>192</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>130</v>
@@ -4025,16 +4033,16 @@
         <v>192</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>130</v>
@@ -4067,16 +4075,16 @@
         <v>192</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>130</v>
@@ -4109,16 +4117,16 @@
         <v>192</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>130</v>
@@ -4138,7 +4146,7 @@
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
       <c r="O58" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4146,28 +4154,28 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I59" s="4" t="s">
-        <v>22</v>
+        <v>132</v>
       </c>
       <c r="J59" s="5" t="n">
         <v>46316</v>
@@ -4180,7 +4188,7 @@
       <c r="M59" s="4"/>
       <c r="N59" s="4"/>
       <c r="O59" s="4" t="s">
-        <v>23</v>
+        <v>227</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4188,25 +4196,25 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I60" s="4" t="s">
         <v>22</v>
@@ -4230,25 +4238,25 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E61" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F61" s="3" t="s">
         <v>230</v>
-      </c>
-      <c r="F61" s="3" t="s">
-        <v>228</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I61" s="4" t="s">
         <v>22</v>
@@ -4272,25 +4280,25 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I62" s="4" t="s">
         <v>22</v>
@@ -4314,25 +4322,25 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I63" s="4" t="s">
         <v>22</v>
@@ -4356,25 +4364,25 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>124</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I64" s="4" t="s">
         <v>22</v>
@@ -4398,25 +4406,25 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G65" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I65" s="4" t="s">
         <v>22</v>
@@ -4440,25 +4448,25 @@
         <v>65</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G66" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>67</v>
@@ -4472,7 +4480,7 @@
       <c r="M66" s="4"/>
       <c r="N66" s="4"/>
       <c r="O66" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4480,39 +4488,41 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J67" s="5"/>
-      <c r="K67" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J67" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K67" s="6" t="n">
         <f aca="false">IF(J67="","",WORKDAY(J67+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L67" s="5"/>
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4520,25 +4530,25 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>67</v>
@@ -4552,7 +4562,7 @@
       <c r="M68" s="4"/>
       <c r="N68" s="4"/>
       <c r="O68" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4560,25 +4570,25 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I69" s="4" t="s">
         <v>67</v>
@@ -4592,7 +4602,7 @@
       <c r="M69" s="4"/>
       <c r="N69" s="4"/>
       <c r="O69" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4600,25 +4610,25 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>67</v>
@@ -4632,7 +4642,7 @@
       <c r="M70" s="4"/>
       <c r="N70" s="4"/>
       <c r="O70" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4640,39 +4650,41 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J71" s="5"/>
-      <c r="K71" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J71" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K71" s="6" t="n">
         <f aca="false">IF(J71="","",WORKDAY(J71+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L71" s="5"/>
       <c r="M71" s="4"/>
       <c r="N71" s="4"/>
       <c r="O71" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4680,25 +4692,25 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I72" s="4" t="s">
         <v>67</v>
@@ -4712,7 +4724,7 @@
       <c r="M72" s="4"/>
       <c r="N72" s="4"/>
       <c r="O72" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4720,39 +4732,41 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J73" s="5"/>
-      <c r="K73" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J73" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K73" s="6" t="n">
         <f aca="false">IF(J73="","",WORKDAY(J73+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L73" s="5"/>
       <c r="M73" s="4"/>
       <c r="N73" s="4"/>
       <c r="O73" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4760,39 +4774,41 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J74" s="5"/>
-      <c r="K74" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J74" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K74" s="6" t="n">
         <f aca="false">IF(J74="","",WORKDAY(J74+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L74" s="5"/>
       <c r="M74" s="4"/>
       <c r="N74" s="4"/>
       <c r="O74" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4800,39 +4816,41 @@
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>100</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I75" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J75" s="5"/>
-      <c r="K75" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J75" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K75" s="6" t="n">
         <f aca="false">IF(J75="","",WORKDAY(J75+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L75" s="5"/>
       <c r="M75" s="4"/>
       <c r="N75" s="4"/>
       <c r="O75" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4840,25 +4858,25 @@
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>151</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>67</v>
@@ -4872,7 +4890,7 @@
       <c r="M76" s="4"/>
       <c r="N76" s="4"/>
       <c r="O76" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4880,25 +4898,25 @@
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>67</v>
@@ -4912,7 +4930,7 @@
       <c r="M77" s="4"/>
       <c r="N77" s="4"/>
       <c r="O77" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4923,36 +4941,38 @@
         <v>15</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>21</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J78" s="5"/>
-      <c r="K78" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J78" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K78" s="6" t="n">
         <f aca="false">IF(J78="","",WORKDAY(J78+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L78" s="5"/>
       <c r="M78" s="4"/>
       <c r="N78" s="4"/>
       <c r="O78" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4963,22 +4983,22 @@
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>67</v>
@@ -4992,7 +5012,7 @@
       <c r="M79" s="4"/>
       <c r="N79" s="4"/>
       <c r="O79" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5003,36 +5023,38 @@
         <v>15</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>38</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J80" s="5"/>
-      <c r="K80" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J80" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K80" s="6" t="n">
         <f aca="false">IF(J80="","",WORKDAY(J80+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L80" s="5"/>
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
       <c r="O80" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5043,36 +5065,38 @@
         <v>15</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J81" s="5"/>
-      <c r="K81" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J81" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K81" s="6" t="n">
         <f aca="false">IF(J81="","",WORKDAY(J81+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L81" s="5"/>
       <c r="M81" s="4"/>
       <c r="N81" s="4"/>
       <c r="O81" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5083,36 +5107,38 @@
         <v>52</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G82" s="3" t="s">
         <v>65</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J82" s="5"/>
-      <c r="K82" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J82" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K82" s="6" t="n">
         <f aca="false">IF(J82="","",WORKDAY(J82+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L82" s="5"/>
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
       <c r="O82" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5123,36 +5149,38 @@
         <v>52</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J83" s="5"/>
-      <c r="K83" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J83" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K83" s="6" t="n">
         <f aca="false">IF(J83="","",WORKDAY(J83+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L83" s="5"/>
       <c r="M83" s="4"/>
       <c r="N83" s="4"/>
       <c r="O83" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5163,36 +5191,38 @@
         <v>52</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J84" s="5"/>
-      <c r="K84" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J84" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K84" s="6" t="n">
         <f aca="false">IF(J84="","",WORKDAY(J84+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L84" s="5"/>
       <c r="M84" s="4"/>
       <c r="N84" s="4"/>
       <c r="O84" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5200,39 +5230,41 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="G85" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="I85" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J85" s="5"/>
-      <c r="K85" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J85" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="K85" s="6" t="n">
         <f aca="false">IF(J85="","",WORKDAY(J85+4,1))</f>
-        <v/>
+        <v>46322</v>
       </c>
       <c r="L85" s="5"/>
       <c r="M85" s="4"/>
       <c r="N85" s="4"/>
       <c r="O85" s="4" t="s">
-        <v>248</v>
+        <v>186</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5240,25 +5272,25 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>100</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G86" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>67</v>
@@ -5272,7 +5304,7 @@
       <c r="M86" s="4"/>
       <c r="N86" s="4"/>
       <c r="O86" s="4" t="s">
-        <v>248</v>
+        <v>320</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5280,25 +5312,25 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="I87" s="4" t="s">
         <v>67</v>
@@ -5323,22 +5355,22 @@
         <v>44</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>167</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="I88" s="4" t="s">
         <v>67</v>
@@ -5363,22 +5395,22 @@
         <v>44</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="G89" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="H89" s="3" t="s">
         <v>329</v>
-      </c>
-      <c r="F89" s="3" t="s">
-        <v>330</v>
-      </c>
-      <c r="G89" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="H89" s="3" t="s">
-        <v>327</v>
       </c>
       <c r="I89" s="4" t="s">
         <v>67</v>
@@ -5403,16 +5435,16 @@
         <v>126</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="G90" s="3" t="s">
         <v>130</v>
@@ -5432,7 +5464,7 @@
       <c r="M90" s="4"/>
       <c r="N90" s="4"/>
       <c r="O90" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5443,16 +5475,16 @@
         <v>126</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="G91" s="3" t="s">
         <v>130</v>
@@ -5472,7 +5504,7 @@
       <c r="M91" s="4"/>
       <c r="N91" s="4"/>
       <c r="O91" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5483,16 +5515,16 @@
         <v>126</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>130</v>
@@ -5512,7 +5544,7 @@
       <c r="M92" s="4"/>
       <c r="N92" s="4"/>
       <c r="O92" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5523,16 +5555,16 @@
         <v>126</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="G93" s="3" t="s">
         <v>130</v>
@@ -5552,7 +5584,7 @@
       <c r="M93" s="4"/>
       <c r="N93" s="4"/>
       <c r="O93" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5563,16 +5595,16 @@
         <v>126</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>130</v>
@@ -5592,7 +5624,7 @@
       <c r="M94" s="4"/>
       <c r="N94" s="4"/>
       <c r="O94" s="4" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5603,16 +5635,16 @@
         <v>126</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>130</v>
@@ -5632,7 +5664,7 @@
       <c r="M95" s="4"/>
       <c r="N95" s="4"/>
       <c r="O95" s="4" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5643,16 +5675,16 @@
         <v>126</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E96" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="F96" s="3" t="s">
         <v>351</v>
-      </c>
-      <c r="F96" s="3" t="s">
-        <v>349</v>
       </c>
       <c r="G96" s="3" t="s">
         <v>130</v>
@@ -5672,7 +5704,7 @@
       <c r="M96" s="4"/>
       <c r="N96" s="4"/>
       <c r="O96" s="4" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5683,16 +5715,16 @@
         <v>126</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>70</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="G97" s="3" t="s">
         <v>130</v>
@@ -5712,7 +5744,7 @@
       <c r="M97" s="4"/>
       <c r="N97" s="4"/>
       <c r="O97" s="4" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7827,12 +7859,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -7841,25 +7873,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>57</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>37</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -7868,7 +7900,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -7877,7 +7909,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -7895,25 +7927,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.0540540540540541</v>
+        <v>0.0416666666666667</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -7922,7 +7954,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -7931,12 +7963,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7944,13 +7976,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7963,7 +7995,7 @@
       </c>
       <c r="C19" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A19,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D19" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A19,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -7997,7 +8029,7 @@
       </c>
       <c r="C21" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A21,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D21" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A21,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8031,7 +8063,7 @@
       </c>
       <c r="C23" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A23,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A23,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8074,7 +8106,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
@@ -8091,7 +8123,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A27)</f>
@@ -8099,7 +8131,7 @@
       </c>
       <c r="C27" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A27,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D27" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A27,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8108,7 +8140,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A28)</f>
@@ -8116,7 +8148,7 @@
       </c>
       <c r="C28" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A28,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A28,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8125,7 +8157,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -8133,7 +8165,7 @@
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">SUM(D19:D28)</f>
@@ -8164,7 +8196,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8172,12 +8204,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8185,27 +8217,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8213,27 +8245,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection 23/10 : 13 envois, 1 rebond
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="389">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -262,802 +262,811 @@
     <t xml:space="preserve">Un outil gratuit pour vos porteurs de projet (facture électronique 2027)</t>
   </si>
   <si>
+    <t xml:space="preserve">Relance prévue le 28/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Bretagne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bretagne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ccir@bretagne.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel ancien (douane.gouv.fr), à vérifier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Hauts-de-France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hauts-de-France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ccideregion@hautsdefrance.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (document CCI repris)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Ouest Normandie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normandie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cci@normandie.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (annuaire-administration.com)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Portes de Normandie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">info-eure@normandie.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Nouvelle-Aquitaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nouvelle-Aquitaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@nouvelle-aquitaine.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Nantes St-Nazaire (création-reprise)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pays de la Loire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">conseil-creation-reprise@44.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers, source non relevée : à vérifier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Val-d'Oise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eco@cma95.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-list artisans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les artisans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Auvergne-Rhône-Alpes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auvergne-Rhône-Alpes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@crma-auvergnerhonealpes.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers, 2018 : peut être obsolète</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Côte-d'Or</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bourgogne-Franche-Comté</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accueil-s21@artisanat-bfc.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Morbihan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accueil@cma-morbihan.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Loiret</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centre-Val de Loire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@cma45.fr</t>
+  </si>
+  <si>
     <t xml:space="preserve">Brouillon prêt</t>
   </si>
   <si>
+    <t xml:space="preserve">Envoi conseillé : jour 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Alsace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grand Est</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cma@cm-alsace.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (strasbourg-europe.eu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Hauts-de-France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@cma-hautsdefrance.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Charente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16-eco@cma-nouvelleaquitaine.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (document de commune)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Vienne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86-cma-info@cma-nouvelleaquitaine.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (lavienne86.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Loire-Atlantique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">entreprises44@cma-paysdelaloire.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel, à revérifier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Alpes-Maritimes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PACA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact06@cmar-paca.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BGE Réseau (national)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accueil@bge.asso.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (bge.asso.fr, 2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulateurs + check-list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Des outils gratuits pour les entrepreneurs que vous accompagnez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adresse invalide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réponse auto 19/10 : boîte plus relevée. Pas de relance. Viser les BGE régionales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Réunion (conseil entreprise)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La Réunion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">conseilentreprise@reunion.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (page d’environ 5 ans)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Loiret</t>
+  </si>
+  <si>
+    <t xml:space="preserve">entreprendre@loiret.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (centre.cci.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Cher, Espace Entreprendre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">espace-entreprendre@cher.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Indre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">entreprendre@indre.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Loir-et-Cher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">entreprendre@41.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Vendée, Espace Création</t>
+  </si>
+  <si>
+    <t xml:space="preserve">espace.creation@vendee.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (paysdelaloire.cci.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Tarn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Occitanie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">monprojetaveclacci@tarn.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (tarn.cci.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Alpes-de-Haute-Provence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">creation@digne.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (digne.cci.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Métropole de Bourgogne, Espace Entreprendre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">espace.entreprendre@mdb.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (metropoledebourgogne.cci.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Lyon Métropole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">infos@lyon-metropole.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (contact général)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI PACA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">information@paca.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Pyrénées-Orientales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@cma66.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (annuaire service-public.gouv.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Val-de-Marne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@cma94.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Île-de-France, Paris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@cma-paris.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (cma-idf.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20/10 : réponse STOP de contact.75@cma-idf.fr. Plus aucun mail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Rhône</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@cma-auvergnerhonealpes.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20/10 : accusé de réception automatique (ticket #880132), transmis au service concerné. Relance prévue le 26/10/2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Grand Est (Metz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@cma-grand-est.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (cma-alsace-moselle-grandest.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20/10 : rebond, domaine cma-grand-est.com introuvable. Pas de relance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Bouches-du-Rhône</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact13@cmar-paca.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Sarthe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact72@cma-paysdelaloire.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relance prévue le 27/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Hérault</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cma34@cma-herault.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Gironde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bonjour@cma-nouvelle-aquitaine.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel, mais domaine différent de cma-nouvelleaquitaine.fr : à surveiller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Sarthe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-sarthe.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (les-aides.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Des outils gratuits pour les créateurs que vous accompagnez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Orne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-orne.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (plaquette)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21/10 : rebond, domaine initiative-orne.com introuvable. Pas de relance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Genevois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-genevois.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Rouen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rouen-initiative@rouen.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Sud Grésivaudan Royans Vercors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-sgrv.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Alpes-de-Haute-Provence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-alpesdehauteprovence.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Calvados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-calvados.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (le site n’affiche qu’un formulaire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Var</t>
+  </si>
+  <si>
+    <t xml:space="preserve">info@initiative-var.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (initiative-var.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Terres de Vaucluse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiativeterresdevaucluse.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (site de la plateforme)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Vallée de la Drôme Diois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-valleedeladromediois.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (liste ancienne)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Envoi conseillé : jour 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre (fédération)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reseau@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (rapport financier 2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Des ressources gratuites pour les dirigeants que vous accompagnez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21/10 : rebond, message bloqué par le serveur de Réseau Entreprendre. Pas de relance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre Lorraine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lorraine@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (page contact)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre Val-de-Marne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valdemarne@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre Aquitaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aquitaine@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre Yvelines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yvelines@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre Rhône-Durance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rhone-durance@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre Loire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">loire@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre Atlantique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">atlantique@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (document de 2019)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Couveuse / CAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Union des couveuses d’entreprises</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@uniondescouveuses.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (jetestemonentreprise.com)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculateur TJM + check-list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un calculateur de TJM gratuit pour les entrepreneurs à l’essai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22/10 : filtre anti-spam Mailinblack, message en attente tant que l'expéditeur n'a pas validé le lien reçu. Relance prévue le 27/10/2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coopérer pour entreprendre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">info@cooperer.coop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (annuaire Avise)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un calculateur de TJM gratuit pour les entrepreneurs-salariés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coopérer pour entreprendre Bretagne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bretagne@cooperer.coop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (ess-bretagne.org)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fédération des CAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">les-cae@scop.coop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (ambition-ess.org)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URSCOP Nouvelle-Aquitaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">urnouvelleaquitaine@scop.coop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (les-scop-nouvelle-aquitaine.coop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-list + TJM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les CAE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cabestan (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@cabestan.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (plaquette)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CoopConnexion (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@coopconnexion.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (coopconnexion.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coopetic (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@coopetic.coop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (coopetic.coop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coopilote (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">administratif@coopilote.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (coopilote.com), adresse administrative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour vos entrepreneurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Comptoir des Entrepreneurs (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@lecomptoirdesentrepreneurs.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (fiche les-scop.coop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coopenates (CAE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@coopenates.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (fiche les-cae.coop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Widoobiz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">redaction@widoobiz.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (page d’environ 6 ans)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baromètre des prix + TJM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22/10 : rebond, message bloqué par le serveur de Widoobiz. Pas de relance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Journal des Entreprises</t>
+  </si>
+  <si>
+    <t xml:space="preserve">redacweb@lejournaldesentreprises.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (leadiq.com), non confirmée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-list + baromètre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les TPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espace Auto-Entrepreneur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@espace-autoentrepreneur.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (page presse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Des simulateurs gratuits pour vos lecteurs auto-entrepreneurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22/10 : accusé de réception automatique (demande 487253). Relance prévue le 27/10/2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Courrier des Entreprises</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@lecourrierdesentreprises.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (site)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SDI (Syndicat des indépendants et TPE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@sdi-pme.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour vos adhérents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNION-Indépendants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@union-independants.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (arpe.gouv.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un calculateur de TJM gratuit pour les indépendants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEPS (portage salarial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">presse@peps-syndicat.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (peps-syndicat.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculateur TJM + baromètre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un calculateur de TJM gratuit pour les consultants indépendants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Association</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60 000 rebonds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@60000rebonds.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (variante en .fr ailleurs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Des simulateurs gratuits pour les entrepreneurs qui rebondissent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60 000 rebonds Bourgogne-Franche-Comté</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bfc@60000rebonds.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (page régionale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moovjee (mentorat)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">moovjee@twoo-mentorat.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (moovjee.fr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulateurs + TJM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Des outils gratuits pour les jeunes entrepreneurs que vous accompagnez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordre des experts-comptables Paris IDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@oec-paris.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-list facture électronique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les clients TPE des cabinets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECF (syndicat des experts-comptables)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@e-c-f.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (page Facebook)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Envoi conseillé : jour 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Bretagne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bretagne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ccir@bretagne.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel ancien (douane.gouv.fr), à vérifier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Hauts-de-France</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hauts-de-France</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ccideregion@hautsdefrance.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (document CCI repris)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Ouest Normandie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Normandie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cci@normandie.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (annuaire-administration.com)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Portes de Normandie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">info-eure@normandie.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Nouvelle-Aquitaine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nouvelle-Aquitaine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@nouvelle-aquitaine.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Nantes St-Nazaire (création-reprise)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pays de la Loire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">conseil-creation-reprise@44.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers, source non relevée : à vérifier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Val-d'Oise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eco@cma95.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-list artisans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les artisans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Auvergne-Rhône-Alpes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auvergne-Rhône-Alpes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@crma-auvergnerhonealpes.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers, 2018 : peut être obsolète</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Côte-d'Or</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bourgogne-Franche-Comté</t>
-  </si>
-  <si>
-    <t xml:space="preserve">accueil-s21@artisanat-bfc.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Morbihan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">accueil@cma-morbihan.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Loiret</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Centre-Val de Loire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@cma45.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Envoi conseillé : jour 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Alsace</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grand Est</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cma@cm-alsace.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (strasbourg-europe.eu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Hauts-de-France</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@cma-hautsdefrance.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Charente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16-eco@cma-nouvelleaquitaine.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (document de commune)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Vienne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86-cma-info@cma-nouvelleaquitaine.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (lavienne86.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Loire-Atlantique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">entreprises44@cma-paysdelaloire.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel, à revérifier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Alpes-Maritimes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PACA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact06@cmar-paca.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BGE Réseau (national)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">accueil@bge.asso.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (bge.asso.fr, 2024)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Simulateurs + check-list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Des outils gratuits pour les entrepreneurs que vous accompagnez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adresse invalide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réponse auto 19/10 : boîte plus relevée. Pas de relance. Viser les BGE régionales.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Réunion (conseil entreprise)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Réunion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">conseilentreprise@reunion.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (page d’environ 5 ans)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Loiret</t>
-  </si>
-  <si>
-    <t xml:space="preserve">entreprendre@loiret.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (centre.cci.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Cher, Espace Entreprendre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">espace-entreprendre@cher.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Indre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">entreprendre@indre.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Loir-et-Cher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">entreprendre@41.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Vendée, Espace Création</t>
-  </si>
-  <si>
-    <t xml:space="preserve">espace.creation@vendee.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (paysdelaloire.cci.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Tarn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Occitanie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">monprojetaveclacci@tarn.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (tarn.cci.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Alpes-de-Haute-Provence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">creation@digne.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (digne.cci.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Métropole de Bourgogne, Espace Entreprendre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">espace.entreprendre@mdb.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (metropoledebourgogne.cci.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI Lyon Métropole</t>
-  </si>
-  <si>
-    <t xml:space="preserve">infos@lyon-metropole.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (contact général)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCI PACA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">information@paca.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Pyrénées-Orientales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@cma66.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (annuaire service-public.gouv.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Val-de-Marne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@cma94.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Île-de-France, Paris</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@cma-paris.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (cma-idf.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Refus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20/10 : réponse STOP de contact.75@cma-idf.fr. Plus aucun mail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Rhône</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@cma-auvergnerhonealpes.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20/10 : accusé de réception automatique (ticket #880132), transmis au service concerné. Relance prévue le 26/10/2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Grand Est (Metz)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@cma-grand-est.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (cma-alsace-moselle-grandest.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20/10 : rebond, domaine cma-grand-est.com introuvable. Pas de relance.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Bouches-du-Rhône</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact13@cmar-paca.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Sarthe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact72@cma-paysdelaloire.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relance prévue le 27/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Hérault</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cma34@cma-herault.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Gironde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bonjour@cma-nouvelle-aquitaine.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel, mais domaine différent de cma-nouvelleaquitaine.fr : à surveiller</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Sarthe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-sarthe.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (les-aides.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Des outils gratuits pour les créateurs que vous accompagnez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Orne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-orne.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (plaquette)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21/10 : rebond, domaine initiative-orne.com introuvable. Pas de relance.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Genevois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-genevois.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Rouen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rouen-initiative@rouen.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Sud Grésivaudan Royans Vercors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-sgrv.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Alpes-de-Haute-Provence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-alpesdehauteprovence.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Calvados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-calvados.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (le site n’affiche qu’un formulaire)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Var</t>
-  </si>
-  <si>
-    <t xml:space="preserve">info@initiative-var.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (initiative-var.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Terres de Vaucluse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiativeterresdevaucluse.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (site de la plateforme)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Vallée de la Drôme Diois</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-valleedeladromediois.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (liste ancienne)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Envoi conseillé : jour 7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau Entreprendre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau Entreprendre (fédération)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reseau@reseau-entreprendre.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (rapport financier 2024)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Des ressources gratuites pour les dirigeants que vous accompagnez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21/10 : rebond, message bloqué par le serveur de Réseau Entreprendre. Pas de relance.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau Entreprendre Lorraine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lorraine@reseau-entreprendre.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (page contact)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau Entreprendre Val-de-Marne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valdemarne@reseau-entreprendre.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau Entreprendre Aquitaine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aquitaine@reseau-entreprendre.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau Entreprendre Yvelines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yvelines@reseau-entreprendre.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau Entreprendre Rhône-Durance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rhone-durance@reseau-entreprendre.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau Entreprendre Loire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">loire@reseau-entreprendre.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau Entreprendre Atlantique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">atlantique@reseau-entreprendre.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (document de 2019)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Couveuse / CAE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Union des couveuses d’entreprises</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@uniondescouveuses.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (jetestemonentreprise.com)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculateur TJM + check-list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un calculateur de TJM gratuit pour les entrepreneurs à l’essai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coopérer pour entreprendre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">info@cooperer.coop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (annuaire Avise)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un calculateur de TJM gratuit pour les entrepreneurs-salariés</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coopérer pour entreprendre Bretagne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bretagne@cooperer.coop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (ess-bretagne.org)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fédération des CAE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">les-cae@scop.coop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (ambition-ess.org)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">URSCOP Nouvelle-Aquitaine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">urnouvelleaquitaine@scop.coop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (les-scop-nouvelle-aquitaine.coop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-list + TJM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les CAE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cabestan (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@cabestan.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (plaquette)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CoopConnexion (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@coopconnexion.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (coopconnexion.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coopetic (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@coopetic.coop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (coopetic.coop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coopilote (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">administratif@coopilote.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (coopilote.com), adresse administrative</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour vos entrepreneurs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Comptoir des Entrepreneurs (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@lecomptoirdesentrepreneurs.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (fiche les-scop.coop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coopenates (CAE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@coopenates.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (fiche les-cae.coop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Widoobiz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">redaction@widoobiz.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (page d’environ 6 ans)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baromètre des prix + TJM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Journal des Entreprises</t>
-  </si>
-  <si>
-    <t xml:space="preserve">redacweb@lejournaldesentreprises.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (leadiq.com), non confirmée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-list + baromètre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les TPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Espace Auto-Entrepreneur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@espace-autoentrepreneur.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (page presse)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Des simulateurs gratuits pour vos lecteurs auto-entrepreneurs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Courrier des Entreprises</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@lecourrierdesentreprises.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (site)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SDI (Syndicat des indépendants et TPE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@sdi-pme.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour vos adhérents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNION-Indépendants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@union-independants.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (arpe.gouv.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un calculateur de TJM gratuit pour les indépendants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PEPS (portage salarial)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">presse@peps-syndicat.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (peps-syndicat.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculateur TJM + baromètre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Un calculateur de TJM gratuit pour les consultants indépendants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Association</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60 000 rebonds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@60000rebonds.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (variante en .fr ailleurs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Des simulateurs gratuits pour les entrepreneurs qui rebondissent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60 000 rebonds Bourgogne-Franche-Comté</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bfc@60000rebonds.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (page régionale)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Envoi conseillé : jour 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moovjee (mentorat)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">moovjee@twoo-mentorat.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (moovjee.fr)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Simulateurs + TJM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Des outils gratuits pour les jeunes entrepreneurs que vous accompagnez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ordre des experts-comptables Paris IDF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@oec-paris.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-list facture électronique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facture électronique 2027 : une check-list gratuite pour les clients TPE des cabinets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ECF (syndicat des experts-comptables)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@e-c-f.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Officiel (page Facebook)</t>
   </si>
   <si>
     <t xml:space="preserve">BGE Hauts-de-France</t>
@@ -2163,18 +2172,20 @@
         <v>66</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J10" s="5"/>
-      <c r="K10" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K10" s="6" t="n">
         <f aca="false">IF(J10="","",WORKDAY(J10+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L10" s="5"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
       <c r="O10" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2185,16 +2196,16 @@
         <v>60</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>71</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>65</v>
@@ -2227,16 +2238,16 @@
         <v>60</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>76</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>65</v>
@@ -2245,18 +2256,20 @@
         <v>66</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J12" s="5"/>
-      <c r="K12" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K12" s="6" t="n">
         <f aca="false">IF(J12="","",WORKDAY(J12+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L12" s="5"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
       <c r="O12" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2267,16 +2280,16 @@
         <v>60</v>
       </c>
       <c r="C13" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>80</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>65</v>
@@ -2285,18 +2298,20 @@
         <v>66</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J13" s="5"/>
-      <c r="K13" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K13" s="6" t="n">
         <f aca="false">IF(J13="","",WORKDAY(J13+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L13" s="5"/>
       <c r="M13" s="4"/>
       <c r="N13" s="4"/>
       <c r="O13" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2307,16 +2322,16 @@
         <v>60</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>82</v>
-      </c>
       <c r="F14" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>65</v>
@@ -2325,18 +2340,20 @@
         <v>66</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J14" s="5"/>
-      <c r="K14" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K14" s="6" t="n">
         <f aca="false">IF(J14="","",WORKDAY(J14+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L14" s="5"/>
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
       <c r="O14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2347,16 +2364,16 @@
         <v>60</v>
       </c>
       <c r="C15" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>85</v>
-      </c>
       <c r="F15" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>65</v>
@@ -2365,18 +2382,20 @@
         <v>66</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J15" s="5"/>
-      <c r="K15" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K15" s="6" t="n">
         <f aca="false">IF(J15="","",WORKDAY(J15+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L15" s="5"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
       <c r="O15" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2387,16 +2406,16 @@
         <v>60</v>
       </c>
       <c r="C16" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>88</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>89</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>65</v>
@@ -2405,18 +2424,20 @@
         <v>66</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J16" s="5"/>
-      <c r="K16" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J16" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K16" s="6" t="n">
         <f aca="false">IF(J16="","",WORKDAY(J16+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L16" s="5"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
       <c r="O16" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2424,39 +2445,41 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>91</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G17" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H17" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H17" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I17" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J17" s="5"/>
-      <c r="K17" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K17" s="6" t="n">
         <f aca="false">IF(J17="","",WORKDAY(J17+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L17" s="5"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
       <c r="O17" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2464,39 +2487,41 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C18" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>98</v>
-      </c>
       <c r="G18" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H18" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H18" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I18" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J18" s="5"/>
-      <c r="K18" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J18" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K18" s="6" t="n">
         <f aca="false">IF(J18="","",WORKDAY(J18+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L18" s="5"/>
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
       <c r="O18" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2504,39 +2529,41 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C19" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>101</v>
-      </c>
       <c r="F19" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G19" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H19" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H19" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I19" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J19" s="5"/>
-      <c r="K19" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K19" s="6" t="n">
         <f aca="false">IF(J19="","",WORKDAY(J19+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L19" s="5"/>
       <c r="M19" s="4"/>
       <c r="N19" s="4"/>
       <c r="O19" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2544,39 +2571,41 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>103</v>
-      </c>
       <c r="F20" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G20" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H20" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H20" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I20" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J20" s="5"/>
-      <c r="K20" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K20" s="6" t="n">
         <f aca="false">IF(J20="","",WORKDAY(J20+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L20" s="5"/>
       <c r="M20" s="4"/>
       <c r="N20" s="4"/>
       <c r="O20" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2584,28 +2613,28 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C21" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="F21" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="I21" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>67</v>
       </c>
       <c r="J21" s="5"/>
       <c r="K21" s="6" t="str">
@@ -2624,7 +2653,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>108</v>
@@ -2639,13 +2668,13 @@
         <v>111</v>
       </c>
       <c r="G22" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H22" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H22" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I22" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J22" s="5"/>
       <c r="K22" s="6" t="str">
@@ -2664,28 +2693,28 @@
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>112</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>113</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G23" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H23" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H23" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I23" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J23" s="5"/>
       <c r="K23" s="6" t="str">
@@ -2704,13 +2733,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>114</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>115</v>
@@ -2719,13 +2748,13 @@
         <v>116</v>
       </c>
       <c r="G24" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H24" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H24" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I24" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J24" s="5"/>
       <c r="K24" s="6" t="str">
@@ -2744,13 +2773,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>117</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>118</v>
@@ -2759,13 +2788,13 @@
         <v>119</v>
       </c>
       <c r="G25" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H25" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H25" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I25" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J25" s="5"/>
       <c r="K25" s="6" t="str">
@@ -2784,13 +2813,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>120</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>121</v>
@@ -2799,10 +2828,10 @@
         <v>122</v>
       </c>
       <c r="G26" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H26" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I26" s="4" t="s">
         <v>22</v>
@@ -2826,7 +2855,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>123</v>
@@ -2838,16 +2867,16 @@
         <v>125</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G27" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H27" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H27" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I27" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J27" s="5"/>
       <c r="K27" s="6" t="str">
@@ -2956,7 +2985,7 @@
         <v>138</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>139</v>
@@ -2998,7 +3027,7 @@
         <v>141</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>142</v>
@@ -3040,7 +3069,7 @@
         <v>143</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>144</v>
@@ -3082,7 +3111,7 @@
         <v>145</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>146</v>
@@ -3124,7 +3153,7 @@
         <v>147</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>148</v>
@@ -3250,7 +3279,7 @@
         <v>157</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>158</v>
@@ -3292,7 +3321,7 @@
         <v>160</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>161</v>
@@ -3370,7 +3399,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>165</v>
@@ -3385,10 +3414,10 @@
         <v>167</v>
       </c>
       <c r="G40" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H40" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I40" s="4" t="s">
         <v>22</v>
@@ -3412,7 +3441,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>168</v>
@@ -3424,16 +3453,16 @@
         <v>169</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G41" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H41" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H41" s="3" t="s">
-        <v>94</v>
-      </c>
       <c r="I41" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J41" s="5"/>
       <c r="K41" s="6" t="str">
@@ -3452,7 +3481,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>170</v>
@@ -3467,10 +3496,10 @@
         <v>172</v>
       </c>
       <c r="G42" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H42" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I42" s="4" t="s">
         <v>173</v>
@@ -3496,13 +3525,13 @@
         <v>42</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>175</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>176</v>
@@ -3511,10 +3540,10 @@
         <v>167</v>
       </c>
       <c r="G43" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H43" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="H43" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I43" s="4" t="s">
         <v>22</v>
@@ -3538,7 +3567,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>178</v>
@@ -3553,10 +3582,10 @@
         <v>180</v>
       </c>
       <c r="G44" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H44" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="H44" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I44" s="4" t="s">
         <v>132</v>
@@ -3580,7 +3609,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>182</v>
@@ -3595,10 +3624,10 @@
         <v>167</v>
       </c>
       <c r="G45" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H45" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="H45" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I45" s="4" t="s">
         <v>22</v>
@@ -3622,13 +3651,13 @@
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>184</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>185</v>
@@ -3637,10 +3666,10 @@
         <v>167</v>
       </c>
       <c r="G46" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H46" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I46" s="4" t="s">
         <v>22</v>
@@ -3664,7 +3693,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>187</v>
@@ -3679,10 +3708,10 @@
         <v>167</v>
       </c>
       <c r="G47" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H47" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="H47" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I47" s="4" t="s">
         <v>22</v>
@@ -3706,13 +3735,13 @@
         <v>47</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>189</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>190</v>
@@ -3721,10 +3750,10 @@
         <v>191</v>
       </c>
       <c r="G48" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H48" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="H48" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I48" s="4" t="s">
         <v>22</v>
@@ -3754,7 +3783,7 @@
         <v>193</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>194</v>
@@ -3769,7 +3798,7 @@
         <v>196</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J49" s="5"/>
       <c r="K49" s="6" t="str">
@@ -3794,7 +3823,7 @@
         <v>197</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>198</v>
@@ -3836,7 +3865,7 @@
         <v>201</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>202</v>
@@ -3851,7 +3880,7 @@
         <v>196</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J51" s="5"/>
       <c r="K51" s="6" t="str">
@@ -3876,7 +3905,7 @@
         <v>203</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>204</v>
@@ -3891,7 +3920,7 @@
         <v>196</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J52" s="5"/>
       <c r="K52" s="6" t="str">
@@ -3916,7 +3945,7 @@
         <v>205</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>206</v>
@@ -3931,7 +3960,7 @@
         <v>196</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J53" s="5"/>
       <c r="K53" s="6" t="str">
@@ -3971,7 +4000,7 @@
         <v>196</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J54" s="5"/>
       <c r="K54" s="6" t="str">
@@ -3996,7 +4025,7 @@
         <v>209</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>210</v>
@@ -4011,7 +4040,7 @@
         <v>196</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J55" s="5"/>
       <c r="K55" s="6" t="str">
@@ -4120,7 +4149,7 @@
         <v>218</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>219</v>
@@ -4135,7 +4164,7 @@
         <v>196</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J58" s="5"/>
       <c r="K58" s="6" t="str">
@@ -4286,7 +4315,7 @@
         <v>233</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>234</v>
@@ -4412,7 +4441,7 @@
         <v>239</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>240</v>
@@ -4454,7 +4483,7 @@
         <v>241</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>242</v>
@@ -4469,7 +4498,7 @@
         <v>226</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J66" s="5"/>
       <c r="K66" s="6" t="str">
@@ -4522,7 +4551,7 @@
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4" t="s">
-        <v>186</v>
+        <v>250</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4533,25 +4562,25 @@
         <v>244</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G68" s="3" t="s">
         <v>248</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J68" s="5"/>
       <c r="K68" s="6" t="str">
@@ -4573,25 +4602,25 @@
         <v>244</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G69" s="3" t="s">
         <v>248</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I69" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J69" s="5"/>
       <c r="K69" s="6" t="str">
@@ -4613,25 +4642,25 @@
         <v>244</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G70" s="3" t="s">
         <v>248</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J70" s="5"/>
       <c r="K70" s="6" t="str">
@@ -4653,22 +4682,22 @@
         <v>244</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I71" s="4" t="s">
         <v>22</v>
@@ -4695,25 +4724,25 @@
         <v>244</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G72" s="3" t="s">
         <v>248</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J72" s="5"/>
       <c r="K72" s="6" t="str">
@@ -4735,22 +4764,22 @@
         <v>244</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G73" s="3" t="s">
         <v>248</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I73" s="4" t="s">
         <v>22</v>
@@ -4777,22 +4806,22 @@
         <v>244</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G74" s="3" t="s">
         <v>248</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I74" s="4" t="s">
         <v>22</v>
@@ -4819,22 +4848,22 @@
         <v>244</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I75" s="4" t="s">
         <v>22</v>
@@ -4861,25 +4890,25 @@
         <v>244</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>151</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G76" s="3" t="s">
         <v>248</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J76" s="5"/>
       <c r="K76" s="6" t="str">
@@ -4901,25 +4930,25 @@
         <v>244</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G77" s="3" t="s">
         <v>248</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J77" s="5"/>
       <c r="K77" s="6" t="str">
@@ -4941,25 +4970,25 @@
         <v>15</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>21</v>
       </c>
       <c r="I78" s="4" t="s">
-        <v>22</v>
+        <v>132</v>
       </c>
       <c r="J78" s="5" t="n">
         <v>46317</v>
@@ -4972,7 +5001,7 @@
       <c r="M78" s="4"/>
       <c r="N78" s="4"/>
       <c r="O78" s="4" t="s">
-        <v>186</v>
+        <v>289</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4983,25 +5012,25 @@
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J79" s="5"/>
       <c r="K79" s="6" t="str">
@@ -5023,22 +5052,22 @@
         <v>15</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>38</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="I80" s="4" t="s">
         <v>22</v>
@@ -5054,7 +5083,7 @@
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
       <c r="O80" s="4" t="s">
-        <v>186</v>
+        <v>299</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5065,22 +5094,22 @@
         <v>15</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="I81" s="4" t="s">
         <v>22</v>
@@ -5107,13 +5136,13 @@
         <v>52</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F82" s="3" t="s">
         <v>230</v>
@@ -5122,7 +5151,7 @@
         <v>65</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="I82" s="4" t="s">
         <v>22</v>
@@ -5149,22 +5178,22 @@
         <v>52</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="G83" s="3" t="s">
         <v>248</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>22</v>
@@ -5191,22 +5220,22 @@
         <v>52</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="I84" s="4" t="s">
         <v>22</v>
@@ -5230,25 +5259,25 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="G85" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>22</v>
@@ -5272,39 +5301,41 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G86" s="3" t="s">
         <v>130</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="I86" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J86" s="5"/>
-      <c r="K86" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J86" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K86" s="6" t="n">
         <f aca="false">IF(J86="","",WORKDAY(J86+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L86" s="5"/>
       <c r="M86" s="4"/>
       <c r="N86" s="4"/>
       <c r="O86" s="4" t="s">
-        <v>320</v>
+        <v>67</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5312,39 +5343,41 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="I87" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J87" s="5"/>
-      <c r="K87" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J87" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K87" s="6" t="n">
         <f aca="false">IF(J87="","",WORKDAY(J87+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L87" s="5"/>
       <c r="M87" s="4"/>
       <c r="N87" s="4"/>
       <c r="O87" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5355,36 +5388,38 @@
         <v>44</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>167</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="I88" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="J88" s="5"/>
-      <c r="K88" s="6" t="str">
+        <v>22</v>
+      </c>
+      <c r="J88" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="K88" s="6" t="n">
         <f aca="false">IF(J88="","",WORKDAY(J88+4,1))</f>
-        <v/>
+        <v>46323</v>
       </c>
       <c r="L88" s="5"/>
       <c r="M88" s="4"/>
       <c r="N88" s="4"/>
       <c r="O88" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5395,25 +5430,25 @@
         <v>44</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="G89" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="H89" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="F89" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="G89" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="H89" s="3" t="s">
-        <v>329</v>
-      </c>
       <c r="I89" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J89" s="5"/>
       <c r="K89" s="6" t="str">
@@ -5424,7 +5459,7 @@
       <c r="M89" s="4"/>
       <c r="N89" s="4"/>
       <c r="O89" s="4" t="s">
-        <v>68</v>
+        <v>335</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5435,16 +5470,16 @@
         <v>126</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="G90" s="3" t="s">
         <v>130</v>
@@ -5453,7 +5488,7 @@
         <v>196</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J90" s="5"/>
       <c r="K90" s="6" t="str">
@@ -5475,16 +5510,16 @@
         <v>126</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="G91" s="3" t="s">
         <v>130</v>
@@ -5493,7 +5528,7 @@
         <v>196</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J91" s="5"/>
       <c r="K91" s="6" t="str">
@@ -5515,16 +5550,16 @@
         <v>126</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>62</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>130</v>
@@ -5533,7 +5568,7 @@
         <v>196</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J92" s="5"/>
       <c r="K92" s="6" t="str">
@@ -5555,16 +5590,16 @@
         <v>126</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="G93" s="3" t="s">
         <v>130</v>
@@ -5573,7 +5608,7 @@
         <v>196</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J93" s="5"/>
       <c r="K93" s="6" t="str">
@@ -5595,16 +5630,16 @@
         <v>126</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>130</v>
@@ -5613,7 +5648,7 @@
         <v>196</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J94" s="5"/>
       <c r="K94" s="6" t="str">
@@ -5624,7 +5659,7 @@
       <c r="M94" s="4"/>
       <c r="N94" s="4"/>
       <c r="O94" s="4" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5635,16 +5670,16 @@
         <v>126</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>130</v>
@@ -5653,7 +5688,7 @@
         <v>196</v>
       </c>
       <c r="I95" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J95" s="5"/>
       <c r="K95" s="6" t="str">
@@ -5664,7 +5699,7 @@
       <c r="M95" s="4"/>
       <c r="N95" s="4"/>
       <c r="O95" s="4" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5675,16 +5710,16 @@
         <v>126</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="G96" s="3" t="s">
         <v>130</v>
@@ -5693,7 +5728,7 @@
         <v>196</v>
       </c>
       <c r="I96" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J96" s="5"/>
       <c r="K96" s="6" t="str">
@@ -5704,7 +5739,7 @@
       <c r="M96" s="4"/>
       <c r="N96" s="4"/>
       <c r="O96" s="4" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5715,16 +5750,16 @@
         <v>126</v>
       </c>
       <c r="C97" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E97" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="F97" s="3" t="s">
         <v>354</v>
-      </c>
-      <c r="D97" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E97" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="F97" s="3" t="s">
-        <v>351</v>
       </c>
       <c r="G97" s="3" t="s">
         <v>130</v>
@@ -5733,7 +5768,7 @@
         <v>196</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
       <c r="J97" s="5"/>
       <c r="K97" s="6" t="str">
@@ -5744,7 +5779,7 @@
       <c r="M97" s="4"/>
       <c r="N97" s="4"/>
       <c r="O97" s="4" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7859,12 +7894,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -7873,25 +7908,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>44</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -7900,7 +7935,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -7909,7 +7944,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -7927,25 +7962,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.0416666666666667</v>
+        <v>0.0333333333333333</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -7954,7 +7989,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -7963,12 +7998,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7976,13 +8011,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8012,7 +8047,7 @@
       </c>
       <c r="C20" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A20,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A20,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8046,7 +8081,7 @@
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A22,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D22" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A22,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8055,7 +8090,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A23)</f>
@@ -8063,7 +8098,7 @@
       </c>
       <c r="C23" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A23,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D23" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A23,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8140,7 +8175,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A28)</f>
@@ -8148,7 +8183,7 @@
       </c>
       <c r="C28" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A28,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D28" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A28,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8157,7 +8192,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -8165,7 +8200,7 @@
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">SUM(D19:D28)</f>
@@ -8196,7 +8231,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8204,12 +8239,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8217,27 +8252,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8245,27 +8280,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection 26/10 : 17 relances supplémentaires (32 au total)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="393">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -506,9 +506,6 @@
   </si>
   <si>
     <t xml:space="preserve">entreprendre@indre.cci.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relance prévue le 26/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">CCI Loir-et-Cher</t>
@@ -1451,7 +1448,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1487,14 +1484,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFF8D6"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFD8A8"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3129,7 +3118,7 @@
         <v>65</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J32" s="5" t="n">
         <v>46315</v>
@@ -3138,11 +3127,13 @@
         <f aca="false">IF(J32="","",WORKDAY(J32+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L32" s="5"/>
+      <c r="L32" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M32" s="4"/>
       <c r="N32" s="4"/>
       <c r="O32" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3153,13 +3144,13 @@
         <v>59</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>144</v>
@@ -3171,7 +3162,7 @@
         <v>65</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J33" s="5" t="n">
         <v>46315</v>
@@ -3180,11 +3171,13 @@
         <f aca="false">IF(J33="","",WORKDAY(J33+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L33" s="5"/>
+      <c r="L33" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M33" s="4"/>
       <c r="N33" s="4"/>
       <c r="O33" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3195,16 +3188,16 @@
         <v>59</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E34" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="F34" s="3" t="s">
         <v>153</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>154</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>64</v>
@@ -3213,7 +3206,7 @@
         <v>65</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J34" s="5" t="n">
         <v>46315</v>
@@ -3222,11 +3215,13 @@
         <f aca="false">IF(J34="","",WORKDAY(J34+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L34" s="5"/>
+      <c r="L34" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M34" s="4"/>
       <c r="N34" s="4"/>
       <c r="O34" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3237,16 +3232,16 @@
         <v>59</v>
       </c>
       <c r="C35" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="E35" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="F35" s="3" t="s">
         <v>157</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>158</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>64</v>
@@ -3255,7 +3250,7 @@
         <v>65</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J35" s="5" t="n">
         <v>46315</v>
@@ -3264,11 +3259,13 @@
         <f aca="false">IF(J35="","",WORKDAY(J35+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L35" s="5"/>
+      <c r="L35" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M35" s="4"/>
       <c r="N35" s="4"/>
       <c r="O35" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3279,16 +3276,16 @@
         <v>59</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>129</v>
       </c>
       <c r="E36" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>161</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>64</v>
@@ -3323,16 +3320,16 @@
         <v>59</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E37" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>163</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>164</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>64</v>
@@ -3341,7 +3338,7 @@
         <v>65</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J37" s="5" t="n">
         <v>46315</v>
@@ -3350,11 +3347,13 @@
         <f aca="false">IF(J37="","",WORKDAY(J37+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L37" s="5"/>
+      <c r="L37" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M37" s="4"/>
       <c r="N37" s="4"/>
       <c r="O37" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3365,16 +3364,16 @@
         <v>59</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E38" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="F38" s="3" t="s">
         <v>166</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>167</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>64</v>
@@ -3383,7 +3382,7 @@
         <v>65</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J38" s="5" t="n">
         <v>46315</v>
@@ -3392,11 +3391,13 @@
         <f aca="false">IF(J38="","",WORKDAY(J38+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L38" s="5"/>
+      <c r="L38" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M38" s="4"/>
       <c r="N38" s="4"/>
       <c r="O38" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3407,16 +3408,16 @@
         <v>59</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>129</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>64</v>
@@ -3425,7 +3426,7 @@
         <v>65</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J39" s="5" t="n">
         <v>46315</v>
@@ -3434,11 +3435,13 @@
         <f aca="false">IF(J39="","",WORKDAY(J39+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L39" s="5"/>
+      <c r="L39" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M39" s="4"/>
       <c r="N39" s="4"/>
       <c r="O39" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3449,16 +3452,16 @@
         <v>92</v>
       </c>
       <c r="C40" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E40" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="D40" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="E40" s="3" t="s">
+      <c r="F40" s="3" t="s">
         <v>171</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>172</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>95</v>
@@ -3493,13 +3496,13 @@
         <v>92</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>81</v>
@@ -3533,16 +3536,16 @@
         <v>92</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E42" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="F42" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>177</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>95</v>
@@ -3551,7 +3554,7 @@
         <v>96</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J42" s="5" t="n">
         <v>46315</v>
@@ -3566,7 +3569,7 @@
       </c>
       <c r="N42" s="4"/>
       <c r="O42" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3577,16 +3580,16 @@
         <v>92</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>95</v>
@@ -3621,16 +3624,16 @@
         <v>92</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>114</v>
       </c>
       <c r="E44" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="F44" s="3" t="s">
         <v>183</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>184</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>95</v>
@@ -3652,7 +3655,7 @@
       <c r="M44" s="4"/>
       <c r="N44" s="4"/>
       <c r="O44" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3663,16 +3666,16 @@
         <v>92</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>129</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>95</v>
@@ -3707,16 +3710,16 @@
         <v>92</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>95</v>
@@ -3738,7 +3741,7 @@
       <c r="M46" s="4"/>
       <c r="N46" s="4"/>
       <c r="O46" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3749,16 +3752,16 @@
         <v>92</v>
       </c>
       <c r="C47" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E47" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D47" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>192</v>
-      </c>
       <c r="F47" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>95</v>
@@ -3767,7 +3770,7 @@
         <v>96</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J47" s="5" t="n">
         <v>46316</v>
@@ -3776,11 +3779,13 @@
         <f aca="false">IF(J47="","",WORKDAY(J47+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L47" s="5"/>
+      <c r="L47" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M47" s="4"/>
       <c r="N47" s="4"/>
       <c r="O47" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3791,16 +3796,16 @@
         <v>92</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E48" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="F48" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="F48" s="3" t="s">
-        <v>195</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>95</v>
@@ -3809,7 +3814,7 @@
         <v>96</v>
       </c>
       <c r="I48" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J48" s="5" t="n">
         <v>46316</v>
@@ -3818,11 +3823,13 @@
         <f aca="false">IF(J48="","",WORKDAY(J48+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L48" s="5"/>
+      <c r="L48" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M48" s="4"/>
       <c r="N48" s="4"/>
       <c r="O48" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3830,25 +3837,25 @@
         <v>48</v>
       </c>
       <c r="B49" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>196</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>197</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E49" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="F49" s="3" t="s">
         <v>198</v>
-      </c>
-      <c r="F49" s="3" t="s">
-        <v>199</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>111</v>
@@ -3870,25 +3877,25 @@
         <v>49</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E50" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F50" s="3" t="s">
         <v>202</v>
-      </c>
-      <c r="F50" s="3" t="s">
-        <v>203</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I50" s="4" t="s">
         <v>76</v>
@@ -3904,7 +3911,7 @@
       <c r="M50" s="4"/>
       <c r="N50" s="4"/>
       <c r="O50" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3912,25 +3919,25 @@
         <v>50</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>111</v>
@@ -3952,25 +3959,25 @@
         <v>51</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>111</v>
@@ -3992,25 +3999,25 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>111</v>
@@ -4032,25 +4039,25 @@
         <v>53</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>129</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G54" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I54" s="4" t="s">
         <v>111</v>
@@ -4072,25 +4079,25 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E55" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="F55" s="3" t="s">
         <v>214</v>
-      </c>
-      <c r="F55" s="3" t="s">
-        <v>215</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I55" s="4" t="s">
         <v>111</v>
@@ -4112,28 +4119,28 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>129</v>
       </c>
       <c r="E56" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="F56" s="3" t="s">
         <v>217</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>218</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J56" s="5" t="n">
         <v>46316</v>
@@ -4142,11 +4149,13 @@
         <f aca="false">IF(J56="","",WORKDAY(J56+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L56" s="5"/>
+      <c r="L56" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M56" s="4"/>
       <c r="N56" s="4"/>
       <c r="O56" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4154,28 +4163,28 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>129</v>
       </c>
       <c r="E57" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="F57" s="3" t="s">
         <v>220</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>221</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J57" s="5" t="n">
         <v>46316</v>
@@ -4184,11 +4193,13 @@
         <f aca="false">IF(J57="","",WORKDAY(J57+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L57" s="5"/>
+      <c r="L57" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M57" s="4"/>
       <c r="N57" s="4"/>
       <c r="O57" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4196,25 +4207,25 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E58" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="F58" s="3" t="s">
         <v>223</v>
-      </c>
-      <c r="F58" s="3" t="s">
-        <v>224</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I58" s="4" t="s">
         <v>111</v>
@@ -4228,7 +4239,7 @@
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
       <c r="O58" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4236,25 +4247,25 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C59" s="3" t="s">
         <v>226</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>227</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E59" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="F59" s="3" t="s">
         <v>228</v>
-      </c>
-      <c r="F59" s="3" t="s">
-        <v>229</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I59" s="4" t="s">
         <v>76</v>
@@ -4270,7 +4281,7 @@
       <c r="M59" s="4"/>
       <c r="N59" s="4"/>
       <c r="O59" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4278,28 +4289,28 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>114</v>
       </c>
       <c r="E60" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F60" s="3" t="s">
         <v>233</v>
-      </c>
-      <c r="F60" s="3" t="s">
-        <v>234</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I60" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J60" s="5" t="n">
         <v>46316</v>
@@ -4308,11 +4319,13 @@
         <f aca="false">IF(J60="","",WORKDAY(J60+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L60" s="5"/>
+      <c r="L60" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M60" s="4"/>
       <c r="N60" s="4"/>
       <c r="O60" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4320,28 +4333,28 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I61" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J61" s="5" t="n">
         <v>46316</v>
@@ -4350,11 +4363,13 @@
         <f aca="false">IF(J61="","",WORKDAY(J61+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L61" s="5"/>
+      <c r="L61" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M61" s="4"/>
       <c r="N61" s="4"/>
       <c r="O61" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4362,28 +4377,28 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I62" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J62" s="5" t="n">
         <v>46316</v>
@@ -4392,11 +4407,13 @@
         <f aca="false">IF(J62="","",WORKDAY(J62+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L62" s="5"/>
+      <c r="L62" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M62" s="4"/>
       <c r="N62" s="4"/>
       <c r="O62" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4404,28 +4421,28 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I63" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J63" s="5" t="n">
         <v>46316</v>
@@ -4434,11 +4451,13 @@
         <f aca="false">IF(J63="","",WORKDAY(J63+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L63" s="5"/>
+      <c r="L63" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M63" s="4"/>
       <c r="N63" s="4"/>
       <c r="O63" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4446,28 +4465,28 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>129</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I64" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J64" s="5" t="n">
         <v>46316</v>
@@ -4476,11 +4495,13 @@
         <f aca="false">IF(J64="","",WORKDAY(J64+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L64" s="5"/>
+      <c r="L64" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M64" s="4"/>
       <c r="N64" s="4"/>
       <c r="O64" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4488,28 +4509,28 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G65" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J65" s="5" t="n">
         <v>46316</v>
@@ -4518,11 +4539,13 @@
         <f aca="false">IF(J65="","",WORKDAY(J65+4,1))</f>
         <v>46321</v>
       </c>
-      <c r="L65" s="5"/>
+      <c r="L65" s="5" t="n">
+        <v>46321</v>
+      </c>
       <c r="M65" s="4"/>
       <c r="N65" s="4"/>
       <c r="O65" s="4" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4530,25 +4553,25 @@
         <v>65</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E66" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="F66" s="3" t="s">
         <v>246</v>
-      </c>
-      <c r="F66" s="3" t="s">
-        <v>247</v>
       </c>
       <c r="G66" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>111</v>
@@ -4562,7 +4585,7 @@
       <c r="M66" s="4"/>
       <c r="N66" s="4"/>
       <c r="O66" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4570,25 +4593,25 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="C67" s="3" t="s">
         <v>248</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>249</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="F67" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="F67" s="3" t="s">
+      <c r="G67" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="G67" s="3" t="s">
+      <c r="H67" s="3" t="s">
         <v>252</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>253</v>
       </c>
       <c r="I67" s="4" t="s">
         <v>66</v>
@@ -4604,7 +4627,7 @@
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4612,25 +4635,25 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="F68" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="F68" s="3" t="s">
+      <c r="G68" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H68" s="3" t="s">
         <v>257</v>
-      </c>
-      <c r="G68" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="H68" s="3" t="s">
-        <v>258</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>111</v>
@@ -4644,7 +4667,7 @@
       <c r="M68" s="4"/>
       <c r="N68" s="4"/>
       <c r="O68" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4652,25 +4675,25 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E69" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="F69" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="F69" s="3" t="s">
-        <v>261</v>
-      </c>
       <c r="G69" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I69" s="4" t="s">
         <v>111</v>
@@ -4684,7 +4707,7 @@
       <c r="M69" s="4"/>
       <c r="N69" s="4"/>
       <c r="O69" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4692,25 +4715,25 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E70" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="F70" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="F70" s="3" t="s">
-        <v>264</v>
-      </c>
       <c r="G70" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>111</v>
@@ -4724,7 +4747,7 @@
       <c r="M70" s="4"/>
       <c r="N70" s="4"/>
       <c r="O70" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4732,25 +4755,25 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E71" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="F71" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="F71" s="3" t="s">
+      <c r="G71" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="G71" s="3" t="s">
+      <c r="H71" s="3" t="s">
         <v>268</v>
-      </c>
-      <c r="H71" s="3" t="s">
-        <v>269</v>
       </c>
       <c r="I71" s="4" t="s">
         <v>66</v>
@@ -4766,7 +4789,7 @@
       <c r="M71" s="4"/>
       <c r="N71" s="4"/>
       <c r="O71" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4774,25 +4797,25 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E72" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="F72" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="F72" s="3" t="s">
-        <v>272</v>
-      </c>
       <c r="G72" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I72" s="4" t="s">
         <v>111</v>
@@ -4806,7 +4829,7 @@
       <c r="M72" s="4"/>
       <c r="N72" s="4"/>
       <c r="O72" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4814,25 +4837,25 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E73" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="F73" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="F73" s="3" t="s">
-        <v>275</v>
-      </c>
       <c r="G73" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I73" s="4" t="s">
         <v>66</v>
@@ -4848,7 +4871,7 @@
       <c r="M73" s="4"/>
       <c r="N73" s="4"/>
       <c r="O73" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4856,25 +4879,25 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E74" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="F74" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="F74" s="3" t="s">
-        <v>278</v>
-      </c>
       <c r="G74" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I74" s="4" t="s">
         <v>66</v>
@@ -4890,7 +4913,7 @@
       <c r="M74" s="4"/>
       <c r="N74" s="4"/>
       <c r="O74" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4898,25 +4921,25 @@
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E75" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="F75" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="F75" s="3" t="s">
+      <c r="G75" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="H75" s="3" t="s">
         <v>281</v>
-      </c>
-      <c r="G75" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="H75" s="3" t="s">
-        <v>282</v>
       </c>
       <c r="I75" s="4" t="s">
         <v>66</v>
@@ -4932,7 +4955,7 @@
       <c r="M75" s="4"/>
       <c r="N75" s="4"/>
       <c r="O75" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4940,25 +4963,25 @@
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C76" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E76" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="D76" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="E76" s="3" t="s">
+      <c r="F76" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="F76" s="3" t="s">
-        <v>285</v>
-      </c>
       <c r="G76" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>111</v>
@@ -4972,7 +4995,7 @@
       <c r="M76" s="4"/>
       <c r="N76" s="4"/>
       <c r="O76" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4980,25 +5003,25 @@
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>114</v>
       </c>
       <c r="E77" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="F77" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="F77" s="3" t="s">
-        <v>288</v>
-      </c>
       <c r="G77" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>111</v>
@@ -5012,7 +5035,7 @@
       <c r="M77" s="4"/>
       <c r="N77" s="4"/>
       <c r="O77" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5023,19 +5046,19 @@
         <v>15</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F78" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="F78" s="3" t="s">
+      <c r="G78" s="3" t="s">
         <v>291</v>
-      </c>
-      <c r="G78" s="3" t="s">
-        <v>292</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>21</v>
@@ -5054,7 +5077,7 @@
       <c r="M78" s="4"/>
       <c r="N78" s="4"/>
       <c r="O78" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5065,22 +5088,22 @@
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="F79" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="F79" s="3" t="s">
+      <c r="G79" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="G79" s="3" t="s">
+      <c r="H79" s="3" t="s">
         <v>297</v>
-      </c>
-      <c r="H79" s="3" t="s">
-        <v>298</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>111</v>
@@ -5094,7 +5117,7 @@
       <c r="M79" s="4"/>
       <c r="N79" s="4"/>
       <c r="O79" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5105,22 +5128,22 @@
         <v>15</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="F80" s="3" t="s">
         <v>300</v>
-      </c>
-      <c r="F80" s="3" t="s">
-        <v>301</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>37</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I80" s="4" t="s">
         <v>66</v>
@@ -5136,7 +5159,7 @@
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
       <c r="O80" s="4" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5147,22 +5170,22 @@
         <v>15</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E81" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="F81" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="F81" s="3" t="s">
-        <v>306</v>
-      </c>
       <c r="G81" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="H81" s="3" t="s">
         <v>297</v>
-      </c>
-      <c r="H81" s="3" t="s">
-        <v>298</v>
       </c>
       <c r="I81" s="4" t="s">
         <v>66</v>
@@ -5178,7 +5201,7 @@
       <c r="M81" s="4"/>
       <c r="N81" s="4"/>
       <c r="O81" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5189,22 +5212,22 @@
         <v>51</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G82" s="3" t="s">
         <v>64</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I82" s="4" t="s">
         <v>66</v>
@@ -5220,7 +5243,7 @@
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
       <c r="O82" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5231,22 +5254,22 @@
         <v>51</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="F83" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="F83" s="3" t="s">
+      <c r="G83" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="H83" s="3" t="s">
         <v>312</v>
-      </c>
-      <c r="G83" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="H83" s="3" t="s">
-        <v>313</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>66</v>
@@ -5262,7 +5285,7 @@
       <c r="M83" s="4"/>
       <c r="N83" s="4"/>
       <c r="O83" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5273,22 +5296,22 @@
         <v>51</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E84" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="F84" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="F84" s="3" t="s">
+      <c r="G84" s="3" t="s">
         <v>316</v>
       </c>
-      <c r="G84" s="3" t="s">
+      <c r="H84" s="3" t="s">
         <v>317</v>
-      </c>
-      <c r="H84" s="3" t="s">
-        <v>318</v>
       </c>
       <c r="I84" s="4" t="s">
         <v>66</v>
@@ -5304,7 +5327,7 @@
       <c r="M84" s="4"/>
       <c r="N84" s="4"/>
       <c r="O84" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5312,25 +5335,25 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C85" s="3" t="s">
         <v>319</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>320</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="F85" s="3" t="s">
         <v>321</v>
-      </c>
-      <c r="F85" s="3" t="s">
-        <v>322</v>
       </c>
       <c r="G85" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>66</v>
@@ -5346,7 +5369,7 @@
       <c r="M85" s="4"/>
       <c r="N85" s="4"/>
       <c r="O85" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5354,25 +5377,25 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E86" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="F86" s="3" t="s">
         <v>325</v>
-      </c>
-      <c r="F86" s="3" t="s">
-        <v>326</v>
       </c>
       <c r="G86" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>66</v>
@@ -5396,25 +5419,25 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="F87" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="F87" s="3" t="s">
+      <c r="G87" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="G87" s="3" t="s">
+      <c r="H87" s="3" t="s">
         <v>330</v>
-      </c>
-      <c r="H87" s="3" t="s">
-        <v>331</v>
       </c>
       <c r="I87" s="4" t="s">
         <v>66</v>
@@ -5441,22 +5464,22 @@
         <v>43</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E88" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="G88" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="F88" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="G88" s="3" t="s">
+      <c r="H88" s="3" t="s">
         <v>334</v>
-      </c>
-      <c r="H88" s="3" t="s">
-        <v>335</v>
       </c>
       <c r="I88" s="4" t="s">
         <v>66</v>
@@ -5472,7 +5495,7 @@
       <c r="M88" s="4"/>
       <c r="N88" s="4"/>
       <c r="O88" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5483,22 +5506,22 @@
         <v>43</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="F89" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="F89" s="3" t="s">
-        <v>339</v>
-      </c>
       <c r="G89" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="H89" s="3" t="s">
         <v>334</v>
-      </c>
-      <c r="H89" s="3" t="s">
-        <v>335</v>
       </c>
       <c r="I89" s="4" t="s">
         <v>111</v>
@@ -5512,7 +5535,7 @@
       <c r="M89" s="4"/>
       <c r="N89" s="4"/>
       <c r="O89" s="4" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5523,22 +5546,22 @@
         <v>131</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E90" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="F90" s="3" t="s">
         <v>342</v>
-      </c>
-      <c r="F90" s="3" t="s">
-        <v>343</v>
       </c>
       <c r="G90" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I90" s="4" t="s">
         <v>111</v>
@@ -5552,7 +5575,7 @@
       <c r="M90" s="4"/>
       <c r="N90" s="4"/>
       <c r="O90" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5563,22 +5586,22 @@
         <v>131</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E91" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="F91" s="3" t="s">
         <v>345</v>
-      </c>
-      <c r="F91" s="3" t="s">
-        <v>346</v>
       </c>
       <c r="G91" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I91" s="4" t="s">
         <v>111</v>
@@ -5592,7 +5615,7 @@
       <c r="M91" s="4"/>
       <c r="N91" s="4"/>
       <c r="O91" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5603,22 +5626,22 @@
         <v>131</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E92" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="F92" s="3" t="s">
         <v>348</v>
-      </c>
-      <c r="F92" s="3" t="s">
-        <v>349</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I92" s="4" t="s">
         <v>111</v>
@@ -5632,7 +5655,7 @@
       <c r="M92" s="4"/>
       <c r="N92" s="4"/>
       <c r="O92" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5643,22 +5666,22 @@
         <v>131</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E93" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="F93" s="3" t="s">
         <v>351</v>
-      </c>
-      <c r="F93" s="3" t="s">
-        <v>352</v>
       </c>
       <c r="G93" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I93" s="4" t="s">
         <v>111</v>
@@ -5672,7 +5695,7 @@
       <c r="M93" s="4"/>
       <c r="N93" s="4"/>
       <c r="O93" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5683,22 +5706,22 @@
         <v>131</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E94" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="F94" s="3" t="s">
         <v>354</v>
-      </c>
-      <c r="F94" s="3" t="s">
-        <v>355</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I94" s="4" t="s">
         <v>111</v>
@@ -5712,7 +5735,7 @@
       <c r="M94" s="4"/>
       <c r="N94" s="4"/>
       <c r="O94" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5723,22 +5746,22 @@
         <v>131</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E95" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F95" s="3" t="s">
         <v>358</v>
-      </c>
-      <c r="F95" s="3" t="s">
-        <v>359</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H95" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I95" s="4" t="s">
         <v>111</v>
@@ -5752,7 +5775,7 @@
       <c r="M95" s="4"/>
       <c r="N95" s="4"/>
       <c r="O95" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5763,22 +5786,22 @@
         <v>131</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G96" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I96" s="4" t="s">
         <v>111</v>
@@ -5792,7 +5815,7 @@
       <c r="M96" s="4"/>
       <c r="N96" s="4"/>
       <c r="O96" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5803,22 +5826,22 @@
         <v>131</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G97" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="I97" s="4" t="s">
         <v>111</v>
@@ -5832,7 +5855,7 @@
       <c r="M97" s="4"/>
       <c r="N97" s="4"/>
       <c r="O97" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7898,15 +7921,15 @@
   </sheetData>
   <autoFilter ref="A1:O200"/>
   <conditionalFormatting sqref="I2:I200">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>"Lien obtenu"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"Adresse invalide"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K200">
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>AND(K2&lt;&gt;"",K2&lt;=TODAY(),L2="",I2="Envoyé")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7947,12 +7970,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -7961,7 +7984,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
@@ -7970,7 +7993,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
@@ -7979,16 +8002,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -7997,7 +8020,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8006,7 +8029,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Refus")</f>
@@ -8015,7 +8038,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
@@ -8024,7 +8047,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
@@ -8033,7 +8056,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -8042,21 +8065,21 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
-        <v>17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8064,13 +8087,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
+        <v>376</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>377</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="D18" s="9" t="s">
         <v>378</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8177,7 +8200,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A25)</f>
@@ -8194,7 +8217,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
@@ -8211,7 +8234,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A27)</f>
@@ -8228,7 +8251,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A28)</f>
@@ -8245,7 +8268,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -8284,7 +8307,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8292,12 +8315,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8305,27 +8328,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8333,27 +8356,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection 26/10 : 8 rebonds enregistrés, nouveau fichier Drive
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="463">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -451,6 +451,9 @@
     <t xml:space="preserve">contact06@cmar-paca.fr</t>
   </si>
   <si>
+    <t xml:space="preserve">26/10 : rebond, l’adresse renvoie vers contact06@urma-paca.fr, qui n’existe pas. Pas de relance.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réseau</t>
   </si>
   <si>
@@ -580,6 +583,9 @@
     <t xml:space="preserve">contact@cma94.com</t>
   </si>
   <si>
+    <t xml:space="preserve">26/10 : rebond, message bloqué par le serveur (Microsoft 365, « Access denied »). Pas de relance.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CMA Île-de-France, Paris</t>
   </si>
   <si>
@@ -730,6 +736,9 @@
     <t xml:space="preserve">Tiers (liste ancienne)</t>
   </si>
   <si>
+    <t xml:space="preserve">26/10 : rebond, adresse inexistante. Pas de relance.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réseau Entreprendre</t>
   </si>
   <si>
@@ -1168,6 +1177,9 @@
     <t xml:space="preserve">contact@portesdebretagne-initiative.fr</t>
   </si>
   <si>
+    <t xml:space="preserve">26/10 : rebond, domaine portesdebretagne-initiative.fr introuvable. Pas de relance.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Initiative Cher</t>
   </si>
   <si>
@@ -1181,6 +1193,9 @@
   </si>
   <si>
     <t xml:space="preserve">Tiers (les-aides.fr, page ancienne)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26/10 : rebond, domaine initiative-aisne.com introuvable. Pas de relance.</t>
   </si>
   <si>
     <t xml:space="preserve">Initiative Melun Val de Seine et Sud 77</t>
@@ -3109,7 +3124,7 @@
         <v>96</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J27" s="5" t="n">
         <v>46321</v>
@@ -3122,7 +3137,7 @@
       <c r="M27" s="4"/>
       <c r="N27" s="4"/>
       <c r="O27" s="4" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3130,25 +3145,25 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I28" s="4" t="s">
         <v>76</v>
@@ -3164,7 +3179,7 @@
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
       <c r="O28" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3175,16 +3190,16 @@
         <v>59</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>64</v>
@@ -3219,16 +3234,16 @@
         <v>59</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>64</v>
@@ -3263,16 +3278,16 @@
         <v>59</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>64</v>
@@ -3307,16 +3322,16 @@
         <v>59</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G32" s="3" t="s">
         <v>64</v>
@@ -3351,16 +3366,16 @@
         <v>59</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G33" s="3" t="s">
         <v>64</v>
@@ -3395,16 +3410,16 @@
         <v>59</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>64</v>
@@ -3439,16 +3454,16 @@
         <v>59</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>64</v>
@@ -3483,16 +3498,16 @@
         <v>59</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>64</v>
@@ -3527,16 +3542,16 @@
         <v>59</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>64</v>
@@ -3571,16 +3586,16 @@
         <v>59</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>64</v>
@@ -3615,16 +3630,16 @@
         <v>59</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>64</v>
@@ -3659,16 +3674,16 @@
         <v>92</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>95</v>
@@ -3703,13 +3718,13 @@
         <v>92</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>81</v>
@@ -3721,7 +3736,7 @@
         <v>96</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J41" s="5" t="n">
         <v>46321</v>
@@ -3734,7 +3749,7 @@
       <c r="M41" s="4"/>
       <c r="N41" s="4"/>
       <c r="O41" s="4" t="s">
-        <v>111</v>
+        <v>174</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3745,16 +3760,16 @@
         <v>92</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>95</v>
@@ -3763,7 +3778,7 @@
         <v>96</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J42" s="5" t="n">
         <v>46315</v>
@@ -3778,7 +3793,7 @@
       </c>
       <c r="N42" s="4"/>
       <c r="O42" s="4" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3789,16 +3804,16 @@
         <v>92</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>95</v>
@@ -3833,16 +3848,16 @@
         <v>92</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>113</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>95</v>
@@ -3864,7 +3879,7 @@
       <c r="M44" s="4"/>
       <c r="N44" s="4"/>
       <c r="O44" s="4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3875,16 +3890,16 @@
         <v>92</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>95</v>
@@ -3919,16 +3934,16 @@
         <v>92</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>95</v>
@@ -3950,7 +3965,7 @@
       <c r="M46" s="4"/>
       <c r="N46" s="4"/>
       <c r="O46" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3961,16 +3976,16 @@
         <v>92</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>95</v>
@@ -4005,16 +4020,16 @@
         <v>92</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>95</v>
@@ -4046,25 +4061,25 @@
         <v>48</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>66</v>
@@ -4088,25 +4103,25 @@
         <v>49</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E50" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H50" s="3" t="s">
         <v>200</v>
-      </c>
-      <c r="F50" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="G50" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="H50" s="3" t="s">
-        <v>198</v>
       </c>
       <c r="I50" s="4" t="s">
         <v>76</v>
@@ -4122,7 +4137,7 @@
       <c r="M50" s="4"/>
       <c r="N50" s="4"/>
       <c r="O50" s="4" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4130,25 +4145,25 @@
         <v>50</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>66</v>
@@ -4172,25 +4187,25 @@
         <v>51</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>66</v>
@@ -4214,25 +4229,25 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>66</v>
@@ -4256,25 +4271,25 @@
         <v>53</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I54" s="4" t="s">
         <v>66</v>
@@ -4298,25 +4313,25 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I55" s="4" t="s">
         <v>66</v>
@@ -4340,25 +4355,25 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I56" s="4" t="s">
         <v>22</v>
@@ -4384,25 +4399,25 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I57" s="4" t="s">
         <v>22</v>
@@ -4428,28 +4443,28 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J58" s="5" t="n">
         <v>46321</v>
@@ -4462,7 +4477,7 @@
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
       <c r="O58" s="4" t="s">
-        <v>111</v>
+        <v>225</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4470,25 +4485,25 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I59" s="4" t="s">
         <v>76</v>
@@ -4504,7 +4519,7 @@
       <c r="M59" s="4"/>
       <c r="N59" s="4"/>
       <c r="O59" s="4" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4512,25 +4527,25 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>113</v>
       </c>
       <c r="E60" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H60" s="3" t="s">
         <v>230</v>
-      </c>
-      <c r="F60" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="G60" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="H60" s="3" t="s">
-        <v>227</v>
       </c>
       <c r="I60" s="4" t="s">
         <v>22</v>
@@ -4556,25 +4571,25 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I61" s="4" t="s">
         <v>22</v>
@@ -4600,25 +4615,25 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I62" s="4" t="s">
         <v>22</v>
@@ -4644,25 +4659,25 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I63" s="4" t="s">
         <v>22</v>
@@ -4688,25 +4703,25 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I64" s="4" t="s">
         <v>22</v>
@@ -4732,25 +4747,25 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I65" s="4" t="s">
         <v>22</v>
@@ -4776,25 +4791,25 @@
         <v>65</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>66</v>
@@ -4818,25 +4833,25 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I67" s="4" t="s">
         <v>66</v>
@@ -4852,7 +4867,7 @@
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4860,25 +4875,25 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>66</v>
@@ -4902,28 +4917,28 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="F69" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="H69" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="G69" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>255</v>
-      </c>
       <c r="I69" s="4" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J69" s="5" t="n">
         <v>46321</v>
@@ -4936,7 +4951,7 @@
       <c r="M69" s="4"/>
       <c r="N69" s="4"/>
       <c r="O69" s="4" t="s">
-        <v>111</v>
+        <v>225</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4944,25 +4959,25 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>66</v>
@@ -4986,25 +5001,25 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="I71" s="4" t="s">
         <v>66</v>
@@ -5020,7 +5035,7 @@
       <c r="M71" s="4"/>
       <c r="N71" s="4"/>
       <c r="O71" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5028,25 +5043,25 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I72" s="4" t="s">
         <v>66</v>
@@ -5070,25 +5085,25 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I73" s="4" t="s">
         <v>66</v>
@@ -5104,7 +5119,7 @@
       <c r="M73" s="4"/>
       <c r="N73" s="4"/>
       <c r="O73" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5112,25 +5127,25 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I74" s="4" t="s">
         <v>66</v>
@@ -5146,7 +5161,7 @@
       <c r="M74" s="4"/>
       <c r="N74" s="4"/>
       <c r="O74" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5154,25 +5169,25 @@
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="I75" s="4" t="s">
         <v>66</v>
@@ -5188,7 +5203,7 @@
       <c r="M75" s="4"/>
       <c r="N75" s="4"/>
       <c r="O75" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5196,25 +5211,25 @@
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>66</v>
@@ -5238,25 +5253,25 @@
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>113</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>66</v>
@@ -5283,19 +5298,19 @@
         <v>15</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>21</v>
@@ -5314,7 +5329,7 @@
       <c r="M78" s="4"/>
       <c r="N78" s="4"/>
       <c r="O78" s="4" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5325,22 +5340,22 @@
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>66</v>
@@ -5367,22 +5382,22 @@
         <v>15</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>37</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="I80" s="4" t="s">
         <v>66</v>
@@ -5398,7 +5413,7 @@
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
       <c r="O80" s="4" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5409,22 +5424,22 @@
         <v>15</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="I81" s="4" t="s">
         <v>66</v>
@@ -5440,7 +5455,7 @@
       <c r="M81" s="4"/>
       <c r="N81" s="4"/>
       <c r="O81" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5451,22 +5466,22 @@
         <v>51</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G82" s="3" t="s">
         <v>64</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="I82" s="4" t="s">
         <v>66</v>
@@ -5482,7 +5497,7 @@
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
       <c r="O82" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5493,22 +5508,22 @@
         <v>51</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>66</v>
@@ -5524,7 +5539,7 @@
       <c r="M83" s="4"/>
       <c r="N83" s="4"/>
       <c r="O83" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5535,22 +5550,22 @@
         <v>51</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="I84" s="4" t="s">
         <v>66</v>
@@ -5566,7 +5581,7 @@
       <c r="M84" s="4"/>
       <c r="N84" s="4"/>
       <c r="O84" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5574,25 +5589,25 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>66</v>
@@ -5608,7 +5623,7 @@
       <c r="M85" s="4"/>
       <c r="N85" s="4"/>
       <c r="O85" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5616,25 +5631,25 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="F86" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="G86" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H86" s="3" t="s">
         <v>323</v>
-      </c>
-      <c r="G86" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="H86" s="3" t="s">
-        <v>320</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>66</v>
@@ -5658,25 +5673,25 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="I87" s="4" t="s">
         <v>66</v>
@@ -5703,22 +5718,22 @@
         <v>43</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="I88" s="4" t="s">
         <v>66</v>
@@ -5734,7 +5749,7 @@
       <c r="M88" s="4"/>
       <c r="N88" s="4"/>
       <c r="O88" s="4" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5745,22 +5760,22 @@
         <v>43</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="G89" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="H89" s="3" t="s">
         <v>335</v>
-      </c>
-      <c r="F89" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="G89" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="H89" s="3" t="s">
-        <v>332</v>
       </c>
       <c r="I89" s="4" t="s">
         <v>66</v>
@@ -5784,25 +5799,25 @@
         <v>89</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I90" s="4" t="s">
         <v>66</v>
@@ -5826,25 +5841,25 @@
         <v>90</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I91" s="4" t="s">
         <v>66</v>
@@ -5868,25 +5883,25 @@
         <v>91</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I92" s="4" t="s">
         <v>66</v>
@@ -5910,25 +5925,25 @@
         <v>92</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I93" s="4" t="s">
         <v>66</v>
@@ -5952,25 +5967,25 @@
         <v>93</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="G94" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H94" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I94" s="4" t="s">
         <v>66</v>
@@ -5994,25 +6009,25 @@
         <v>94</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="G95" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H95" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I95" s="4" t="s">
         <v>66</v>
@@ -6036,25 +6051,25 @@
         <v>95</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I96" s="4" t="s">
         <v>66</v>
@@ -6078,25 +6093,25 @@
         <v>96</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="G97" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I97" s="4" t="s">
         <v>66</v>
@@ -6120,25 +6135,25 @@
         <v>97</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G98" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I98" s="4" t="s">
         <v>66</v>
@@ -6162,25 +6177,25 @@
         <v>98</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I99" s="4" t="s">
         <v>66</v>
@@ -6204,25 +6219,25 @@
         <v>99</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C100" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="E100" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="F100" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="G100" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="D100" s="3" t="s">
-        <v>365</v>
-      </c>
-      <c r="E100" s="3" t="s">
-        <v>366</v>
-      </c>
-      <c r="F100" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="G100" s="3" t="s">
-        <v>361</v>
-      </c>
       <c r="H100" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I100" s="4" t="s">
         <v>66</v>
@@ -6246,28 +6261,28 @@
         <v>100</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H101" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I101" s="4" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J101" s="5" t="n">
         <v>46321</v>
@@ -6280,7 +6295,7 @@
       <c r="M101" s="4"/>
       <c r="N101" s="4"/>
       <c r="O101" s="4" t="s">
-        <v>111</v>
+        <v>372</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6288,25 +6303,25 @@
         <v>101</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G102" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I102" s="4" t="s">
         <v>66</v>
@@ -6330,28 +6345,28 @@
         <v>102</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I103" s="4" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J103" s="5" t="n">
         <v>46321</v>
@@ -6364,7 +6379,7 @@
       <c r="M103" s="4"/>
       <c r="N103" s="4"/>
       <c r="O103" s="4" t="s">
-        <v>111</v>
+        <v>378</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6372,28 +6387,28 @@
         <v>103</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="F104" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G104" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H104" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I104" s="4" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J104" s="5" t="n">
         <v>46321</v>
@@ -6406,7 +6421,7 @@
       <c r="M104" s="4"/>
       <c r="N104" s="4"/>
       <c r="O104" s="4" t="s">
-        <v>111</v>
+        <v>174</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6414,25 +6429,25 @@
         <v>104</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="G105" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H105" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I105" s="4" t="s">
         <v>66</v>
@@ -6456,25 +6471,25 @@
         <v>105</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="G106" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H106" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I106" s="4" t="s">
         <v>66</v>
@@ -6498,25 +6513,25 @@
         <v>106</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E107" s="3" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="G107" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H107" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I107" s="4" t="s">
         <v>66</v>
@@ -6540,25 +6555,25 @@
         <v>107</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H108" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I108" s="4" t="s">
         <v>66</v>
@@ -6582,25 +6597,25 @@
         <v>108</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="G109" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H109" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I109" s="4" t="s">
         <v>66</v>
@@ -6624,25 +6639,25 @@
         <v>109</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E110" s="3" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="G110" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H110" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I110" s="4" t="s">
         <v>66</v>
@@ -6666,25 +6681,25 @@
         <v>110</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E111" s="3" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="G111" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I111" s="4" t="s">
         <v>66</v>
@@ -6708,25 +6723,25 @@
         <v>111</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E112" s="3" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="F112" s="3" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H112" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="I112" s="4" t="s">
         <v>66</v>
@@ -6750,25 +6765,25 @@
         <v>112</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H113" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I113" s="4" t="s">
         <v>66</v>
@@ -6792,25 +6807,25 @@
         <v>113</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H114" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I114" s="4" t="s">
         <v>66</v>
@@ -6834,25 +6849,25 @@
         <v>114</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G115" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H115" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I115" s="4" t="s">
         <v>66</v>
@@ -6876,25 +6891,25 @@
         <v>115</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G116" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H116" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I116" s="4" t="s">
         <v>66</v>
@@ -6918,25 +6933,25 @@
         <v>116</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="D117" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G117" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H117" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I117" s="4" t="s">
         <v>66</v>
@@ -6960,25 +6975,25 @@
         <v>117</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E118" s="3" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G118" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H118" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I118" s="4" t="s">
         <v>66</v>
@@ -7002,25 +7017,25 @@
         <v>118</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E119" s="3" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G119" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H119" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I119" s="4" t="s">
         <v>66</v>
@@ -7044,25 +7059,25 @@
         <v>119</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E120" s="3" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="G120" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H120" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I120" s="4" t="s">
         <v>66</v>
@@ -7089,22 +7104,22 @@
         <v>59</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E121" s="3" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="G121" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H121" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I121" s="4" t="s">
         <v>66</v>
@@ -7128,25 +7143,25 @@
         <v>121</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="F122" s="3" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="G122" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H122" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I122" s="4" t="s">
         <v>66</v>
@@ -7173,16 +7188,16 @@
         <v>92</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E123" s="3" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="F123" s="3" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="G123" s="3" t="s">
         <v>95</v>
@@ -7215,16 +7230,16 @@
         <v>92</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E124" s="3" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="G124" s="3" t="s">
         <v>95</v>
@@ -7233,7 +7248,7 @@
         <v>96</v>
       </c>
       <c r="I124" s="4" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="J124" s="5" t="n">
         <v>46321</v>
@@ -7246,7 +7261,7 @@
       <c r="M124" s="4"/>
       <c r="N124" s="4"/>
       <c r="O124" s="4" t="s">
-        <v>111</v>
+        <v>174</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7257,22 +7272,22 @@
         <v>15</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="G125" s="3" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="H125" s="3" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="I125" s="4" t="s">
         <v>66</v>
@@ -8843,12 +8858,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -8857,7 +8872,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
@@ -8866,16 +8881,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -8884,7 +8899,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -8893,7 +8908,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8902,7 +8917,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Refus")</f>
@@ -8911,25 +8926,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.0172413793103448</v>
+        <v>0.0185185185185185</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -8938,7 +8953,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -8947,12 +8962,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8960,13 +8975,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9056,7 +9071,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A24)</f>
@@ -9073,7 +9088,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A25)</f>
@@ -9090,7 +9105,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
@@ -9107,7 +9122,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A27)</f>
@@ -9124,7 +9139,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A28)</f>
@@ -9141,7 +9156,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -9180,7 +9195,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9188,12 +9203,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9201,27 +9216,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9229,27 +9244,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection : 9 relais dans les départements à forte création (brouillons)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1256" uniqueCount="495">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -1358,6 +1358,102 @@
   </si>
   <si>
     <t xml:space="preserve">83 % des logiciels de caisse cachent leur prix : notre baromètre 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paris Initiative Entreprise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@paris-initiative.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (les-aides.fr, 2021)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boîte à outils créateur + chiffres Sirene</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 269 créations à Paris en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brouillon prêt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Envoi conseillé : jour 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre Paris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">paris@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (annuaire régional des financeurs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hauts-de-Seine Initiative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accueil@hdsi.asso.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (les-aides.fr, 2022)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">278 créations dans les Hauts-de-Seine en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre 92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Terres d’Azur (Grasse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-terres-dazur.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">246 créations dans les Alpes-Maritimes en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CCI Nice Côte d’Azur (financement)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">financement@cote-azur.cci.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Officiel (brochure cote-azur.cci.fr, 2023)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Lille Métropole Nord</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-lmnord.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">215 créations dans le Nord en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Réunion Entreprendre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-reunion.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (fiche du Département 974)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">68 créations à La Réunion en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Montreuillois</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-montreuillois.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">77 créations dans le Pas-de-Calais en octobre : des outils gratuits pour vos porteurs de projet</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de bord de la prospection</t>
@@ -7307,15 +7403,33 @@
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A126" s="3"/>
-      <c r="B126" s="3"/>
-      <c r="C126" s="3"/>
-      <c r="D126" s="3"/>
-      <c r="E126" s="3"/>
-      <c r="F126" s="3"/>
-      <c r="G126" s="3"/>
-      <c r="H126" s="3"/>
-      <c r="I126" s="4"/>
+      <c r="A126" s="3" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E126" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="F126" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="G126" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H126" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="I126" s="4" t="s">
+        <v>438</v>
+      </c>
       <c r="J126" s="5"/>
       <c r="K126" s="6" t="str">
         <f aca="false">IF(J126="","",WORKDAY(J126+4,1))</f>
@@ -7324,18 +7438,38 @@
       <c r="L126" s="5"/>
       <c r="M126" s="4"/>
       <c r="N126" s="4"/>
-      <c r="O126" s="4"/>
+      <c r="O126" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A127" s="3"/>
-      <c r="B127" s="3"/>
-      <c r="C127" s="3"/>
-      <c r="D127" s="3"/>
-      <c r="E127" s="3"/>
-      <c r="F127" s="3"/>
-      <c r="G127" s="3"/>
-      <c r="H127" s="3"/>
-      <c r="I127" s="4"/>
+      <c r="A127" s="3" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="D127" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E127" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="F127" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="G127" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H127" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="I127" s="4" t="s">
+        <v>438</v>
+      </c>
       <c r="J127" s="5"/>
       <c r="K127" s="6" t="str">
         <f aca="false">IF(J127="","",WORKDAY(J127+4,1))</f>
@@ -7344,18 +7478,38 @@
       <c r="L127" s="5"/>
       <c r="M127" s="4"/>
       <c r="N127" s="4"/>
-      <c r="O127" s="4"/>
+      <c r="O127" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A128" s="3"/>
-      <c r="B128" s="3"/>
-      <c r="C128" s="3"/>
-      <c r="D128" s="3"/>
-      <c r="E128" s="3"/>
-      <c r="F128" s="3"/>
-      <c r="G128" s="3"/>
-      <c r="H128" s="3"/>
-      <c r="I128" s="4"/>
+      <c r="A128" s="3" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E128" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="F128" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="G128" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H128" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="I128" s="4" t="s">
+        <v>438</v>
+      </c>
       <c r="J128" s="5"/>
       <c r="K128" s="6" t="str">
         <f aca="false">IF(J128="","",WORKDAY(J128+4,1))</f>
@@ -7364,18 +7518,38 @@
       <c r="L128" s="5"/>
       <c r="M128" s="4"/>
       <c r="N128" s="4"/>
-      <c r="O128" s="4"/>
+      <c r="O128" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A129" s="3"/>
-      <c r="B129" s="3"/>
-      <c r="C129" s="3"/>
-      <c r="D129" s="3"/>
-      <c r="E129" s="3"/>
-      <c r="F129" s="3"/>
-      <c r="G129" s="3"/>
-      <c r="H129" s="3"/>
-      <c r="I129" s="4"/>
+      <c r="A129" s="3" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E129" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="G129" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H129" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="I129" s="4" t="s">
+        <v>438</v>
+      </c>
       <c r="J129" s="5"/>
       <c r="K129" s="6" t="str">
         <f aca="false">IF(J129="","",WORKDAY(J129+4,1))</f>
@@ -7384,18 +7558,38 @@
       <c r="L129" s="5"/>
       <c r="M129" s="4"/>
       <c r="N129" s="4"/>
-      <c r="O129" s="4"/>
+      <c r="O129" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A130" s="3"/>
-      <c r="B130" s="3"/>
-      <c r="C130" s="3"/>
-      <c r="D130" s="3"/>
-      <c r="E130" s="3"/>
-      <c r="F130" s="3"/>
-      <c r="G130" s="3"/>
-      <c r="H130" s="3"/>
-      <c r="I130" s="4"/>
+      <c r="A130" s="3" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E130" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="F130" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="G130" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H130" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="I130" s="4" t="s">
+        <v>438</v>
+      </c>
       <c r="J130" s="5"/>
       <c r="K130" s="6" t="str">
         <f aca="false">IF(J130="","",WORKDAY(J130+4,1))</f>
@@ -7404,18 +7598,38 @@
       <c r="L130" s="5"/>
       <c r="M130" s="4"/>
       <c r="N130" s="4"/>
-      <c r="O130" s="4"/>
+      <c r="O130" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A131" s="3"/>
-      <c r="B131" s="3"/>
-      <c r="C131" s="3"/>
-      <c r="D131" s="3"/>
-      <c r="E131" s="3"/>
-      <c r="F131" s="3"/>
-      <c r="G131" s="3"/>
-      <c r="H131" s="3"/>
-      <c r="I131" s="4"/>
+      <c r="A131" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E131" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="F131" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="G131" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H131" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="I131" s="4" t="s">
+        <v>438</v>
+      </c>
       <c r="J131" s="5"/>
       <c r="K131" s="6" t="str">
         <f aca="false">IF(J131="","",WORKDAY(J131+4,1))</f>
@@ -7424,18 +7638,38 @@
       <c r="L131" s="5"/>
       <c r="M131" s="4"/>
       <c r="N131" s="4"/>
-      <c r="O131" s="4"/>
+      <c r="O131" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A132" s="3"/>
-      <c r="B132" s="3"/>
-      <c r="C132" s="3"/>
-      <c r="D132" s="3"/>
-      <c r="E132" s="3"/>
-      <c r="F132" s="3"/>
-      <c r="G132" s="3"/>
-      <c r="H132" s="3"/>
-      <c r="I132" s="4"/>
+      <c r="A132" s="3" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E132" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="G132" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H132" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="I132" s="4" t="s">
+        <v>438</v>
+      </c>
       <c r="J132" s="5"/>
       <c r="K132" s="6" t="str">
         <f aca="false">IF(J132="","",WORKDAY(J132+4,1))</f>
@@ -7444,18 +7678,38 @@
       <c r="L132" s="5"/>
       <c r="M132" s="4"/>
       <c r="N132" s="4"/>
-      <c r="O132" s="4"/>
+      <c r="O132" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A133" s="3"/>
-      <c r="B133" s="3"/>
-      <c r="C133" s="3"/>
-      <c r="D133" s="3"/>
-      <c r="E133" s="3"/>
-      <c r="F133" s="3"/>
-      <c r="G133" s="3"/>
-      <c r="H133" s="3"/>
-      <c r="I133" s="4"/>
+      <c r="A133" s="3" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E133" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="F133" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="G133" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H133" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="I133" s="4" t="s">
+        <v>438</v>
+      </c>
       <c r="J133" s="5"/>
       <c r="K133" s="6" t="str">
         <f aca="false">IF(J133="","",WORKDAY(J133+4,1))</f>
@@ -7464,18 +7718,38 @@
       <c r="L133" s="5"/>
       <c r="M133" s="4"/>
       <c r="N133" s="4"/>
-      <c r="O133" s="4"/>
+      <c r="O133" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A134" s="3"/>
-      <c r="B134" s="3"/>
-      <c r="C134" s="3"/>
-      <c r="D134" s="3"/>
-      <c r="E134" s="3"/>
-      <c r="F134" s="3"/>
-      <c r="G134" s="3"/>
-      <c r="H134" s="3"/>
-      <c r="I134" s="4"/>
+      <c r="A134" s="3" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E134" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="G134" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H134" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="I134" s="4" t="s">
+        <v>438</v>
+      </c>
       <c r="J134" s="5"/>
       <c r="K134" s="6" t="str">
         <f aca="false">IF(J134="","",WORKDAY(J134+4,1))</f>
@@ -7484,7 +7758,9 @@
       <c r="L134" s="5"/>
       <c r="M134" s="4"/>
       <c r="N134" s="4"/>
-      <c r="O134" s="4"/>
+      <c r="O134" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="3"/>
@@ -8858,30 +9134,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>433</v>
+        <v>465</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>434</v>
+        <v>466</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
-        <v>123</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>435</v>
+        <v>467</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>436</v>
+        <v>468</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
@@ -8890,7 +9166,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>437</v>
+        <v>469</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -8899,7 +9175,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>438</v>
+        <v>470</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -8908,7 +9184,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>439</v>
+        <v>471</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -8926,7 +9202,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>440</v>
+        <v>472</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
@@ -8935,7 +9211,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>441</v>
+        <v>473</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
@@ -8944,7 +9220,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>442</v>
+        <v>474</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -8953,7 +9229,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>443</v>
+        <v>475</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -8962,12 +9238,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>444</v>
+        <v>476</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>445</v>
+        <v>477</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8975,13 +9251,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>446</v>
+        <v>478</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>447</v>
+        <v>479</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>448</v>
+        <v>480</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9041,7 +9317,7 @@
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A22)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A22,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
@@ -9092,7 +9368,7 @@
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A25)</f>
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
@@ -9109,7 +9385,7 @@
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A26,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
@@ -9156,11 +9432,11 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>449</v>
+        <v>481</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
@@ -9195,7 +9471,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>450</v>
+        <v>482</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9203,12 +9479,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>451</v>
+        <v>483</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>452</v>
+        <v>484</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9216,27 +9492,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>453</v>
+        <v>485</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>454</v>
+        <v>486</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>455</v>
+        <v>487</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>456</v>
+        <v>488</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>457</v>
+        <v>489</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9244,27 +9520,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>458</v>
+        <v>490</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>459</v>
+        <v>491</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>460</v>
+        <v>492</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>461</v>
+        <v>493</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>462</v>
+        <v>494</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection 26/10 : 9 relais envoyés, 1 rebond
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1256" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1256" uniqueCount="493">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -1373,12 +1373,6 @@
   </si>
   <si>
     <t xml:space="preserve">1 269 créations à Paris en octobre : des outils gratuits pour vos porteurs de projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brouillon prêt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Envoi conseillé : jour 9</t>
   </si>
   <si>
     <t xml:space="preserve">Réseau Entreprendre Paris</t>
@@ -7428,18 +7422,20 @@
         <v>437</v>
       </c>
       <c r="I126" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="J126" s="5"/>
-      <c r="K126" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="J126" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="K126" s="6" t="n">
         <f aca="false">IF(J126="","",WORKDAY(J126+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L126" s="5"/>
       <c r="M126" s="4"/>
       <c r="N126" s="4"/>
       <c r="O126" s="4" t="s">
-        <v>439</v>
+        <v>111</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7450,16 +7446,16 @@
         <v>226</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="F127" s="3" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="G127" s="3" t="s">
         <v>436</v>
@@ -7468,18 +7464,20 @@
         <v>437</v>
       </c>
       <c r="I127" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="J127" s="5"/>
-      <c r="K127" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="J127" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="K127" s="6" t="n">
         <f aca="false">IF(J127="","",WORKDAY(J127+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L127" s="5"/>
       <c r="M127" s="4"/>
       <c r="N127" s="4"/>
       <c r="O127" s="4" t="s">
-        <v>439</v>
+        <v>111</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7490,36 +7488,38 @@
         <v>196</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="G128" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H128" s="3" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="I128" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="J128" s="5"/>
-      <c r="K128" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="J128" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="K128" s="6" t="n">
         <f aca="false">IF(J128="","",WORKDAY(J128+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L128" s="5"/>
       <c r="M128" s="4"/>
       <c r="N128" s="4"/>
       <c r="O128" s="4" t="s">
-        <v>439</v>
+        <v>111</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7530,36 +7530,38 @@
         <v>226</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="F129" s="3" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="G129" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H129" s="3" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="I129" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="J129" s="5"/>
-      <c r="K129" s="6" t="str">
+        <v>76</v>
+      </c>
+      <c r="J129" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="K129" s="6" t="n">
         <f aca="false">IF(J129="","",WORKDAY(J129+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L129" s="5"/>
       <c r="M129" s="4"/>
       <c r="N129" s="4"/>
       <c r="O129" s="4" t="s">
-        <v>439</v>
+        <v>174</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7570,13 +7572,13 @@
         <v>196</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="F130" s="3" t="s">
         <v>199</v>
@@ -7585,21 +7587,23 @@
         <v>436</v>
       </c>
       <c r="H130" s="3" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="I130" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="J130" s="5"/>
-      <c r="K130" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="J130" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="K130" s="6" t="n">
         <f aca="false">IF(J130="","",WORKDAY(J130+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L130" s="5"/>
       <c r="M130" s="4"/>
       <c r="N130" s="4"/>
       <c r="O130" s="4" t="s">
-        <v>439</v>
+        <v>111</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7610,36 +7614,38 @@
         <v>59</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="D131" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="G131" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H131" s="3" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="I131" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="J131" s="5"/>
-      <c r="K131" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="J131" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="K131" s="6" t="n">
         <f aca="false">IF(J131="","",WORKDAY(J131+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L131" s="5"/>
       <c r="M131" s="4"/>
       <c r="N131" s="4"/>
       <c r="O131" s="4" t="s">
-        <v>439</v>
+        <v>111</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7650,13 +7656,13 @@
         <v>196</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="D132" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="F132" s="3" t="s">
         <v>435</v>
@@ -7665,21 +7671,23 @@
         <v>436</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="I132" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="J132" s="5"/>
-      <c r="K132" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="J132" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="K132" s="6" t="n">
         <f aca="false">IF(J132="","",WORKDAY(J132+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L132" s="5"/>
       <c r="M132" s="4"/>
       <c r="N132" s="4"/>
       <c r="O132" s="4" t="s">
-        <v>439</v>
+        <v>111</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7690,36 +7698,38 @@
         <v>196</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>139</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="G133" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H133" s="3" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="I133" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="J133" s="5"/>
-      <c r="K133" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="J133" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="K133" s="6" t="n">
         <f aca="false">IF(J133="","",WORKDAY(J133+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L133" s="5"/>
       <c r="M133" s="4"/>
       <c r="N133" s="4"/>
       <c r="O133" s="4" t="s">
-        <v>439</v>
+        <v>111</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7730,13 +7740,13 @@
         <v>196</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="D134" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="F134" s="3" t="s">
         <v>435</v>
@@ -7745,21 +7755,23 @@
         <v>436</v>
       </c>
       <c r="H134" s="3" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="I134" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="J134" s="5"/>
-      <c r="K134" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="J134" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="K134" s="6" t="n">
         <f aca="false">IF(J134="","",WORKDAY(J134+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L134" s="5"/>
       <c r="M134" s="4"/>
       <c r="N134" s="4"/>
       <c r="O134" s="4" t="s">
-        <v>439</v>
+        <v>111</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9134,12 +9146,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -9148,25 +9160,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>108</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -9175,7 +9187,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -9184,7 +9196,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9202,25 +9214,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.0185185185185185</v>
+        <v>0.0172413793103448</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -9229,7 +9241,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -9238,12 +9250,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9251,13 +9263,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>477</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>478</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>479</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9321,7 +9333,7 @@
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A22,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D22" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A22,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9372,7 +9384,7 @@
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9389,7 +9401,7 @@
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A26,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D26" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A26,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9432,7 +9444,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -9440,7 +9452,7 @@
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">SUM(D19:D28)</f>
@@ -9471,7 +9483,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9479,12 +9491,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9492,27 +9504,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9520,27 +9532,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection : 14 relais supplémentaires (brouillons)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1256" uniqueCount="493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="540">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -1448,6 +1448,147 @@
   </si>
   <si>
     <t xml:space="preserve">77 créations dans le Pas-de-Calais en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Essonne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-essonne.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (les-aides.fr ; variante .fr sur un document de 2019)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">124 créations dans l'Essonne en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brouillon prêt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Envoi conseillé : jour 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réseau Entreprendre Val d’Oise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valdoise@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">128 créations dans le Val-d'Oise en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Nord Seine-et-Marne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-nord77.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">154 créations en Seine-et-Marne en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Melun Val de Seine et Sud 77 (nouvelle adresse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plateforme@initiative-mvs-sud77.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (annuaire régional ; l’ancienne adresse camvs.com a été bloquée)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Béziers Ouest Hérault</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@iboh.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">167 créations dans l'Hérault en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Oise Est</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@oise-est.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34 créations dans l'Oise en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Oise Ouest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@oise-ouest.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Haute-Garonne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-haute-garonne.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">156 créations en Haute-Garonne en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Loire-Atlantique Nord</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiativeloireatlantiquenord.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93 créations en Loire-Atlantique en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Loire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-loire.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">74 créations dans la Loire en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Moselle Nord</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pfil@synergie-ceei.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (les-aides.fr, PDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90 créations en Moselle en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Guadeloupe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guadeloupe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guadeloupe-active@wanadoo.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (les-aides.fr, 2021), adresse ancienne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">73 créations en Guadeloupe en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Anjou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-anjou.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">59 créations en Maine-et-Loire en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Dombes Val de Saône</t>
+  </si>
+  <si>
+    <t xml:space="preserve">idvs@initiative-dombesvaldesaone.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51 créations dans l'Ain en octobre : des outils gratuits pour vos porteurs de projet</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de bord de la prospection</t>
@@ -7775,15 +7916,33 @@
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A135" s="3"/>
-      <c r="B135" s="3"/>
-      <c r="C135" s="3"/>
-      <c r="D135" s="3"/>
-      <c r="E135" s="3"/>
-      <c r="F135" s="3"/>
-      <c r="G135" s="3"/>
-      <c r="H135" s="3"/>
-      <c r="I135" s="4"/>
+      <c r="A135" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C135" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="D135" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E135" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="F135" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="G135" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H135" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="I135" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J135" s="5"/>
       <c r="K135" s="6" t="str">
         <f aca="false">IF(J135="","",WORKDAY(J135+4,1))</f>
@@ -7792,18 +7951,38 @@
       <c r="L135" s="5"/>
       <c r="M135" s="4"/>
       <c r="N135" s="4"/>
-      <c r="O135" s="4"/>
+      <c r="O135" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A136" s="3"/>
-      <c r="B136" s="3"/>
-      <c r="C136" s="3"/>
-      <c r="D136" s="3"/>
-      <c r="E136" s="3"/>
-      <c r="F136" s="3"/>
-      <c r="G136" s="3"/>
-      <c r="H136" s="3"/>
-      <c r="I136" s="4"/>
+      <c r="A136" s="3" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E136" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="F136" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="G136" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H136" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="I136" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J136" s="5"/>
       <c r="K136" s="6" t="str">
         <f aca="false">IF(J136="","",WORKDAY(J136+4,1))</f>
@@ -7812,18 +7991,38 @@
       <c r="L136" s="5"/>
       <c r="M136" s="4"/>
       <c r="N136" s="4"/>
-      <c r="O136" s="4"/>
+      <c r="O136" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A137" s="3"/>
-      <c r="B137" s="3"/>
-      <c r="C137" s="3"/>
-      <c r="D137" s="3"/>
-      <c r="E137" s="3"/>
-      <c r="F137" s="3"/>
-      <c r="G137" s="3"/>
-      <c r="H137" s="3"/>
-      <c r="I137" s="4"/>
+      <c r="A137" s="3" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C137" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="D137" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E137" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="F137" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="G137" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H137" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="I137" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J137" s="5"/>
       <c r="K137" s="6" t="str">
         <f aca="false">IF(J137="","",WORKDAY(J137+4,1))</f>
@@ -7832,18 +8031,38 @@
       <c r="L137" s="5"/>
       <c r="M137" s="4"/>
       <c r="N137" s="4"/>
-      <c r="O137" s="4"/>
+      <c r="O137" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A138" s="3"/>
-      <c r="B138" s="3"/>
-      <c r="C138" s="3"/>
-      <c r="D138" s="3"/>
-      <c r="E138" s="3"/>
-      <c r="F138" s="3"/>
-      <c r="G138" s="3"/>
-      <c r="H138" s="3"/>
-      <c r="I138" s="4"/>
+      <c r="A138" s="3" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E138" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="F138" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="G138" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H138" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="I138" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J138" s="5"/>
       <c r="K138" s="6" t="str">
         <f aca="false">IF(J138="","",WORKDAY(J138+4,1))</f>
@@ -7852,18 +8071,38 @@
       <c r="L138" s="5"/>
       <c r="M138" s="4"/>
       <c r="N138" s="4"/>
-      <c r="O138" s="4"/>
+      <c r="O138" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A139" s="3"/>
-      <c r="B139" s="3"/>
-      <c r="C139" s="3"/>
-      <c r="D139" s="3"/>
-      <c r="E139" s="3"/>
-      <c r="F139" s="3"/>
-      <c r="G139" s="3"/>
-      <c r="H139" s="3"/>
-      <c r="I139" s="4"/>
+      <c r="A139" s="3" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E139" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="F139" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="G139" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H139" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="I139" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J139" s="5"/>
       <c r="K139" s="6" t="str">
         <f aca="false">IF(J139="","",WORKDAY(J139+4,1))</f>
@@ -7872,18 +8111,38 @@
       <c r="L139" s="5"/>
       <c r="M139" s="4"/>
       <c r="N139" s="4"/>
-      <c r="O139" s="4"/>
+      <c r="O139" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A140" s="3"/>
-      <c r="B140" s="3"/>
-      <c r="C140" s="3"/>
-      <c r="D140" s="3"/>
-      <c r="E140" s="3"/>
-      <c r="F140" s="3"/>
-      <c r="G140" s="3"/>
-      <c r="H140" s="3"/>
-      <c r="I140" s="4"/>
+      <c r="A140" s="3" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="D140" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E140" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="F140" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="G140" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H140" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="I140" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J140" s="5"/>
       <c r="K140" s="6" t="str">
         <f aca="false">IF(J140="","",WORKDAY(J140+4,1))</f>
@@ -7892,18 +8151,38 @@
       <c r="L140" s="5"/>
       <c r="M140" s="4"/>
       <c r="N140" s="4"/>
-      <c r="O140" s="4"/>
+      <c r="O140" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A141" s="3"/>
-      <c r="B141" s="3"/>
-      <c r="C141" s="3"/>
-      <c r="D141" s="3"/>
-      <c r="E141" s="3"/>
-      <c r="F141" s="3"/>
-      <c r="G141" s="3"/>
-      <c r="H141" s="3"/>
-      <c r="I141" s="4"/>
+      <c r="A141" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E141" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="F141" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="G141" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H141" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="I141" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J141" s="5"/>
       <c r="K141" s="6" t="str">
         <f aca="false">IF(J141="","",WORKDAY(J141+4,1))</f>
@@ -7912,18 +8191,38 @@
       <c r="L141" s="5"/>
       <c r="M141" s="4"/>
       <c r="N141" s="4"/>
-      <c r="O141" s="4"/>
+      <c r="O141" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A142" s="3"/>
-      <c r="B142" s="3"/>
-      <c r="C142" s="3"/>
-      <c r="D142" s="3"/>
-      <c r="E142" s="3"/>
-      <c r="F142" s="3"/>
-      <c r="G142" s="3"/>
-      <c r="H142" s="3"/>
-      <c r="I142" s="4"/>
+      <c r="A142" s="3" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="D142" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E142" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="F142" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="G142" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H142" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="I142" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J142" s="5"/>
       <c r="K142" s="6" t="str">
         <f aca="false">IF(J142="","",WORKDAY(J142+4,1))</f>
@@ -7932,18 +8231,38 @@
       <c r="L142" s="5"/>
       <c r="M142" s="4"/>
       <c r="N142" s="4"/>
-      <c r="O142" s="4"/>
+      <c r="O142" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A143" s="3"/>
-      <c r="B143" s="3"/>
-      <c r="C143" s="3"/>
-      <c r="D143" s="3"/>
-      <c r="E143" s="3"/>
-      <c r="F143" s="3"/>
-      <c r="G143" s="3"/>
-      <c r="H143" s="3"/>
-      <c r="I143" s="4"/>
+      <c r="A143" s="3" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C143" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E143" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="F143" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="G143" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H143" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="I143" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J143" s="5"/>
       <c r="K143" s="6" t="str">
         <f aca="false">IF(J143="","",WORKDAY(J143+4,1))</f>
@@ -7952,18 +8271,38 @@
       <c r="L143" s="5"/>
       <c r="M143" s="4"/>
       <c r="N143" s="4"/>
-      <c r="O143" s="4"/>
+      <c r="O143" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A144" s="3"/>
-      <c r="B144" s="3"/>
-      <c r="C144" s="3"/>
-      <c r="D144" s="3"/>
-      <c r="E144" s="3"/>
-      <c r="F144" s="3"/>
-      <c r="G144" s="3"/>
-      <c r="H144" s="3"/>
-      <c r="I144" s="4"/>
+      <c r="A144" s="3" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C144" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="D144" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E144" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="F144" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="G144" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H144" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="I144" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J144" s="5"/>
       <c r="K144" s="6" t="str">
         <f aca="false">IF(J144="","",WORKDAY(J144+4,1))</f>
@@ -7972,18 +8311,38 @@
       <c r="L144" s="5"/>
       <c r="M144" s="4"/>
       <c r="N144" s="4"/>
-      <c r="O144" s="4"/>
+      <c r="O144" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A145" s="3"/>
-      <c r="B145" s="3"/>
-      <c r="C145" s="3"/>
-      <c r="D145" s="3"/>
-      <c r="E145" s="3"/>
-      <c r="F145" s="3"/>
-      <c r="G145" s="3"/>
-      <c r="H145" s="3"/>
-      <c r="I145" s="4"/>
+      <c r="A145" s="3" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E145" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="F145" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="G145" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H145" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="I145" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J145" s="5"/>
       <c r="K145" s="6" t="str">
         <f aca="false">IF(J145="","",WORKDAY(J145+4,1))</f>
@@ -7992,18 +8351,38 @@
       <c r="L145" s="5"/>
       <c r="M145" s="4"/>
       <c r="N145" s="4"/>
-      <c r="O145" s="4"/>
+      <c r="O145" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A146" s="3"/>
-      <c r="B146" s="3"/>
-      <c r="C146" s="3"/>
-      <c r="D146" s="3"/>
-      <c r="E146" s="3"/>
-      <c r="F146" s="3"/>
-      <c r="G146" s="3"/>
-      <c r="H146" s="3"/>
-      <c r="I146" s="4"/>
+      <c r="A146" s="3" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="E146" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="F146" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="G146" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H146" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="I146" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J146" s="5"/>
       <c r="K146" s="6" t="str">
         <f aca="false">IF(J146="","",WORKDAY(J146+4,1))</f>
@@ -8012,18 +8391,38 @@
       <c r="L146" s="5"/>
       <c r="M146" s="4"/>
       <c r="N146" s="4"/>
-      <c r="O146" s="4"/>
+      <c r="O146" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A147" s="3"/>
-      <c r="B147" s="3"/>
-      <c r="C147" s="3"/>
-      <c r="D147" s="3"/>
-      <c r="E147" s="3"/>
-      <c r="F147" s="3"/>
-      <c r="G147" s="3"/>
-      <c r="H147" s="3"/>
-      <c r="I147" s="4"/>
+      <c r="A147" s="3" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="D147" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E147" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="F147" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="G147" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H147" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="I147" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J147" s="5"/>
       <c r="K147" s="6" t="str">
         <f aca="false">IF(J147="","",WORKDAY(J147+4,1))</f>
@@ -8032,18 +8431,38 @@
       <c r="L147" s="5"/>
       <c r="M147" s="4"/>
       <c r="N147" s="4"/>
-      <c r="O147" s="4"/>
+      <c r="O147" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A148" s="3"/>
-      <c r="B148" s="3"/>
-      <c r="C148" s="3"/>
-      <c r="D148" s="3"/>
-      <c r="E148" s="3"/>
-      <c r="F148" s="3"/>
-      <c r="G148" s="3"/>
-      <c r="H148" s="3"/>
-      <c r="I148" s="4"/>
+      <c r="A148" s="3" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E148" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="G148" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H148" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="I148" s="4" t="s">
+        <v>467</v>
+      </c>
       <c r="J148" s="5"/>
       <c r="K148" s="6" t="str">
         <f aca="false">IF(J148="","",WORKDAY(J148+4,1))</f>
@@ -8052,7 +8471,9 @@
       <c r="L148" s="5"/>
       <c r="M148" s="4"/>
       <c r="N148" s="4"/>
-      <c r="O148" s="4"/>
+      <c r="O148" s="4" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="3"/>
@@ -9146,30 +9567,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>463</v>
+        <v>510</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>464</v>
+        <v>511</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
-        <v>132</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>465</v>
+        <v>512</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>466</v>
+        <v>513</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
@@ -9178,7 +9599,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>467</v>
+        <v>514</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -9187,7 +9608,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>468</v>
+        <v>515</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -9196,7 +9617,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>469</v>
+        <v>516</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9214,7 +9635,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>470</v>
+        <v>517</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
@@ -9223,7 +9644,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>471</v>
+        <v>518</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
@@ -9232,7 +9653,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>472</v>
+        <v>519</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -9241,7 +9662,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>473</v>
+        <v>520</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -9250,12 +9671,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>474</v>
+        <v>521</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>475</v>
+        <v>522</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9263,13 +9684,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>476</v>
+        <v>523</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>477</v>
+        <v>524</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>478</v>
+        <v>525</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9380,7 +9801,7 @@
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A25)</f>
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
@@ -9397,7 +9818,7 @@
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A26,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
@@ -9444,11 +9865,11 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>479</v>
+        <v>526</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
@@ -9483,7 +9904,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>480</v>
+        <v>527</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9491,12 +9912,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>481</v>
+        <v>528</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>482</v>
+        <v>529</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9504,27 +9925,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>483</v>
+        <v>530</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>484</v>
+        <v>531</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>485</v>
+        <v>532</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>486</v>
+        <v>533</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>487</v>
+        <v>534</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9532,27 +9953,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>488</v>
+        <v>535</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>489</v>
+        <v>536</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>490</v>
+        <v>537</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>491</v>
+        <v>538</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>492</v>
+        <v>539</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection : réponse de Réseau Entreprendre Paris
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="541">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -1382,6 +1382,9 @@
   </si>
   <si>
     <t xml:space="preserve">Tiers (annuaire régional des financeurs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26/10 : réponse de Félicité et Maroussia (« Merci pour votre message et votre outil ! »). Réponse préparée en brouillon : proposition d’un texte de présentation et du décompte des créations parisiennes. Pas de relance.</t>
   </si>
   <si>
     <t xml:space="preserve">Hauts-de-Seine Initiative</t>
@@ -7605,7 +7608,7 @@
         <v>437</v>
       </c>
       <c r="I127" s="4" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="J127" s="5" t="n">
         <v>46321</v>
@@ -7615,10 +7618,12 @@
         <v>46328</v>
       </c>
       <c r="L127" s="5"/>
-      <c r="M127" s="4"/>
+      <c r="M127" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="N127" s="4"/>
       <c r="O127" s="4" t="s">
-        <v>111</v>
+        <v>441</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7629,22 +7634,22 @@
         <v>196</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G128" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H128" s="3" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="I128" s="4" t="s">
         <v>66</v>
@@ -7671,13 +7676,13 @@
         <v>226</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F129" s="3" t="s">
         <v>440</v>
@@ -7686,7 +7691,7 @@
         <v>436</v>
       </c>
       <c r="H129" s="3" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="I129" s="4" t="s">
         <v>76</v>
@@ -7713,13 +7718,13 @@
         <v>196</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F130" s="3" t="s">
         <v>199</v>
@@ -7728,7 +7733,7 @@
         <v>436</v>
       </c>
       <c r="H130" s="3" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="I130" s="4" t="s">
         <v>66</v>
@@ -7755,22 +7760,22 @@
         <v>59</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D131" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G131" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H131" s="3" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="I131" s="4" t="s">
         <v>66</v>
@@ -7797,13 +7802,13 @@
         <v>196</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D132" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F132" s="3" t="s">
         <v>435</v>
@@ -7812,7 +7817,7 @@
         <v>436</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="I132" s="4" t="s">
         <v>66</v>
@@ -7839,22 +7844,22 @@
         <v>196</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>139</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G133" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H133" s="3" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="I133" s="4" t="s">
         <v>66</v>
@@ -7881,13 +7886,13 @@
         <v>196</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D134" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F134" s="3" t="s">
         <v>435</v>
@@ -7896,7 +7901,7 @@
         <v>436</v>
       </c>
       <c r="H134" s="3" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="I134" s="4" t="s">
         <v>66</v>
@@ -7923,25 +7928,25 @@
         <v>196</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D135" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F135" s="3" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="G135" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="I135" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J135" s="5"/>
       <c r="K135" s="6" t="str">
@@ -7952,7 +7957,7 @@
       <c r="M135" s="4"/>
       <c r="N135" s="4"/>
       <c r="O135" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7963,13 +7968,13 @@
         <v>226</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D136" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F136" s="3" t="s">
         <v>199</v>
@@ -7978,10 +7983,10 @@
         <v>436</v>
       </c>
       <c r="H136" s="3" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="I136" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J136" s="5"/>
       <c r="K136" s="6" t="str">
@@ -7992,7 +7997,7 @@
       <c r="M136" s="4"/>
       <c r="N136" s="4"/>
       <c r="O136" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8003,13 +8008,13 @@
         <v>196</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E137" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F137" s="3" t="s">
         <v>440</v>
@@ -8018,10 +8023,10 @@
         <v>436</v>
       </c>
       <c r="H137" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="I137" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J137" s="5"/>
       <c r="K137" s="6" t="str">
@@ -8032,7 +8037,7 @@
       <c r="M137" s="4"/>
       <c r="N137" s="4"/>
       <c r="O137" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8043,25 +8048,25 @@
         <v>196</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D138" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E138" s="3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F138" s="3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G138" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H138" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="I138" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J138" s="5"/>
       <c r="K138" s="6" t="str">
@@ -8072,7 +8077,7 @@
       <c r="M138" s="4"/>
       <c r="N138" s="4"/>
       <c r="O138" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8083,25 +8088,25 @@
         <v>196</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F139" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G139" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H139" s="3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="I139" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J139" s="5"/>
       <c r="K139" s="6" t="str">
@@ -8112,7 +8117,7 @@
       <c r="M139" s="4"/>
       <c r="N139" s="4"/>
       <c r="O139" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8123,13 +8128,13 @@
         <v>196</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F140" s="3" t="s">
         <v>199</v>
@@ -8138,10 +8143,10 @@
         <v>436</v>
       </c>
       <c r="H140" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="I140" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J140" s="5"/>
       <c r="K140" s="6" t="str">
@@ -8152,7 +8157,7 @@
       <c r="M140" s="4"/>
       <c r="N140" s="4"/>
       <c r="O140" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8163,13 +8168,13 @@
         <v>196</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D141" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F141" s="3" t="s">
         <v>199</v>
@@ -8178,10 +8183,10 @@
         <v>436</v>
       </c>
       <c r="H141" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="I141" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J141" s="5"/>
       <c r="K141" s="6" t="str">
@@ -8192,7 +8197,7 @@
       <c r="M141" s="4"/>
       <c r="N141" s="4"/>
       <c r="O141" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8203,13 +8208,13 @@
         <v>196</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F142" s="3" t="s">
         <v>435</v>
@@ -8218,10 +8223,10 @@
         <v>436</v>
       </c>
       <c r="H142" s="3" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="I142" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J142" s="5"/>
       <c r="K142" s="6" t="str">
@@ -8232,7 +8237,7 @@
       <c r="M142" s="4"/>
       <c r="N142" s="4"/>
       <c r="O142" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8243,13 +8248,13 @@
         <v>196</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E143" s="3" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F143" s="3" t="s">
         <v>435</v>
@@ -8258,10 +8263,10 @@
         <v>436</v>
       </c>
       <c r="H143" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="I143" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J143" s="5"/>
       <c r="K143" s="6" t="str">
@@ -8272,7 +8277,7 @@
       <c r="M143" s="4"/>
       <c r="N143" s="4"/>
       <c r="O143" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8283,13 +8288,13 @@
         <v>196</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F144" s="3" t="s">
         <v>199</v>
@@ -8298,10 +8303,10 @@
         <v>436</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="I144" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J144" s="5"/>
       <c r="K144" s="6" t="str">
@@ -8312,7 +8317,7 @@
       <c r="M144" s="4"/>
       <c r="N144" s="4"/>
       <c r="O144" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8323,25 +8328,25 @@
         <v>196</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>113</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="G145" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H145" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="I145" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J145" s="5"/>
       <c r="K145" s="6" t="str">
@@ -8352,7 +8357,7 @@
       <c r="M145" s="4"/>
       <c r="N145" s="4"/>
       <c r="O145" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8363,25 +8368,25 @@
         <v>196</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="G146" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="I146" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J146" s="5"/>
       <c r="K146" s="6" t="str">
@@ -8392,7 +8397,7 @@
       <c r="M146" s="4"/>
       <c r="N146" s="4"/>
       <c r="O146" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8403,25 +8408,25 @@
         <v>196</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G147" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H147" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="I147" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J147" s="5"/>
       <c r="K147" s="6" t="str">
@@ -8432,7 +8437,7 @@
       <c r="M147" s="4"/>
       <c r="N147" s="4"/>
       <c r="O147" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8443,13 +8448,13 @@
         <v>196</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F148" s="3" t="s">
         <v>199</v>
@@ -8458,10 +8463,10 @@
         <v>436</v>
       </c>
       <c r="H148" s="3" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="I148" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J148" s="5"/>
       <c r="K148" s="6" t="str">
@@ -8472,7 +8477,7 @@
       <c r="M148" s="4"/>
       <c r="N148" s="4"/>
       <c r="O148" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9567,12 +9572,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -9581,7 +9586,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
@@ -9590,7 +9595,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
@@ -9599,7 +9604,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -9608,16 +9613,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9635,7 +9640,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
@@ -9644,16 +9649,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.0172413793103448</v>
+        <v>0.0258620689655172</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -9662,7 +9667,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -9671,12 +9676,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9684,13 +9689,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9865,7 +9870,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -9904,7 +9909,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9912,12 +9917,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9925,27 +9930,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9953,27 +9958,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection 27/10 : 11 relances, 2 envois
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="543">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -682,6 +682,9 @@
     <t xml:space="preserve">contact@initiative-genevois.fr</t>
   </si>
   <si>
+    <t xml:space="preserve">26/10 : filtre anti-spam Mailinblack, l’expéditeur doit être validé (lien dans le mail reçu). Relance prévue le 02/11/2026.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Initiative Rouen</t>
   </si>
   <si>
@@ -919,6 +922,9 @@
     <t xml:space="preserve">Tiers (fiche les-scop.coop)</t>
   </si>
   <si>
+    <t xml:space="preserve">26/10 : devenue LCE - La Coopérative pour Entreprendre, nouvelle adresse contact@lce.coop (message redirigé). Relance à envoyer à la nouvelle adresse.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Coopenates (CAE)</t>
   </si>
   <si>
@@ -1384,7 +1390,7 @@
     <t xml:space="preserve">Tiers (annuaire régional des financeurs)</t>
   </si>
   <si>
-    <t xml:space="preserve">26/10 : réponse de Félicité et Maroussia (« Merci pour votre message et votre outil ! »). Réponse préparée en brouillon : proposition d’un texte de présentation et du décompte des créations parisiennes. Pas de relance.</t>
+    <t xml:space="preserve">26/10 : réponse de Félicité et Maroussia (« Merci pour votre message et votre outil ! »). Réponse envoyée le 26/10 : proposition d’un texte de présentation et du décompte des créations parisiennes. Pas de relance.</t>
   </si>
   <si>
     <t xml:space="preserve">Hauts-de-Seine Initiative</t>
@@ -1465,19 +1471,19 @@
     <t xml:space="preserve">124 créations dans l'Essonne en octobre : des outils gratuits pour vos porteurs de projet</t>
   </si>
   <si>
+    <t xml:space="preserve">Réseau Entreprendre Val d’Oise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valdoise@reseau-entreprendre.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">128 créations dans le Val-d'Oise en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
     <t xml:space="preserve">Brouillon prêt</t>
   </si>
   <si>
     <t xml:space="preserve">Envoi conseillé : jour 9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réseau Entreprendre Val d’Oise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valdoise@reseau-entreprendre.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">128 créations dans le Val-d'Oise en octobre : des outils gratuits pour vos porteurs de projet</t>
   </si>
   <si>
     <t xml:space="preserve">Initiative Nord Seine-et-Marne</t>
@@ -1892,7 +1898,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1928,6 +1934,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFF8D6"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFD8A8"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -4413,7 +4427,7 @@
       <c r="M51" s="4"/>
       <c r="N51" s="4"/>
       <c r="O51" s="4" t="s">
-        <v>111</v>
+        <v>207</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4424,13 +4438,13 @@
         <v>196</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>199</v>
@@ -4466,13 +4480,13 @@
         <v>196</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>199</v>
@@ -4508,13 +4522,13 @@
         <v>196</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>199</v>
@@ -4550,16 +4564,16 @@
         <v>196</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>135</v>
@@ -4592,16 +4606,16 @@
         <v>196</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>135</v>
@@ -4636,16 +4650,16 @@
         <v>196</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>135</v>
@@ -4680,16 +4694,16 @@
         <v>196</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>135</v>
@@ -4711,7 +4725,7 @@
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
       <c r="O58" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4719,25 +4733,25 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I59" s="4" t="s">
         <v>76</v>
@@ -4753,7 +4767,7 @@
       <c r="M59" s="4"/>
       <c r="N59" s="4"/>
       <c r="O59" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4761,25 +4775,25 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>113</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I60" s="4" t="s">
         <v>22</v>
@@ -4805,25 +4819,25 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I61" s="4" t="s">
         <v>22</v>
@@ -4849,25 +4863,25 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I62" s="4" t="s">
         <v>22</v>
@@ -4893,25 +4907,25 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I63" s="4" t="s">
         <v>22</v>
@@ -4937,25 +4951,25 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I64" s="4" t="s">
         <v>22</v>
@@ -4981,25 +4995,25 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G65" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I65" s="4" t="s">
         <v>22</v>
@@ -5025,25 +5039,25 @@
         <v>65</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G66" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>66</v>
@@ -5067,28 +5081,28 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I67" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J67" s="5" t="n">
         <v>46317</v>
@@ -5097,11 +5111,13 @@
         <f aca="false">IF(J67="","",WORKDAY(J67+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L67" s="5"/>
+      <c r="L67" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5109,25 +5125,25 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>66</v>
@@ -5151,25 +5167,25 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I69" s="4" t="s">
         <v>76</v>
@@ -5185,7 +5201,7 @@
       <c r="M69" s="4"/>
       <c r="N69" s="4"/>
       <c r="O69" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5193,25 +5209,25 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>66</v>
@@ -5235,28 +5251,28 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I71" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J71" s="5" t="n">
         <v>46317</v>
@@ -5265,11 +5281,13 @@
         <f aca="false">IF(J71="","",WORKDAY(J71+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L71" s="5"/>
+      <c r="L71" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M71" s="4"/>
       <c r="N71" s="4"/>
       <c r="O71" s="4" t="s">
-        <v>190</v>
+        <v>22</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5277,25 +5295,25 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I72" s="4" t="s">
         <v>66</v>
@@ -5311,7 +5329,7 @@
       <c r="M72" s="4"/>
       <c r="N72" s="4"/>
       <c r="O72" s="4" t="s">
-        <v>111</v>
+        <v>207</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5319,28 +5337,28 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I73" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J73" s="5" t="n">
         <v>46317</v>
@@ -5349,11 +5367,13 @@
         <f aca="false">IF(J73="","",WORKDAY(J73+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L73" s="5"/>
+      <c r="L73" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M73" s="4"/>
       <c r="N73" s="4"/>
       <c r="O73" s="4" t="s">
-        <v>190</v>
+        <v>22</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5361,28 +5381,28 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I74" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J74" s="5" t="n">
         <v>46317</v>
@@ -5391,11 +5411,13 @@
         <f aca="false">IF(J74="","",WORKDAY(J74+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L74" s="5"/>
+      <c r="L74" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M74" s="4"/>
       <c r="N74" s="4"/>
       <c r="O74" s="4" t="s">
-        <v>190</v>
+        <v>22</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5403,28 +5425,28 @@
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="I75" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J75" s="5" t="n">
         <v>46317</v>
@@ -5433,11 +5455,13 @@
         <f aca="false">IF(J75="","",WORKDAY(J75+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L75" s="5"/>
+      <c r="L75" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M75" s="4"/>
       <c r="N75" s="4"/>
       <c r="O75" s="4" t="s">
-        <v>190</v>
+        <v>22</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5445,25 +5469,25 @@
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>66</v>
@@ -5479,7 +5503,7 @@
       <c r="M76" s="4"/>
       <c r="N76" s="4"/>
       <c r="O76" s="4" t="s">
-        <v>111</v>
+        <v>287</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5487,25 +5511,25 @@
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>113</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>66</v>
@@ -5532,19 +5556,19 @@
         <v>15</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>21</v>
@@ -5563,7 +5587,7 @@
       <c r="M78" s="4"/>
       <c r="N78" s="4"/>
       <c r="O78" s="4" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5574,22 +5598,22 @@
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>66</v>
@@ -5616,25 +5640,25 @@
         <v>15</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>37</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="I80" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J80" s="5" t="n">
         <v>46317</v>
@@ -5643,11 +5667,13 @@
         <f aca="false">IF(J80="","",WORKDAY(J80+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L80" s="5"/>
+      <c r="L80" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
       <c r="O80" s="4" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5658,25 +5684,25 @@
         <v>15</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="I81" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J81" s="5" t="n">
         <v>46317</v>
@@ -5685,11 +5711,13 @@
         <f aca="false">IF(J81="","",WORKDAY(J81+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L81" s="5"/>
+      <c r="L81" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M81" s="4"/>
       <c r="N81" s="4"/>
       <c r="O81" s="4" t="s">
-        <v>190</v>
+        <v>22</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5700,25 +5728,25 @@
         <v>51</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G82" s="3" t="s">
         <v>64</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J82" s="5" t="n">
         <v>46317</v>
@@ -5727,11 +5755,13 @@
         <f aca="false">IF(J82="","",WORKDAY(J82+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L82" s="5"/>
+      <c r="L82" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
       <c r="O82" s="4" t="s">
-        <v>190</v>
+        <v>22</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5742,25 +5772,25 @@
         <v>51</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J83" s="5" t="n">
         <v>46317</v>
@@ -5769,11 +5799,13 @@
         <f aca="false">IF(J83="","",WORKDAY(J83+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L83" s="5"/>
+      <c r="L83" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M83" s="4"/>
       <c r="N83" s="4"/>
       <c r="O83" s="4" t="s">
-        <v>190</v>
+        <v>22</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5784,25 +5816,25 @@
         <v>51</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J84" s="5" t="n">
         <v>46317</v>
@@ -5811,11 +5843,13 @@
         <f aca="false">IF(J84="","",WORKDAY(J84+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L84" s="5"/>
+      <c r="L84" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M84" s="4"/>
       <c r="N84" s="4"/>
       <c r="O84" s="4" t="s">
-        <v>190</v>
+        <v>22</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5823,28 +5857,28 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="G85" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="I85" s="4" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
       <c r="J85" s="5" t="n">
         <v>46317</v>
@@ -5853,11 +5887,13 @@
         <f aca="false">IF(J85="","",WORKDAY(J85+4,1))</f>
         <v>46322</v>
       </c>
-      <c r="L85" s="5"/>
+      <c r="L85" s="5" t="n">
+        <v>46322</v>
+      </c>
       <c r="M85" s="4"/>
       <c r="N85" s="4"/>
       <c r="O85" s="4" t="s">
-        <v>190</v>
+        <v>22</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5865,25 +5901,25 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>104</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="G86" s="3" t="s">
         <v>135</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>66</v>
@@ -5907,25 +5943,25 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I87" s="4" t="s">
         <v>66</v>
@@ -5952,22 +5988,22 @@
         <v>43</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>171</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="I88" s="4" t="s">
         <v>66</v>
@@ -5983,7 +6019,7 @@
       <c r="M88" s="4"/>
       <c r="N88" s="4"/>
       <c r="O88" s="4" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5994,22 +6030,22 @@
         <v>43</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="I89" s="4" t="s">
         <v>66</v>
@@ -6036,16 +6072,16 @@
         <v>131</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="G90" s="3" t="s">
         <v>135</v>
@@ -6078,16 +6114,16 @@
         <v>131</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="G91" s="3" t="s">
         <v>135</v>
@@ -6120,16 +6156,16 @@
         <v>131</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>135</v>
@@ -6162,16 +6198,16 @@
         <v>131</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="G93" s="3" t="s">
         <v>135</v>
@@ -6193,7 +6229,7 @@
       <c r="M93" s="4"/>
       <c r="N93" s="4"/>
       <c r="O93" s="4" t="s">
-        <v>111</v>
+        <v>207</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6204,16 +6240,16 @@
         <v>131</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>135</v>
@@ -6246,16 +6282,16 @@
         <v>131</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>135</v>
@@ -6288,16 +6324,16 @@
         <v>131</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E96" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="F96" s="3" t="s">
         <v>359</v>
-      </c>
-      <c r="F96" s="3" t="s">
-        <v>357</v>
       </c>
       <c r="G96" s="3" t="s">
         <v>135</v>
@@ -6330,16 +6366,16 @@
         <v>131</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="G97" s="3" t="s">
         <v>135</v>
@@ -6372,19 +6408,19 @@
         <v>196</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="F98" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G98" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H98" s="3" t="s">
         <v>200</v>
@@ -6414,19 +6450,19 @@
         <v>196</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F99" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H99" s="3" t="s">
         <v>200</v>
@@ -6456,19 +6492,19 @@
         <v>196</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="F100" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G100" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H100" s="3" t="s">
         <v>200</v>
@@ -6498,19 +6534,19 @@
         <v>196</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="F101" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H101" s="3" t="s">
         <v>200</v>
@@ -6529,7 +6565,7 @@
       <c r="M101" s="4"/>
       <c r="N101" s="4"/>
       <c r="O101" s="4" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6540,19 +6576,19 @@
         <v>196</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>109</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F102" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G102" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H102" s="3" t="s">
         <v>200</v>
@@ -6582,19 +6618,19 @@
         <v>196</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H103" s="3" t="s">
         <v>200</v>
@@ -6613,7 +6649,7 @@
       <c r="M103" s="4"/>
       <c r="N103" s="4"/>
       <c r="O103" s="4" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6624,19 +6660,19 @@
         <v>196</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F104" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G104" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H104" s="3" t="s">
         <v>200</v>
@@ -6666,19 +6702,19 @@
         <v>196</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="G105" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H105" s="3" t="s">
         <v>200</v>
@@ -6697,7 +6733,7 @@
       <c r="M105" s="4"/>
       <c r="N105" s="4"/>
       <c r="O105" s="4" t="s">
-        <v>111</v>
+        <v>207</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6708,19 +6744,19 @@
         <v>196</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E106" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="F106" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="F106" s="3" t="s">
-        <v>383</v>
-      </c>
       <c r="G106" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H106" s="3" t="s">
         <v>200</v>
@@ -6750,19 +6786,19 @@
         <v>196</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E107" s="3" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="G107" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H107" s="3" t="s">
         <v>200</v>
@@ -6792,19 +6828,19 @@
         <v>196</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H108" s="3" t="s">
         <v>200</v>
@@ -6834,19 +6870,19 @@
         <v>196</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="G109" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H109" s="3" t="s">
         <v>200</v>
@@ -6876,19 +6912,19 @@
         <v>196</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E110" s="3" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="G110" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H110" s="3" t="s">
         <v>200</v>
@@ -6918,19 +6954,19 @@
         <v>196</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E111" s="3" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="G111" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H111" s="3" t="s">
         <v>200</v>
@@ -6960,22 +6996,22 @@
         <v>196</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E112" s="3" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="F112" s="3" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H112" s="3" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="I112" s="4" t="s">
         <v>66</v>
@@ -7002,19 +7038,19 @@
         <v>196</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H113" s="3" t="s">
         <v>200</v>
@@ -7041,22 +7077,22 @@
         <v>113</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H114" s="3" t="s">
         <v>200</v>
@@ -7083,22 +7119,22 @@
         <v>114</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G115" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H115" s="3" t="s">
         <v>200</v>
@@ -7125,22 +7161,22 @@
         <v>115</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G116" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H116" s="3" t="s">
         <v>200</v>
@@ -7167,22 +7203,22 @@
         <v>116</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="D117" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G117" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H117" s="3" t="s">
         <v>200</v>
@@ -7209,22 +7245,22 @@
         <v>117</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>79</v>
       </c>
       <c r="E118" s="3" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G118" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H118" s="3" t="s">
         <v>200</v>
@@ -7251,22 +7287,22 @@
         <v>118</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>69</v>
       </c>
       <c r="E119" s="3" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G119" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H119" s="3" t="s">
         <v>200</v>
@@ -7293,22 +7329,22 @@
         <v>119</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E120" s="3" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G120" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H120" s="3" t="s">
         <v>200</v>
@@ -7338,19 +7374,19 @@
         <v>59</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E121" s="3" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="G121" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H121" s="3" t="s">
         <v>200</v>
@@ -7380,19 +7416,19 @@
         <v>131</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F122" s="3" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="G122" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="H122" s="3" t="s">
         <v>200</v>
@@ -7422,16 +7458,16 @@
         <v>92</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E123" s="3" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="F123" s="3" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="G123" s="3" t="s">
         <v>95</v>
@@ -7464,16 +7500,16 @@
         <v>92</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E124" s="3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="G124" s="3" t="s">
         <v>95</v>
@@ -7506,22 +7542,22 @@
         <v>15</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="G125" s="3" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="H125" s="3" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="I125" s="4" t="s">
         <v>66</v>
@@ -7548,22 +7584,22 @@
         <v>196</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D126" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="F126" s="3" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="G126" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H126" s="3" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="I126" s="4" t="s">
         <v>66</v>
@@ -7587,25 +7623,25 @@
         <v>126</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E127" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="F127" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="G127" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="H127" s="3" t="s">
         <v>439</v>
-      </c>
-      <c r="F127" s="3" t="s">
-        <v>440</v>
-      </c>
-      <c r="G127" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="H127" s="3" t="s">
-        <v>437</v>
       </c>
       <c r="I127" s="4" t="s">
         <v>27</v>
@@ -7623,7 +7659,7 @@
       </c>
       <c r="N127" s="4"/>
       <c r="O127" s="4" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7634,22 +7670,22 @@
         <v>196</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="G128" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H128" s="3" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="I128" s="4" t="s">
         <v>66</v>
@@ -7673,25 +7709,25 @@
         <v>128</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E129" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="G129" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="H129" s="3" t="s">
         <v>447</v>
-      </c>
-      <c r="F129" s="3" t="s">
-        <v>440</v>
-      </c>
-      <c r="G129" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="H129" s="3" t="s">
-        <v>445</v>
       </c>
       <c r="I129" s="4" t="s">
         <v>76</v>
@@ -7718,22 +7754,22 @@
         <v>196</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="F130" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G130" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H130" s="3" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="I130" s="4" t="s">
         <v>66</v>
@@ -7760,22 +7796,22 @@
         <v>59</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D131" s="3" t="s">
         <v>128</v>
       </c>
       <c r="E131" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="F131" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="G131" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="H131" s="3" t="s">
         <v>452</v>
-      </c>
-      <c r="F131" s="3" t="s">
-        <v>453</v>
-      </c>
-      <c r="G131" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="H131" s="3" t="s">
-        <v>450</v>
       </c>
       <c r="I131" s="4" t="s">
         <v>66</v>
@@ -7802,22 +7838,22 @@
         <v>196</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="D132" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="F132" s="3" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="G132" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="I132" s="4" t="s">
         <v>66</v>
@@ -7844,22 +7880,22 @@
         <v>196</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>139</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="G133" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H133" s="3" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="I133" s="4" t="s">
         <v>66</v>
@@ -7886,22 +7922,22 @@
         <v>196</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D134" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="F134" s="3" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="G134" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H134" s="3" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="I134" s="4" t="s">
         <v>66</v>
@@ -7928,36 +7964,38 @@
         <v>196</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="D135" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="F135" s="3" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G135" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="I135" s="4" t="s">
-        <v>468</v>
-      </c>
-      <c r="J135" s="5"/>
-      <c r="K135" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="J135" s="5" t="n">
+        <v>46322</v>
+      </c>
+      <c r="K135" s="6" t="n">
         <f aca="false">IF(J135="","",WORKDAY(J135+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L135" s="5"/>
       <c r="M135" s="4"/>
       <c r="N135" s="4"/>
       <c r="O135" s="4" t="s">
-        <v>469</v>
+        <v>111</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7965,7 +8003,7 @@
         <v>135</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C136" s="3" t="s">
         <v>470</v>
@@ -7980,13 +8018,13 @@
         <v>199</v>
       </c>
       <c r="G136" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H136" s="3" t="s">
         <v>472</v>
       </c>
       <c r="I136" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J136" s="5"/>
       <c r="K136" s="6" t="str">
@@ -7997,7 +8035,7 @@
       <c r="M136" s="4"/>
       <c r="N136" s="4"/>
       <c r="O136" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8008,36 +8046,38 @@
         <v>196</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E137" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="F137" s="3" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="G137" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H137" s="3" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="I137" s="4" t="s">
-        <v>468</v>
-      </c>
-      <c r="J137" s="5"/>
-      <c r="K137" s="6" t="str">
+        <v>66</v>
+      </c>
+      <c r="J137" s="5" t="n">
+        <v>46322</v>
+      </c>
+      <c r="K137" s="6" t="n">
         <f aca="false">IF(J137="","",WORKDAY(J137+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L137" s="5"/>
       <c r="M137" s="4"/>
       <c r="N137" s="4"/>
       <c r="O137" s="4" t="s">
-        <v>469</v>
+        <v>111</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8048,25 +8088,25 @@
         <v>196</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="D138" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E138" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="F138" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="G138" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="H138" s="3" t="s">
         <v>477</v>
       </c>
-      <c r="F138" s="3" t="s">
-        <v>478</v>
-      </c>
-      <c r="G138" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="H138" s="3" t="s">
-        <v>475</v>
-      </c>
       <c r="I138" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J138" s="5"/>
       <c r="K138" s="6" t="str">
@@ -8077,7 +8117,7 @@
       <c r="M138" s="4"/>
       <c r="N138" s="4"/>
       <c r="O138" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8088,25 +8128,25 @@
         <v>196</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="F139" s="3" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="G139" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H139" s="3" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="I139" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J139" s="5"/>
       <c r="K139" s="6" t="str">
@@ -8117,7 +8157,7 @@
       <c r="M139" s="4"/>
       <c r="N139" s="4"/>
       <c r="O139" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8128,25 +8168,25 @@
         <v>196</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F140" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H140" s="3" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="I140" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J140" s="5"/>
       <c r="K140" s="6" t="str">
@@ -8157,7 +8197,7 @@
       <c r="M140" s="4"/>
       <c r="N140" s="4"/>
       <c r="O140" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8168,25 +8208,25 @@
         <v>196</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D141" s="3" t="s">
         <v>73</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="F141" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G141" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H141" s="3" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="I141" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J141" s="5"/>
       <c r="K141" s="6" t="str">
@@ -8197,7 +8237,7 @@
       <c r="M141" s="4"/>
       <c r="N141" s="4"/>
       <c r="O141" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8208,25 +8248,25 @@
         <v>196</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F142" s="3" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="G142" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H142" s="3" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="I142" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J142" s="5"/>
       <c r="K142" s="6" t="str">
@@ -8237,7 +8277,7 @@
       <c r="M142" s="4"/>
       <c r="N142" s="4"/>
       <c r="O142" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8248,25 +8288,25 @@
         <v>196</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E143" s="3" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="F143" s="3" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="G143" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H143" s="3" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="I143" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J143" s="5"/>
       <c r="K143" s="6" t="str">
@@ -8277,7 +8317,7 @@
       <c r="M143" s="4"/>
       <c r="N143" s="4"/>
       <c r="O143" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8288,25 +8328,25 @@
         <v>196</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="F144" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G144" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="I144" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J144" s="5"/>
       <c r="K144" s="6" t="str">
@@ -8317,7 +8357,7 @@
       <c r="M144" s="4"/>
       <c r="N144" s="4"/>
       <c r="O144" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8328,25 +8368,25 @@
         <v>196</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>113</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="G145" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H145" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="I145" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J145" s="5"/>
       <c r="K145" s="6" t="str">
@@ -8357,7 +8397,7 @@
       <c r="M145" s="4"/>
       <c r="N145" s="4"/>
       <c r="O145" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8368,25 +8408,25 @@
         <v>196</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="G146" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="I146" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J146" s="5"/>
       <c r="K146" s="6" t="str">
@@ -8397,7 +8437,7 @@
       <c r="M146" s="4"/>
       <c r="N146" s="4"/>
       <c r="O146" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8408,25 +8448,25 @@
         <v>196</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>89</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="G147" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H147" s="3" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="I147" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J147" s="5"/>
       <c r="K147" s="6" t="str">
@@ -8437,7 +8477,7 @@
       <c r="M147" s="4"/>
       <c r="N147" s="4"/>
       <c r="O147" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8448,25 +8488,25 @@
         <v>196</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>99</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="F148" s="3" t="s">
         <v>199</v>
       </c>
       <c r="G148" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H148" s="3" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="I148" s="4" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="J148" s="5"/>
       <c r="K148" s="6" t="str">
@@ -8477,7 +8517,7 @@
       <c r="M148" s="4"/>
       <c r="N148" s="4"/>
       <c r="O148" s="4" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9523,15 +9563,15 @@
   </sheetData>
   <autoFilter ref="A1:O200"/>
   <conditionalFormatting sqref="I2:I200">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"Lien obtenu"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Adresse invalide"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K200">
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>AND(K2&lt;&gt;"",K2&lt;=TODAY(),L2="",I2="Envoyé")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9572,12 +9612,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -9586,34 +9626,34 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -9622,7 +9662,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9640,7 +9680,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
@@ -9649,16 +9689,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.0258620689655172</v>
+        <v>0.0254237288135593</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -9667,21 +9707,21 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9689,13 +9729,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9810,7 +9850,7 @@
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9819,7 +9859,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
@@ -9836,7 +9876,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A27)</f>
@@ -9853,7 +9893,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A28)</f>
@@ -9870,7 +9910,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -9878,7 +9918,7 @@
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">SUM(D19:D28)</f>
@@ -9909,7 +9949,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9917,12 +9957,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9930,27 +9970,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9958,27 +9998,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection : CRMA ARA marquée adresse non suivie
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -361,34 +361,34 @@
     <t xml:space="preserve">Tiers, 2018 : peut être obsolète</t>
   </si>
   <si>
+    <t xml:space="preserve">23/10 : réponse automatique, l'adresse n'est plus suivie : contacter la CMA départementale. Pas de relance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Côte-d'Or</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bourgogne-Franche-Comté</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accueil-s21@artisanat-bfc.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Morbihan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accueil@cma-morbihan.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMA Loiret</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centre-Val de Loire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@cma45.fr</t>
+  </si>
+  <si>
     <t xml:space="preserve">Envoyé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23/10 : réponse automatique, l'adresse n'est plus suivie : contacter la CMA départementale. Pas de relance.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Côte-d'Or</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bourgogne-Franche-Comté</t>
-  </si>
-  <si>
-    <t xml:space="preserve">accueil-s21@artisanat-bfc.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Morbihan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">accueil@cma-morbihan.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CMA Loiret</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Centre-Val de Loire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@cma45.fr</t>
   </si>
   <si>
     <t xml:space="preserve">Relance prévue le 02/11/2026</t>
@@ -2983,7 +2983,7 @@
         <v>94</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="J18" s="5" t="n">
         <v>46318</v>
@@ -2996,7 +2996,7 @@
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
       <c r="O18" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3007,13 +3007,13 @@
         <v>90</v>
       </c>
       <c r="C19" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>103</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>104</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>79</v>
@@ -3051,13 +3051,13 @@
         <v>90</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>79</v>
@@ -3095,13 +3095,13 @@
         <v>90</v>
       </c>
       <c r="C21" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>108</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>109</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>79</v>
@@ -3113,7 +3113,7 @@
         <v>94</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J21" s="5" t="n">
         <v>46321</v>
@@ -3155,7 +3155,7 @@
         <v>94</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J22" s="5" t="n">
         <v>46321</v>
@@ -3197,7 +3197,7 @@
         <v>94</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J23" s="5" t="n">
         <v>46321</v>
@@ -3239,7 +3239,7 @@
         <v>94</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J24" s="5" t="n">
         <v>46321</v>
@@ -3281,7 +3281,7 @@
         <v>94</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J25" s="5" t="n">
         <v>46321</v>
@@ -3480,7 +3480,7 @@
         <v>141</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>142</v>
@@ -3524,7 +3524,7 @@
         <v>144</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>145</v>
@@ -3568,7 +3568,7 @@
         <v>146</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>147</v>
@@ -3612,7 +3612,7 @@
         <v>148</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>149</v>
@@ -3788,7 +3788,7 @@
         <v>160</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>161</v>
@@ -4327,7 +4327,7 @@
         <v>198</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J49" s="5" t="n">
         <v>46321</v>
@@ -4411,7 +4411,7 @@
         <v>198</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J51" s="5" t="n">
         <v>46321</v>
@@ -4453,7 +4453,7 @@
         <v>198</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J52" s="5" t="n">
         <v>46321</v>
@@ -4495,7 +4495,7 @@
         <v>198</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J53" s="5" t="n">
         <v>46321</v>
@@ -4537,7 +4537,7 @@
         <v>198</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J54" s="5" t="n">
         <v>46321</v>
@@ -4579,7 +4579,7 @@
         <v>198</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J55" s="5" t="n">
         <v>46321</v>
@@ -5057,7 +5057,7 @@
         <v>229</v>
       </c>
       <c r="I66" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J66" s="5" t="n">
         <v>46321</v>
@@ -5143,7 +5143,7 @@
         <v>257</v>
       </c>
       <c r="I68" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J68" s="5" t="n">
         <v>46321</v>
@@ -5227,7 +5227,7 @@
         <v>257</v>
       </c>
       <c r="I70" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J70" s="5" t="n">
         <v>46321</v>
@@ -5313,7 +5313,7 @@
         <v>257</v>
       </c>
       <c r="I72" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J72" s="5" t="n">
         <v>46321</v>
@@ -5428,7 +5428,7 @@
         <v>278</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E75" s="3" t="s">
         <v>279</v>
@@ -5487,7 +5487,7 @@
         <v>257</v>
       </c>
       <c r="I76" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J76" s="5" t="n">
         <v>46321</v>
@@ -5529,7 +5529,7 @@
         <v>257</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J77" s="5" t="n">
         <v>46321</v>
@@ -5613,7 +5613,7 @@
         <v>298</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J79" s="5" t="n">
         <v>46321</v>
@@ -5904,7 +5904,7 @@
         <v>324</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>325</v>
@@ -6051,7 +6051,7 @@
         <v>335</v>
       </c>
       <c r="I89" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J89" s="5" t="n">
         <v>46321</v>
@@ -6093,7 +6093,7 @@
         <v>198</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J90" s="5" t="n">
         <v>46321</v>
@@ -6135,7 +6135,7 @@
         <v>198</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J91" s="5" t="n">
         <v>46321</v>
@@ -6177,7 +6177,7 @@
         <v>198</v>
       </c>
       <c r="I92" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J92" s="5" t="n">
         <v>46321</v>
@@ -6219,7 +6219,7 @@
         <v>198</v>
       </c>
       <c r="I93" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J93" s="5" t="n">
         <v>46321</v>
@@ -6261,7 +6261,7 @@
         <v>198</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J94" s="5" t="n">
         <v>46321</v>
@@ -6303,7 +6303,7 @@
         <v>198</v>
       </c>
       <c r="I95" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J95" s="5" t="n">
         <v>46321</v>
@@ -6345,7 +6345,7 @@
         <v>198</v>
       </c>
       <c r="I96" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J96" s="5" t="n">
         <v>46321</v>
@@ -6387,7 +6387,7 @@
         <v>198</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J97" s="5" t="n">
         <v>46321</v>
@@ -6429,7 +6429,7 @@
         <v>198</v>
       </c>
       <c r="I98" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J98" s="5" t="n">
         <v>46321</v>
@@ -6471,7 +6471,7 @@
         <v>198</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J99" s="5" t="n">
         <v>46321</v>
@@ -6513,7 +6513,7 @@
         <v>198</v>
       </c>
       <c r="I100" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J100" s="5" t="n">
         <v>46321</v>
@@ -6582,7 +6582,7 @@
         <v>372</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E102" s="3" t="s">
         <v>373</v>
@@ -6597,7 +6597,7 @@
         <v>198</v>
       </c>
       <c r="I102" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J102" s="5" t="n">
         <v>46321</v>
@@ -6723,7 +6723,7 @@
         <v>198</v>
       </c>
       <c r="I105" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J105" s="5" t="n">
         <v>46321</v>
@@ -6765,7 +6765,7 @@
         <v>198</v>
       </c>
       <c r="I106" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J106" s="5" t="n">
         <v>46321</v>
@@ -6807,7 +6807,7 @@
         <v>198</v>
       </c>
       <c r="I107" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J107" s="5" t="n">
         <v>46321</v>
@@ -6849,7 +6849,7 @@
         <v>198</v>
       </c>
       <c r="I108" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J108" s="5" t="n">
         <v>46321</v>
@@ -6891,7 +6891,7 @@
         <v>198</v>
       </c>
       <c r="I109" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J109" s="5" t="n">
         <v>46321</v>
@@ -6933,7 +6933,7 @@
         <v>198</v>
       </c>
       <c r="I110" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J110" s="5" t="n">
         <v>46321</v>
@@ -6975,7 +6975,7 @@
         <v>198</v>
       </c>
       <c r="I111" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J111" s="5" t="n">
         <v>46321</v>
@@ -7017,7 +7017,7 @@
         <v>398</v>
       </c>
       <c r="I112" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J112" s="5" t="n">
         <v>46321</v>
@@ -7059,7 +7059,7 @@
         <v>198</v>
       </c>
       <c r="I113" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J113" s="5" t="n">
         <v>46321</v>
@@ -7101,7 +7101,7 @@
         <v>198</v>
       </c>
       <c r="I114" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J114" s="5" t="n">
         <v>46321</v>
@@ -7143,7 +7143,7 @@
         <v>198</v>
       </c>
       <c r="I115" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J115" s="5" t="n">
         <v>46321</v>
@@ -7185,7 +7185,7 @@
         <v>198</v>
       </c>
       <c r="I116" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J116" s="5" t="n">
         <v>46321</v>
@@ -7227,7 +7227,7 @@
         <v>198</v>
       </c>
       <c r="I117" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J117" s="5" t="n">
         <v>46321</v>
@@ -7269,7 +7269,7 @@
         <v>198</v>
       </c>
       <c r="I118" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J118" s="5" t="n">
         <v>46321</v>
@@ -7311,7 +7311,7 @@
         <v>198</v>
       </c>
       <c r="I119" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J119" s="5" t="n">
         <v>46321</v>
@@ -7353,7 +7353,7 @@
         <v>198</v>
       </c>
       <c r="I120" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J120" s="5" t="n">
         <v>46321</v>
@@ -7395,7 +7395,7 @@
         <v>198</v>
       </c>
       <c r="I121" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J121" s="5" t="n">
         <v>46321</v>
@@ -7437,7 +7437,7 @@
         <v>198</v>
       </c>
       <c r="I122" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J122" s="5" t="n">
         <v>46321</v>
@@ -7479,7 +7479,7 @@
         <v>94</v>
       </c>
       <c r="I123" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J123" s="5" t="n">
         <v>46321</v>
@@ -7563,7 +7563,7 @@
         <v>431</v>
       </c>
       <c r="I125" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J125" s="5" t="n">
         <v>46321</v>
@@ -7605,7 +7605,7 @@
         <v>436</v>
       </c>
       <c r="I126" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J126" s="5" t="n">
         <v>46321</v>
@@ -7691,7 +7691,7 @@
         <v>444</v>
       </c>
       <c r="I128" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J128" s="5" t="n">
         <v>46321</v>
@@ -7775,7 +7775,7 @@
         <v>449</v>
       </c>
       <c r="I130" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J130" s="5" t="n">
         <v>46321</v>
@@ -7817,7 +7817,7 @@
         <v>449</v>
       </c>
       <c r="I131" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J131" s="5" t="n">
         <v>46321</v>
@@ -7859,7 +7859,7 @@
         <v>455</v>
       </c>
       <c r="I132" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J132" s="5" t="n">
         <v>46321</v>
@@ -7901,7 +7901,7 @@
         <v>459</v>
       </c>
       <c r="I133" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J133" s="5" t="n">
         <v>46321</v>
@@ -7943,7 +7943,7 @@
         <v>462</v>
       </c>
       <c r="I134" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J134" s="5" t="n">
         <v>46321</v>
@@ -7985,7 +7985,7 @@
         <v>466</v>
       </c>
       <c r="I135" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J135" s="5" t="n">
         <v>46322</v>
@@ -8067,7 +8067,7 @@
         <v>474</v>
       </c>
       <c r="I137" s="4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="J137" s="5" t="n">
         <v>46322</v>
@@ -9642,7 +9642,7 @@
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9687,7 +9687,7 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9696,7 +9696,7 @@
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.0254237288135593</v>
+        <v>0.0256410256410256</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Prospection 28/10 : 3 envois
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="541">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -685,6 +685,9 @@
     <t xml:space="preserve">rouen-initiative@rouen.cci.fr</t>
   </si>
   <si>
+    <t xml:space="preserve">27/10 : avis de retard de remise (Delivery Status Notification - Delay), le serveur réessaie. Relance prévue le 02/11/2026.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Initiative Sud Grésivaudan Royans Vercors</t>
   </si>
   <si>
@@ -1471,28 +1474,28 @@
     <t xml:space="preserve">128 créations dans le Val-d'Oise en octobre : des outils gratuits pour vos porteurs de projet</t>
   </si>
   <si>
+    <t xml:space="preserve">Initiative Nord Seine-et-Marne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-nord77.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">154 créations en Seine-et-Marne en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Melun Val de Seine et Sud 77 (nouvelle adresse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plateforme@initiative-mvs-sud77.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (annuaire régional ; l’ancienne adresse camvs.com a été bloquée)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Brouillon prêt</t>
   </si>
   <si>
     <t xml:space="preserve">Envoi conseillé : jour 9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Nord Seine-et-Marne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-nord77.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">154 créations en Seine-et-Marne en octobre : des outils gratuits pour vos porteurs de projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Melun Val de Seine et Sud 77 (nouvelle adresse)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">plateforme@initiative-mvs-sud77.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (annuaire régional ; l’ancienne adresse camvs.com a été bloquée)</t>
   </si>
   <si>
     <t xml:space="preserve">Initiative Béziers Ouest Hérault</t>
@@ -4466,7 +4469,7 @@
       <c r="M52" s="4"/>
       <c r="N52" s="4"/>
       <c r="O52" s="4" t="s">
-        <v>110</v>
+        <v>208</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4477,13 +4480,13 @@
         <v>194</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>197</v>
@@ -4519,13 +4522,13 @@
         <v>194</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>127</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>197</v>
@@ -4561,16 +4564,16 @@
         <v>194</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>77</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>134</v>
@@ -4603,16 +4606,16 @@
         <v>194</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>127</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>134</v>
@@ -4647,16 +4650,16 @@
         <v>194</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>127</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>134</v>
@@ -4691,16 +4694,16 @@
         <v>194</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G58" s="3" t="s">
         <v>134</v>
@@ -4722,7 +4725,7 @@
       <c r="M58" s="4"/>
       <c r="N58" s="4"/>
       <c r="O58" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4730,25 +4733,25 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>134</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I59" s="4" t="s">
         <v>74</v>
@@ -4764,7 +4767,7 @@
       <c r="M59" s="4"/>
       <c r="N59" s="4"/>
       <c r="O59" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4772,25 +4775,25 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>112</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G60" s="3" t="s">
         <v>134</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I60" s="4" t="s">
         <v>22</v>
@@ -4816,25 +4819,25 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>134</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I61" s="4" t="s">
         <v>22</v>
@@ -4860,25 +4863,25 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>134</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I62" s="4" t="s">
         <v>22</v>
@@ -4904,25 +4907,25 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G63" s="3" t="s">
         <v>134</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I63" s="4" t="s">
         <v>22</v>
@@ -4948,25 +4951,25 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>127</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>134</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I64" s="4" t="s">
         <v>22</v>
@@ -4992,25 +4995,25 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G65" s="3" t="s">
         <v>134</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I65" s="4" t="s">
         <v>22</v>
@@ -5036,25 +5039,25 @@
         <v>65</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G66" s="3" t="s">
         <v>134</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>109</v>
@@ -5078,25 +5081,25 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I67" s="4" t="s">
         <v>22</v>
@@ -5114,7 +5117,7 @@
       <c r="M67" s="4"/>
       <c r="N67" s="4"/>
       <c r="O67" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5122,25 +5125,25 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>109</v>
@@ -5164,25 +5167,25 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I69" s="4" t="s">
         <v>74</v>
@@ -5198,7 +5201,7 @@
       <c r="M69" s="4"/>
       <c r="N69" s="4"/>
       <c r="O69" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5206,25 +5209,25 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>109</v>
@@ -5248,25 +5251,25 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="I71" s="4" t="s">
         <v>22</v>
@@ -5292,25 +5295,25 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E72" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I72" s="4" t="s">
         <v>109</v>
@@ -5334,25 +5337,25 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I73" s="4" t="s">
         <v>22</v>
@@ -5378,25 +5381,25 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I74" s="4" t="s">
         <v>22</v>
@@ -5422,25 +5425,25 @@
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>102</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="I75" s="4" t="s">
         <v>22</v>
@@ -5466,25 +5469,25 @@
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E76" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>109</v>
@@ -5500,7 +5503,7 @@
       <c r="M76" s="4"/>
       <c r="N76" s="4"/>
       <c r="O76" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5508,25 +5511,25 @@
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>112</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>109</v>
@@ -5553,19 +5556,19 @@
         <v>15</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>21</v>
@@ -5584,7 +5587,7 @@
       <c r="M78" s="4"/>
       <c r="N78" s="4"/>
       <c r="O78" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5595,22 +5598,22 @@
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>109</v>
@@ -5637,22 +5640,22 @@
         <v>15</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>37</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="I80" s="4" t="s">
         <v>22</v>
@@ -5670,7 +5673,7 @@
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
       <c r="O80" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5681,22 +5684,22 @@
         <v>15</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E81" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="I81" s="4" t="s">
         <v>22</v>
@@ -5725,22 +5728,22 @@
         <v>51</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E82" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G82" s="3" t="s">
         <v>64</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="I82" s="4" t="s">
         <v>22</v>
@@ -5769,22 +5772,22 @@
         <v>51</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>22</v>
@@ -5813,22 +5816,22 @@
         <v>51</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="I84" s="4" t="s">
         <v>22</v>
@@ -5854,25 +5857,25 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E85" s="3" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G85" s="3" t="s">
         <v>134</v>
       </c>
       <c r="H85" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>22</v>
@@ -5898,25 +5901,25 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>102</v>
       </c>
       <c r="E86" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G86" s="3" t="s">
         <v>134</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="I86" s="4" t="s">
         <v>22</v>
@@ -5942,25 +5945,25 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E87" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="I87" s="4" t="s">
         <v>22</v>
@@ -5989,22 +5992,22 @@
         <v>43</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>170</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="I88" s="4" t="s">
         <v>22</v>
@@ -6033,22 +6036,22 @@
         <v>43</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="I89" s="4" t="s">
         <v>109</v>
@@ -6075,16 +6078,16 @@
         <v>130</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E90" s="3" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G90" s="3" t="s">
         <v>134</v>
@@ -6117,16 +6120,16 @@
         <v>130</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E91" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G91" s="3" t="s">
         <v>134</v>
@@ -6159,16 +6162,16 @@
         <v>130</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E92" s="3" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G92" s="3" t="s">
         <v>134</v>
@@ -6201,16 +6204,16 @@
         <v>130</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E93" s="3" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G93" s="3" t="s">
         <v>134</v>
@@ -6243,16 +6246,16 @@
         <v>130</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>134</v>
@@ -6285,16 +6288,16 @@
         <v>130</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>134</v>
@@ -6327,16 +6330,16 @@
         <v>130</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G96" s="3" t="s">
         <v>134</v>
@@ -6369,16 +6372,16 @@
         <v>130</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G97" s="3" t="s">
         <v>134</v>
@@ -6411,19 +6414,19 @@
         <v>194</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>77</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F98" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G98" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H98" s="3" t="s">
         <v>198</v>
@@ -6453,19 +6456,19 @@
         <v>194</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E99" s="3" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F99" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H99" s="3" t="s">
         <v>198</v>
@@ -6495,19 +6498,19 @@
         <v>194</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F100" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G100" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H100" s="3" t="s">
         <v>198</v>
@@ -6537,19 +6540,19 @@
         <v>194</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F101" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H101" s="3" t="s">
         <v>198</v>
@@ -6568,7 +6571,7 @@
       <c r="M101" s="4"/>
       <c r="N101" s="4"/>
       <c r="O101" s="4" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6579,19 +6582,19 @@
         <v>194</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>107</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F102" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G102" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H102" s="3" t="s">
         <v>198</v>
@@ -6621,19 +6624,19 @@
         <v>194</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H103" s="3" t="s">
         <v>198</v>
@@ -6652,7 +6655,7 @@
       <c r="M103" s="4"/>
       <c r="N103" s="4"/>
       <c r="O103" s="4" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6663,19 +6666,19 @@
         <v>194</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E104" s="3" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F104" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G104" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H104" s="3" t="s">
         <v>198</v>
@@ -6705,19 +6708,19 @@
         <v>194</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E105" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G105" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H105" s="3" t="s">
         <v>198</v>
@@ -6747,19 +6750,19 @@
         <v>194</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G106" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H106" s="3" t="s">
         <v>198</v>
@@ -6789,19 +6792,19 @@
         <v>194</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E107" s="3" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G107" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H107" s="3" t="s">
         <v>198</v>
@@ -6831,19 +6834,19 @@
         <v>194</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E108" s="3" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H108" s="3" t="s">
         <v>198</v>
@@ -6873,19 +6876,19 @@
         <v>194</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G109" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H109" s="3" t="s">
         <v>198</v>
@@ -6915,19 +6918,19 @@
         <v>194</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E110" s="3" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G110" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H110" s="3" t="s">
         <v>198</v>
@@ -6957,19 +6960,19 @@
         <v>194</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E111" s="3" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G111" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H111" s="3" t="s">
         <v>198</v>
@@ -6999,22 +7002,22 @@
         <v>194</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E112" s="3" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F112" s="3" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H112" s="3" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I112" s="4" t="s">
         <v>109</v>
@@ -7041,19 +7044,19 @@
         <v>194</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H113" s="3" t="s">
         <v>198</v>
@@ -7080,22 +7083,22 @@
         <v>113</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H114" s="3" t="s">
         <v>198</v>
@@ -7122,22 +7125,22 @@
         <v>114</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G115" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H115" s="3" t="s">
         <v>198</v>
@@ -7164,22 +7167,22 @@
         <v>115</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G116" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H116" s="3" t="s">
         <v>198</v>
@@ -7206,22 +7209,22 @@
         <v>116</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D117" s="3" t="s">
         <v>84</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G117" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H117" s="3" t="s">
         <v>198</v>
@@ -7248,22 +7251,22 @@
         <v>117</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>77</v>
       </c>
       <c r="E118" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G118" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H118" s="3" t="s">
         <v>198</v>
@@ -7290,22 +7293,22 @@
         <v>118</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>67</v>
       </c>
       <c r="E119" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G119" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H119" s="3" t="s">
         <v>198</v>
@@ -7332,22 +7335,22 @@
         <v>119</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E120" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G120" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H120" s="3" t="s">
         <v>198</v>
@@ -7377,19 +7380,19 @@
         <v>59</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E121" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G121" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H121" s="3" t="s">
         <v>198</v>
@@ -7419,19 +7422,19 @@
         <v>130</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F122" s="3" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G122" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H122" s="3" t="s">
         <v>198</v>
@@ -7461,16 +7464,16 @@
         <v>90</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E123" s="3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F123" s="3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G123" s="3" t="s">
         <v>93</v>
@@ -7503,16 +7506,16 @@
         <v>90</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E124" s="3" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G124" s="3" t="s">
         <v>93</v>
@@ -7545,22 +7548,22 @@
         <v>15</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>17</v>
       </c>
       <c r="E125" s="3" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="G125" s="3" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="H125" s="3" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="I125" s="4" t="s">
         <v>109</v>
@@ -7587,22 +7590,22 @@
         <v>194</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D126" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F126" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="G126" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H126" s="3" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="I126" s="4" t="s">
         <v>109</v>
@@ -7626,25 +7629,25 @@
         <v>126</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F127" s="3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G127" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H127" s="3" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="I127" s="4" t="s">
         <v>27</v>
@@ -7662,7 +7665,7 @@
       </c>
       <c r="N127" s="4"/>
       <c r="O127" s="4" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7673,22 +7676,22 @@
         <v>194</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G128" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H128" s="3" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="I128" s="4" t="s">
         <v>109</v>
@@ -7712,25 +7715,25 @@
         <v>128</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F129" s="3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G129" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H129" s="3" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="I129" s="4" t="s">
         <v>74</v>
@@ -7757,22 +7760,22 @@
         <v>194</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>127</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F130" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G130" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H130" s="3" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="I130" s="4" t="s">
         <v>109</v>
@@ -7799,22 +7802,22 @@
         <v>59</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D131" s="3" t="s">
         <v>127</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G131" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H131" s="3" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="I131" s="4" t="s">
         <v>109</v>
@@ -7841,22 +7844,22 @@
         <v>194</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D132" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="F132" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="G132" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="I132" s="4" t="s">
         <v>109</v>
@@ -7883,22 +7886,22 @@
         <v>194</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>138</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G133" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H133" s="3" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="I133" s="4" t="s">
         <v>109</v>
@@ -7925,22 +7928,22 @@
         <v>194</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D134" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F134" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="G134" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H134" s="3" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="I134" s="4" t="s">
         <v>109</v>
@@ -7967,22 +7970,22 @@
         <v>194</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D135" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F135" s="3" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="G135" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="I135" s="4" t="s">
         <v>109</v>
@@ -8006,39 +8009,41 @@
         <v>135</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D136" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F136" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G136" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H136" s="3" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="I136" s="4" t="s">
-        <v>470</v>
-      </c>
-      <c r="J136" s="5"/>
-      <c r="K136" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J136" s="5" t="n">
+        <v>46323</v>
+      </c>
+      <c r="K136" s="6" t="n">
         <f aca="false">IF(J136="","",WORKDAY(J136+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L136" s="5"/>
       <c r="M136" s="4"/>
       <c r="N136" s="4"/>
       <c r="O136" s="4" t="s">
-        <v>471</v>
+        <v>110</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8049,22 +8054,22 @@
         <v>194</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E137" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="F137" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="G137" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H137" s="3" t="s">
         <v>473</v>
-      </c>
-      <c r="F137" s="3" t="s">
-        <v>439</v>
-      </c>
-      <c r="G137" s="3" t="s">
-        <v>435</v>
-      </c>
-      <c r="H137" s="3" t="s">
-        <v>474</v>
       </c>
       <c r="I137" s="4" t="s">
         <v>109</v>
@@ -8091,25 +8096,25 @@
         <v>194</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D138" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E138" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="F138" s="3" t="s">
         <v>476</v>
       </c>
-      <c r="F138" s="3" t="s">
+      <c r="G138" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H138" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="I138" s="4" t="s">
         <v>477</v>
-      </c>
-      <c r="G138" s="3" t="s">
-        <v>435</v>
-      </c>
-      <c r="H138" s="3" t="s">
-        <v>474</v>
-      </c>
-      <c r="I138" s="4" t="s">
-        <v>470</v>
       </c>
       <c r="J138" s="5"/>
       <c r="K138" s="6" t="str">
@@ -8120,7 +8125,7 @@
       <c r="M138" s="4"/>
       <c r="N138" s="4"/>
       <c r="O138" s="4" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8131,25 +8136,25 @@
         <v>194</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F139" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G139" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H139" s="3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="I139" s="4" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="J139" s="5"/>
       <c r="K139" s="6" t="str">
@@ -8160,7 +8165,7 @@
       <c r="M139" s="4"/>
       <c r="N139" s="4"/>
       <c r="O139" s="4" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8171,36 +8176,38 @@
         <v>194</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F140" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H140" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="I140" s="4" t="s">
-        <v>470</v>
-      </c>
-      <c r="J140" s="5"/>
-      <c r="K140" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J140" s="5" t="n">
+        <v>46323</v>
+      </c>
+      <c r="K140" s="6" t="n">
         <f aca="false">IF(J140="","",WORKDAY(J140+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L140" s="5"/>
       <c r="M140" s="4"/>
       <c r="N140" s="4"/>
       <c r="O140" s="4" t="s">
-        <v>471</v>
+        <v>110</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8211,36 +8218,38 @@
         <v>194</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D141" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F141" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G141" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H141" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="I141" s="4" t="s">
-        <v>470</v>
-      </c>
-      <c r="J141" s="5"/>
-      <c r="K141" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J141" s="5" t="n">
+        <v>46323</v>
+      </c>
+      <c r="K141" s="6" t="n">
         <f aca="false">IF(J141="","",WORKDAY(J141+4,1))</f>
-        <v/>
+        <v>46328</v>
       </c>
       <c r="L141" s="5"/>
       <c r="M141" s="4"/>
       <c r="N141" s="4"/>
       <c r="O141" s="4" t="s">
-        <v>471</v>
+        <v>110</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8251,25 +8260,25 @@
         <v>194</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F142" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="G142" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H142" s="3" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="I142" s="4" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="J142" s="5"/>
       <c r="K142" s="6" t="str">
@@ -8280,7 +8289,7 @@
       <c r="M142" s="4"/>
       <c r="N142" s="4"/>
       <c r="O142" s="4" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8291,25 +8300,25 @@
         <v>194</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E143" s="3" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F143" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="G143" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H143" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="I143" s="4" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="J143" s="5"/>
       <c r="K143" s="6" t="str">
@@ -8320,7 +8329,7 @@
       <c r="M143" s="4"/>
       <c r="N143" s="4"/>
       <c r="O143" s="4" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8331,25 +8340,25 @@
         <v>194</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F144" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G144" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="I144" s="4" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="J144" s="5"/>
       <c r="K144" s="6" t="str">
@@ -8360,7 +8369,7 @@
       <c r="M144" s="4"/>
       <c r="N144" s="4"/>
       <c r="O144" s="4" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8371,25 +8380,25 @@
         <v>194</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>112</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="G145" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H145" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="I145" s="4" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="J145" s="5"/>
       <c r="K145" s="6" t="str">
@@ -8400,7 +8409,7 @@
       <c r="M145" s="4"/>
       <c r="N145" s="4"/>
       <c r="O145" s="4" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8411,25 +8420,25 @@
         <v>194</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="G146" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="I146" s="4" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="J146" s="5"/>
       <c r="K146" s="6" t="str">
@@ -8440,7 +8449,7 @@
       <c r="M146" s="4"/>
       <c r="N146" s="4"/>
       <c r="O146" s="4" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8451,25 +8460,25 @@
         <v>194</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G147" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H147" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="I147" s="4" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="J147" s="5"/>
       <c r="K147" s="6" t="str">
@@ -8480,7 +8489,7 @@
       <c r="M147" s="4"/>
       <c r="N147" s="4"/>
       <c r="O147" s="4" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8491,25 +8500,25 @@
         <v>194</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F148" s="3" t="s">
         <v>197</v>
       </c>
       <c r="G148" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H148" s="3" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="I148" s="4" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="J148" s="5"/>
       <c r="K148" s="6" t="str">
@@ -8520,7 +8529,7 @@
       <c r="M148" s="4"/>
       <c r="N148" s="4"/>
       <c r="O148" s="4" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9615,12 +9624,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -9629,25 +9638,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -9656,7 +9665,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -9665,7 +9674,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9683,7 +9692,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
@@ -9692,16 +9701,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.0256410256410256</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -9710,7 +9719,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -9719,12 +9728,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9732,13 +9741,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9853,7 +9862,7 @@
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9862,7 +9871,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A26)</f>
@@ -9870,7 +9879,7 @@
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A26,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D26" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A26,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9879,7 +9888,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A27)</f>
@@ -9896,7 +9905,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">COUNTIF(Suivi!$B$2:$B$200,A28)</f>
@@ -9913,7 +9922,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -9921,7 +9930,7 @@
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">SUM(D19:D28)</f>
@@ -9952,7 +9961,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9960,12 +9969,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9973,27 +9982,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10001,27 +10010,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection 29/10 : 5 envois
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="542">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -1529,6 +1529,9 @@
   </si>
   <si>
     <t xml:space="preserve">156 créations en Haute-Garonne en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relance prévue le 03/11/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Initiative Loire-Atlantique Nord</t>
@@ -8278,18 +8281,20 @@
         <v>489</v>
       </c>
       <c r="I142" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="J142" s="5"/>
-      <c r="K142" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J142" s="5" t="n">
+        <v>46324</v>
+      </c>
+      <c r="K142" s="6" t="n">
         <f aca="false">IF(J142="","",WORKDAY(J142+4,1))</f>
-        <v/>
+        <v>46329</v>
       </c>
       <c r="L142" s="5"/>
       <c r="M142" s="4"/>
       <c r="N142" s="4"/>
       <c r="O142" s="4" t="s">
-        <v>478</v>
+        <v>490</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8300,13 +8305,13 @@
         <v>194</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E143" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F143" s="3" t="s">
         <v>435</v>
@@ -8315,21 +8320,23 @@
         <v>436</v>
       </c>
       <c r="H143" s="3" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="I143" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="J143" s="5"/>
-      <c r="K143" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J143" s="5" t="n">
+        <v>46324</v>
+      </c>
+      <c r="K143" s="6" t="n">
         <f aca="false">IF(J143="","",WORKDAY(J143+4,1))</f>
-        <v/>
+        <v>46329</v>
       </c>
       <c r="L143" s="5"/>
       <c r="M143" s="4"/>
       <c r="N143" s="4"/>
       <c r="O143" s="4" t="s">
-        <v>478</v>
+        <v>490</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8340,13 +8347,13 @@
         <v>194</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F144" s="3" t="s">
         <v>197</v>
@@ -8355,21 +8362,23 @@
         <v>436</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="I144" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="J144" s="5"/>
-      <c r="K144" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J144" s="5" t="n">
+        <v>46324</v>
+      </c>
+      <c r="K144" s="6" t="n">
         <f aca="false">IF(J144="","",WORKDAY(J144+4,1))</f>
-        <v/>
+        <v>46329</v>
       </c>
       <c r="L144" s="5"/>
       <c r="M144" s="4"/>
       <c r="N144" s="4"/>
       <c r="O144" s="4" t="s">
-        <v>478</v>
+        <v>490</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8380,36 +8389,38 @@
         <v>194</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>112</v>
       </c>
       <c r="E145" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="G145" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H145" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="I145" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="J145" s="5"/>
-      <c r="K145" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J145" s="5" t="n">
+        <v>46324</v>
+      </c>
+      <c r="K145" s="6" t="n">
         <f aca="false">IF(J145="","",WORKDAY(J145+4,1))</f>
-        <v/>
+        <v>46329</v>
       </c>
       <c r="L145" s="5"/>
       <c r="M145" s="4"/>
       <c r="N145" s="4"/>
       <c r="O145" s="4" t="s">
-        <v>478</v>
+        <v>490</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8420,36 +8431,38 @@
         <v>194</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E146" s="3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="G146" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="I146" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="J146" s="5"/>
-      <c r="K146" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J146" s="5" t="n">
+        <v>46324</v>
+      </c>
+      <c r="K146" s="6" t="n">
         <f aca="false">IF(J146="","",WORKDAY(J146+4,1))</f>
-        <v/>
+        <v>46329</v>
       </c>
       <c r="L146" s="5"/>
       <c r="M146" s="4"/>
       <c r="N146" s="4"/>
       <c r="O146" s="4" t="s">
-        <v>478</v>
+        <v>490</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8460,13 +8473,13 @@
         <v>194</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F147" s="3" t="s">
         <v>444</v>
@@ -8475,7 +8488,7 @@
         <v>436</v>
       </c>
       <c r="H147" s="3" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="I147" s="4" t="s">
         <v>477</v>
@@ -8500,13 +8513,13 @@
         <v>194</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F148" s="3" t="s">
         <v>197</v>
@@ -8515,7 +8528,7 @@
         <v>436</v>
       </c>
       <c r="H148" s="3" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="I148" s="4" t="s">
         <v>477</v>
@@ -9624,12 +9637,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -9638,25 +9651,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -9665,7 +9678,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -9674,7 +9687,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9692,7 +9705,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
@@ -9701,16 +9714,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
-        <v>0.025</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -9719,7 +9732,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -9728,12 +9741,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9741,13 +9754,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9862,7 +9875,7 @@
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9922,7 +9935,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -9930,7 +9943,7 @@
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">SUM(D19:D28)</f>
@@ -9961,7 +9974,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9969,12 +9982,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9982,27 +9995,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10010,27 +10023,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Prospection : 3 envois et 3 rebonds du 30/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2n36AfHh3DyxxtwxTALqC
</commit_message>
<xml_diff>
--- a/docs/suivi-emailing.xlsx
+++ b/docs/suivi-emailing.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="545">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -685,7 +685,7 @@
     <t xml:space="preserve">rouen-initiative@rouen.cci.fr</t>
   </si>
   <si>
-    <t xml:space="preserve">27/10 : avis de retard de remise (Delivery Status Notification - Delay), le serveur réessaie. Relance prévue le 02/11/2026.</t>
+    <t xml:space="preserve">29/10 : échec définitif après 48 h, serveur rouen.cci.fr injoignable. Pas de relance.</t>
   </si>
   <si>
     <t xml:space="preserve">Initiative Sud Grésivaudan Royans Vercors</t>
@@ -1492,100 +1492,109 @@
     <t xml:space="preserve">Tiers (annuaire régional ; l’ancienne adresse camvs.com a été bloquée)</t>
   </si>
   <si>
+    <t xml:space="preserve">Relance prévue le 04/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Béziers Ouest Hérault</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@iboh.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">167 créations dans l'Hérault en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Oise Est</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@oise-est.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34 créations dans l'Oise en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Oise Ouest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@oise-ouest.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Haute-Garonne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-haute-garonne.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">156 créations en Haute-Garonne en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relance prévue le 03/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Loire-Atlantique Nord</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiativeloireatlantiquenord.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93 créations en Loire-Atlantique en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Loire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-loire.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">74 créations dans la Loire en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Moselle Nord</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pfil@synergie-ceei.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (les-aides.fr, PDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90 créations en Moselle en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30/10 : rebond 550 5.4.1 (Microsoft 365, accès refusé). Pas de relance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Guadeloupe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guadeloupe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guadeloupe-active@wanadoo.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiers (les-aides.fr, 2021), adresse ancienne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">73 créations en Guadeloupe en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30/10 : rebond 550 5.1.1, adresse inexistante chez Orange. Pas de relance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initiative Anjou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact@initiative-anjou.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">59 créations en Maine-et-Loire en octobre : des outils gratuits pour vos porteurs de projet</t>
+  </si>
+  <si>
     <t xml:space="preserve">Brouillon prêt</t>
   </si>
   <si>
     <t xml:space="preserve">Envoi conseillé : jour 9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Béziers Ouest Hérault</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@iboh.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">167 créations dans l'Hérault en octobre : des outils gratuits pour vos porteurs de projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Oise Est</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@oise-est.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">34 créations dans l'Oise en octobre : des outils gratuits pour vos porteurs de projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Oise Ouest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@oise-ouest.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Haute-Garonne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-haute-garonne.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">156 créations en Haute-Garonne en octobre : des outils gratuits pour vos porteurs de projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relance prévue le 03/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Loire-Atlantique Nord</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiativeloireatlantiquenord.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">93 créations en Loire-Atlantique en octobre : des outils gratuits pour vos porteurs de projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Loire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-loire.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">74 créations dans la Loire en octobre : des outils gratuits pour vos porteurs de projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Moselle Nord</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pfil@synergie-ceei.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (les-aides.fr, PDF)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">90 créations en Moselle en octobre : des outils gratuits pour vos porteurs de projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Guadeloupe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guadeloupe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">guadeloupe-active@wanadoo.fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiers (les-aides.fr, 2021), adresse ancienne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">73 créations en Guadeloupe en octobre : des outils gratuits pour vos porteurs de projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Initiative Anjou</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact@initiative-anjou.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">59 créations en Maine-et-Loire en octobre : des outils gratuits pour vos porteurs de projet</t>
   </si>
   <si>
     <t xml:space="preserve">Initiative Dombes Val de Saône</t>
@@ -4459,7 +4468,7 @@
         <v>198</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="J52" s="5" t="n">
         <v>46321</v>
@@ -8117,18 +8126,20 @@
         <v>473</v>
       </c>
       <c r="I138" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="J138" s="5"/>
-      <c r="K138" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J138" s="5" t="n">
+        <v>46325</v>
+      </c>
+      <c r="K138" s="6" t="n">
         <f aca="false">IF(J138="","",WORKDAY(J138+4,1))</f>
-        <v/>
+        <v>46330</v>
       </c>
       <c r="L138" s="5"/>
       <c r="M138" s="4"/>
       <c r="N138" s="4"/>
       <c r="O138" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8139,13 +8150,13 @@
         <v>194</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="F139" s="3" t="s">
         <v>444</v>
@@ -8154,21 +8165,23 @@
         <v>436</v>
       </c>
       <c r="H139" s="3" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="I139" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="J139" s="5"/>
-      <c r="K139" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J139" s="5" t="n">
+        <v>46325</v>
+      </c>
+      <c r="K139" s="6" t="n">
         <f aca="false">IF(J139="","",WORKDAY(J139+4,1))</f>
-        <v/>
+        <v>46330</v>
       </c>
       <c r="L139" s="5"/>
       <c r="M139" s="4"/>
       <c r="N139" s="4"/>
       <c r="O139" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8179,13 +8192,13 @@
         <v>194</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="F140" s="3" t="s">
         <v>197</v>
@@ -8194,7 +8207,7 @@
         <v>436</v>
       </c>
       <c r="H140" s="3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="I140" s="4" t="s">
         <v>109</v>
@@ -8221,13 +8234,13 @@
         <v>194</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D141" s="3" t="s">
         <v>71</v>
       </c>
       <c r="E141" s="3" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F141" s="3" t="s">
         <v>197</v>
@@ -8236,7 +8249,7 @@
         <v>436</v>
       </c>
       <c r="H141" s="3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="I141" s="4" t="s">
         <v>109</v>
@@ -8263,13 +8276,13 @@
         <v>194</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E142" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F142" s="3" t="s">
         <v>435</v>
@@ -8278,7 +8291,7 @@
         <v>436</v>
       </c>
       <c r="H142" s="3" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="I142" s="4" t="s">
         <v>109</v>
@@ -8294,7 +8307,7 @@
       <c r="M142" s="4"/>
       <c r="N142" s="4"/>
       <c r="O142" s="4" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8305,13 +8318,13 @@
         <v>194</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E143" s="3" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F143" s="3" t="s">
         <v>435</v>
@@ -8320,7 +8333,7 @@
         <v>436</v>
       </c>
       <c r="H143" s="3" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="I143" s="4" t="s">
         <v>109</v>
@@ -8336,7 +8349,7 @@
       <c r="M143" s="4"/>
       <c r="N143" s="4"/>
       <c r="O143" s="4" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8347,13 +8360,13 @@
         <v>194</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E144" s="3" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F144" s="3" t="s">
         <v>197</v>
@@ -8362,7 +8375,7 @@
         <v>436</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="I144" s="4" t="s">
         <v>109</v>
@@ -8378,7 +8391,7 @@
       <c r="M144" s="4"/>
       <c r="N144" s="4"/>
       <c r="O144" s="4" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8389,25 +8402,25 @@
         <v>194</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>112</v>
       </c>
       <c r="E145" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="F145" s="3" t="s">
         <v>498</v>
-      </c>
-      <c r="F145" s="3" t="s">
-        <v>499</v>
       </c>
       <c r="G145" s="3" t="s">
         <v>436</v>
       </c>
       <c r="H145" s="3" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="I145" s="4" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="J145" s="5" t="n">
         <v>46324</v>
@@ -8420,7 +8433,7 @@
       <c r="M145" s="4"/>
       <c r="N145" s="4"/>
       <c r="O145" s="4" t="s">
-        <v>490</v>
+        <v>500</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8449,7 +8462,7 @@
         <v>505</v>
       </c>
       <c r="I146" s="4" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="J146" s="5" t="n">
         <v>46324</v>
@@ -8462,7 +8475,7 @@
       <c r="M146" s="4"/>
       <c r="N146" s="4"/>
       <c r="O146" s="4" t="s">
-        <v>490</v>
+        <v>506</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8473,13 +8486,13 @@
         <v>194</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>87</v>
       </c>
       <c r="E147" s="3" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F147" s="3" t="s">
         <v>444</v>
@@ -8488,10 +8501,10 @@
         <v>436</v>
       </c>
       <c r="H147" s="3" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="I147" s="4" t="s">
-        <v>477</v>
+        <v>510</v>
       </c>
       <c r="J147" s="5"/>
       <c r="K147" s="6" t="str">
@@ -8502,7 +8515,7 @@
       <c r="M147" s="4"/>
       <c r="N147" s="4"/>
       <c r="O147" s="4" t="s">
-        <v>478</v>
+        <v>511</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8513,13 +8526,13 @@
         <v>194</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>97</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="F148" s="3" t="s">
         <v>197</v>
@@ -8528,21 +8541,23 @@
         <v>436</v>
       </c>
       <c r="H148" s="3" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="I148" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="J148" s="5"/>
-      <c r="K148" s="6" t="str">
+        <v>109</v>
+      </c>
+      <c r="J148" s="5" t="n">
+        <v>46325</v>
+      </c>
+      <c r="K148" s="6" t="n">
         <f aca="false">IF(J148="","",WORKDAY(J148+4,1))</f>
-        <v/>
+        <v>46330</v>
       </c>
       <c r="L148" s="5"/>
       <c r="M148" s="4"/>
       <c r="N148" s="4"/>
       <c r="O148" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9637,12 +9652,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$E$2:$E$200,"*@*")</f>
@@ -9651,16 +9666,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Brouillon prêt")</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Envoyé")+COUNTIF(Suivi!$I$2:$I$200,"Relancé")+COUNTIF(Suivi!$I$2:$I$200,"Répondu")+COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")+COUNTIF(Suivi!$I$2:$I$200,"Refus")+COUNTIF(Suivi!$I$2:$I$200,"Pas de réponse")</f>
@@ -9669,7 +9684,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Relancé")</f>
@@ -9678,7 +9693,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$M$2:$M$200,"Oui")</f>
@@ -9687,7 +9702,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9705,16 +9720,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF(Suivi!$I$2:$I$200,"Adresse invalide")</f>
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">IFERROR(B7/B5,0)</f>
@@ -9723,7 +9738,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">IFERROR(B8/B5,0)</f>
@@ -9732,7 +9747,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="true">COUNTIFS(Suivi!$K$2:$K$200,"&lt;="&amp;TODAY(),Suivi!$I$2:$I$200,"Envoyé",Suivi!$L$2:$L$200,"")</f>
@@ -9741,12 +9756,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9754,13 +9769,13 @@
         <v>1</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9875,7 +9890,7 @@
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$J$2:$J$200,"&lt;&gt;")</f>
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">COUNTIFS(Suivi!$B$2:$B$200,A25,Suivi!$I$2:$I$200,"Lien obtenu")</f>
@@ -9935,7 +9950,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUM(B19:B28)</f>
@@ -9943,7 +9958,7 @@
       </c>
       <c r="C29" s="8" t="n">
         <f aca="false">SUM(C19:C28)</f>
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D29" s="8" t="n">
         <f aca="false">SUM(D19:D28)</f>
@@ -9974,7 +9989,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9982,12 +9997,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9995,27 +10010,27 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10023,27 +10038,27 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>